<commit_message>
Simple Flow: apply API-folder rule — route API cases to 'API —' sections; record standing rule
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AZ5XzKsK9wv7M41cSPaMyg
</commit_message>
<xml_diff>
--- a/build/simple-flow/SimpleFlow_Blockers_Tracker.xlsx
+++ b/build/simple-flow/SimpleFlow_Blockers_Tracker.xlsx
@@ -702,7 +702,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Work Order Settings</t>
+          <t>API — Work Order Settings</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -843,7 +843,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Work Order Settings</t>
+          <t>API — Work Order Settings</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -937,7 +937,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Work Order Settings</t>
+          <t>API — Work Order Settings</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -1031,7 +1031,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Work Order Settings</t>
+          <t>API — Work Order Settings</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -1078,7 +1078,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Work Order Settings</t>
+          <t>API — Work Order Settings</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -6671,7 +6671,7 @@
       </c>
       <c r="B132" s="2" t="inlineStr">
         <is>
-          <t>Permissions</t>
+          <t>API — Permissions</t>
         </is>
       </c>
       <c r="C132" s="2" t="inlineStr">
@@ -6906,7 +6906,7 @@
       </c>
       <c r="B137" s="6" t="inlineStr">
         <is>
-          <t>Permissions</t>
+          <t>API — Permissions</t>
         </is>
       </c>
       <c r="C137" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Simple Flow: VIU batch 3 + sub-classify remaining pending
Verified 12 built-surface VIU-Pending cases on sv7301 QA (admin+tech):
SF-VAL-03, SF-COMP-16/17/04, SF-TECH-05/06/07, SF-VPART-01/02/03/05, SF-PERM-09.
New totals: READY 54 / VIU-pending(QA) 59 / DEV 25 / Milos 15 / bug 6 = 159.

Sub-classified the 59 remaining VIU-PENDING(QA) into reachable-now (19),
needs-data (39), needs-account (1); added a 'VIU sub-bucket' column + Summary
count to the Blockers Tracker (gen_blockers.py).

New deviation BUG-9: vendorless part-add requires a Category (spec S5-R1 = only
desc+qty+sell); sell price not enforced. Settings + tech role restored/verified.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AZ5XzKsK9wv7M41cSPaMyg
</commit_message>
<xml_diff>
--- a/build/simple-flow/SimpleFlow_Blockers_Tracker.xlsx
+++ b/build/simple-flow/SimpleFlow_Blockers_Tracker.xlsx
@@ -492,7 +492,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I160"/>
+  <dimension ref="A1:K160"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -504,6 +504,8 @@
     <col width="26" customWidth="1" min="7" max="7"/>
     <col width="60" customWidth="1" min="8" max="8"/>
     <col width="34" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="65" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -552,6 +554,16 @@
           <t>Related story/question</t>
         </is>
       </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>VIU sub-bucket</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>VIU sub-bucket detail (QA-pending only)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -599,6 +611,12 @@
           <t>S1-R1..R8 / Story 1 AC</t>
         </is>
       </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -646,6 +664,12 @@
           <t>S1 AC / Key Decision (no operatingMode)</t>
         </is>
       </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -693,6 +717,12 @@
           <t>Q5 | S1-R2 (Create purchase orders)</t>
         </is>
       </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K4" s="3" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -740,6 +770,12 @@
           <t>S1-R3 (Vendor invoice Optional/Required)</t>
         </is>
       </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -787,6 +823,12 @@
           <t>S1-R1 (Auto-approve ON)</t>
         </is>
       </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -834,6 +876,12 @@
           <t>S1-R1 (Auto-approve OFF)</t>
         </is>
       </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -881,6 +929,12 @@
           <t>S1-R5..R8 (existing settings surfaced)</t>
         </is>
       </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -928,6 +982,12 @@
           <t>Q3, Q4 | S1 first-use defaults / §4</t>
         </is>
       </c>
+      <c r="J9" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K9" s="3" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -975,6 +1035,12 @@
           <t>S1-R9 (Save persists org-wide)</t>
         </is>
       </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
@@ -1022,6 +1088,16 @@
           <t>S1-R9 (future completions only, never retroactive)</t>
         </is>
       </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>reachable-now</t>
+        </is>
+      </c>
+      <c r="K11" s="4" t="inlineStr">
+        <is>
+          <t>admin+tech + normal WO data; needs another VIU pass (no new inputs).</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1069,6 +1145,12 @@
           <t>S1 AC (non-admin can't see/modify)</t>
         </is>
       </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1116,6 +1198,12 @@
           <t>S1 AC (no requireVin / no operatingMode field)</t>
         </is>
       </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -1163,6 +1251,12 @@
           <t>Q6 | S1 (Save dirty-state)</t>
         </is>
       </c>
+      <c r="J14" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K14" s="3" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1210,6 +1304,12 @@
           <t>S1-R4 (Require review before completion)</t>
         </is>
       </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1257,6 +1357,12 @@
           <t>S1 AC (helper text per toggle)</t>
         </is>
       </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1304,6 +1410,12 @@
           <t>S2-R1</t>
         </is>
       </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1351,6 +1463,12 @@
           <t>S2-R2 / S2-R3 / S2-R4</t>
         </is>
       </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1398,53 +1516,65 @@
           <t>S2-R4 / S2-R5 / S15-R3</t>
         </is>
       </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K19" s="2" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" s="4" t="inlineStr">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t>SF-COMP-04</t>
         </is>
       </c>
-      <c r="B20" s="4" t="inlineStr">
+      <c r="B20" s="2" t="inlineStr">
         <is>
           <t>Completion — No-PO / Skip (Story 2)</t>
         </is>
       </c>
-      <c r="C20" s="4" t="inlineStr">
+      <c r="C20" s="2" t="inlineStr">
         <is>
           <t>Verify Go to Invoice from the Success screen opens the Finance step where the invoice number is shown</t>
         </is>
       </c>
-      <c r="D20" s="4" t="inlineStr">
-        <is>
-          <t>VIU-Pending</t>
-        </is>
-      </c>
-      <c r="E20" s="4" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
-        </is>
-      </c>
-      <c r="F20" s="4" t="inlineStr">
-        <is>
-          <t>VIU PENDING (QA)</t>
-        </is>
-      </c>
-      <c r="G20" s="4" t="inlineStr">
-        <is>
-          <t>QA (needs cookies+seed data)</t>
-        </is>
-      </c>
-      <c r="H20" s="4" t="inlineStr">
-        <is>
-          <t>QA VIU: seed the specific completion configuration and drive the wizard to Success.</t>
-        </is>
-      </c>
-      <c r="I20" s="4" t="inlineStr">
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>VIU-Verified</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>READY (VIU-Verified)</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>None — VIU-verified; uploadable now.</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
         <is>
           <t>S2-R5 / S15-R3</t>
         </is>
       </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K20" s="2" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1492,6 +1622,12 @@
           <t>S2-R2 / S2 AC (missing required fields blocked)</t>
         </is>
       </c>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K21" s="2" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
@@ -1539,6 +1675,12 @@
           <t>Q5 | S2-R6 / S2 AC (Create POs off ⇒ no PO)</t>
         </is>
       </c>
+      <c r="J22" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K22" s="3" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
@@ -1586,6 +1728,12 @@
           <t>Q2 | S2-R6 / §5 invariant 1</t>
         </is>
       </c>
+      <c r="J23" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K23" s="3" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
@@ -1633,6 +1781,16 @@
           <t>S2-R2 / S2 AC (auto-pick off ⇒ pick in modal)</t>
         </is>
       </c>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>reachable-now</t>
+        </is>
+      </c>
+      <c r="K24" s="4" t="inlineStr">
+        <is>
+          <t>flip Auto-pick Inventory OFF and drive the completion modal pick step.</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -1680,6 +1838,12 @@
           <t>S2-R6 / S2 AC (re-open returns to Approved)</t>
         </is>
       </c>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K25" s="2" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
@@ -1727,6 +1891,16 @@
           <t>S2 AC (individual-line Complete + per-part receive kept)</t>
         </is>
       </c>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>reachable-now</t>
+        </is>
+      </c>
+      <c r="K26" s="4" t="inlineStr">
+        <is>
+          <t>admin+tech + normal WO data; needs another VIU pass (no new inputs).</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -1774,6 +1948,12 @@
           <t>S3-R4</t>
         </is>
       </c>
+      <c r="J27" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K27" s="2" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -1821,6 +2001,12 @@
           <t>S3-R1 / S3-R2 / S3-R9</t>
         </is>
       </c>
+      <c r="J28" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K28" s="2" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
@@ -1868,6 +2054,16 @@
           <t>S3-R5</t>
         </is>
       </c>
+      <c r="J29" s="4" t="inlineStr">
+        <is>
+          <t>needs-data</t>
+        </is>
+      </c>
+      <c r="K29" s="4" t="inlineStr">
+        <is>
+          <t>a WO PO in an ORDERED/deliverable state (vendor-assigned part on a PO with pending delivery); optional-flow 'Receive Parts' routed back to the WO, not Accept Delivery.</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -1915,6 +2111,12 @@
           <t>S3-R6</t>
         </is>
       </c>
+      <c r="J30" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K30" s="2" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
@@ -1962,100 +2164,122 @@
           <t>S3-R7 / S3-R9 (Cancel idempotent)</t>
         </is>
       </c>
+      <c r="J31" s="2" t="inlineStr">
+        <is>
+          <t>reachable-now</t>
+        </is>
+      </c>
+      <c r="K31" s="4" t="inlineStr">
+        <is>
+          <t>drive optional-flow Cancel and re-open; check no duplicate POs.</t>
+        </is>
+      </c>
     </row>
     <row r="32">
-      <c r="A32" s="4" t="inlineStr">
+      <c r="A32" s="2" t="inlineStr">
         <is>
           <t>SF-COMP-16</t>
         </is>
       </c>
-      <c r="B32" s="4" t="inlineStr">
+      <c r="B32" s="2" t="inlineStr">
         <is>
           <t>Completion — PO + Optional Invoice (Story 3)</t>
         </is>
       </c>
-      <c r="C32" s="4" t="inlineStr">
+      <c r="C32" s="2" t="inlineStr">
         <is>
           <t>Verify the optional-invoice modal collects required vehicle fields (mileage, VIN, engine hours) when missing</t>
         </is>
       </c>
-      <c r="D32" s="4" t="inlineStr">
-        <is>
-          <t>VIU-Pending</t>
-        </is>
-      </c>
-      <c r="E32" s="4" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
-        </is>
-      </c>
-      <c r="F32" s="4" t="inlineStr">
-        <is>
-          <t>VIU PENDING (QA)</t>
-        </is>
-      </c>
-      <c r="G32" s="4" t="inlineStr">
-        <is>
-          <t>QA (needs cookies+seed data)</t>
-        </is>
-      </c>
-      <c r="H32" s="4" t="inlineStr">
-        <is>
-          <t>QA VIU: seed the specific completion configuration and drive the wizard to Success.</t>
-        </is>
-      </c>
-      <c r="I32" s="4" t="inlineStr">
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>VIU-Verified</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>READY (VIU-Verified)</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>None — VIU-verified; uploadable now.</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="inlineStr">
         <is>
           <t>S3-R3</t>
         </is>
       </c>
+      <c r="J32" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K32" s="2" t="inlineStr"/>
     </row>
     <row r="33">
-      <c r="A33" s="4" t="inlineStr">
+      <c r="A33" s="2" t="inlineStr">
         <is>
           <t>SF-COMP-17</t>
         </is>
       </c>
-      <c r="B33" s="4" t="inlineStr">
+      <c r="B33" s="2" t="inlineStr">
         <is>
           <t>Completion — PO + Optional Invoice (Story 3)</t>
         </is>
       </c>
-      <c r="C33" s="4" t="inlineStr">
+      <c r="C33" s="2" t="inlineStr">
         <is>
           <t>Verify the optional-invoice flow reaches the Success screen with WO number and total</t>
         </is>
       </c>
-      <c r="D33" s="4" t="inlineStr">
-        <is>
-          <t>VIU-Pending</t>
-        </is>
-      </c>
-      <c r="E33" s="4" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
-        </is>
-      </c>
-      <c r="F33" s="4" t="inlineStr">
-        <is>
-          <t>VIU PENDING (QA)</t>
-        </is>
-      </c>
-      <c r="G33" s="4" t="inlineStr">
-        <is>
-          <t>QA (needs cookies+seed data)</t>
-        </is>
-      </c>
-      <c r="H33" s="4" t="inlineStr">
-        <is>
-          <t>QA VIU: seed the specific completion configuration and drive the wizard to Success.</t>
-        </is>
-      </c>
-      <c r="I33" s="4" t="inlineStr">
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>VIU-Verified</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>READY (VIU-Verified)</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>None — VIU-verified; uploadable now.</t>
+        </is>
+      </c>
+      <c r="I33" s="2" t="inlineStr">
         <is>
           <t>S3-R8</t>
         </is>
       </c>
+      <c r="J33" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K33" s="2" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -2103,6 +2327,12 @@
           <t>S4-R4</t>
         </is>
       </c>
+      <c r="J34" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K34" s="2" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
@@ -2150,6 +2380,16 @@
           <t>S4-R5 / S4-R7</t>
         </is>
       </c>
+      <c r="J35" s="4" t="inlineStr">
+        <is>
+          <t>needs-data</t>
+        </is>
+      </c>
+      <c r="K35" s="4" t="inlineStr">
+        <is>
+          <t>a receivable PO + vendor invoice number to drive the required-invoice receive round-trip.</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
@@ -2197,6 +2437,16 @@
           <t>S4-R6</t>
         </is>
       </c>
+      <c r="J36" s="2" t="inlineStr">
+        <is>
+          <t>reachable-now</t>
+        </is>
+      </c>
+      <c r="K36" s="4" t="inlineStr">
+        <is>
+          <t>required-invoice flow (requireVendorInvoiceNumber=ON) + part-bearing WO; Cancel = no change.</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -2244,6 +2494,12 @@
           <t>Key Decision (all lines approved) / S3-R9 / S4-R8</t>
         </is>
       </c>
+      <c r="J37" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K37" s="2" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -2291,6 +2547,12 @@
           <t>Key Decision (holds regardless of Auto-approve)</t>
         </is>
       </c>
+      <c r="J38" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K38" s="2" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
@@ -2338,6 +2600,16 @@
           <t>S3-R9 (no duplicate POs on re-Complete)</t>
         </is>
       </c>
+      <c r="J39" s="2" t="inlineStr">
+        <is>
+          <t>reachable-now</t>
+        </is>
+      </c>
+      <c r="K39" s="4" t="inlineStr">
+        <is>
+          <t>re-run completion after a prior attempt; check no duplicate POs.</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
@@ -2385,6 +2657,16 @@
           <t>S3-C1 / S4-C1 / Resolve Cores handoff</t>
         </is>
       </c>
+      <c r="J40" s="4" t="inlineStr">
+        <is>
+          <t>needs-data</t>
+        </is>
+      </c>
+      <c r="K40" s="4" t="inlineStr">
+        <is>
+          <t>an inventory/catalog part flagged is_core (genuine core) + a received cored line; the manual sub-form only sets core_charge (is_core stays false) and resolve-cores needs receiving.</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
@@ -2432,6 +2714,16 @@
           <t>S3-C1 (skipped if none)</t>
         </is>
       </c>
+      <c r="J41" s="4" t="inlineStr">
+        <is>
+          <t>needs-data</t>
+        </is>
+      </c>
+      <c r="K41" s="4" t="inlineStr">
+        <is>
+          <t>a genuine core part to prove the Resolve-Cores step appears, plus a no-core WO to prove it is skipped (is_core not seedable via canned/sub-form).</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
@@ -2479,6 +2771,16 @@
           <t>S3-C2</t>
         </is>
       </c>
+      <c r="J42" s="4" t="inlineStr">
+        <is>
+          <t>needs-data</t>
+        </is>
+      </c>
+      <c r="K42" s="4" t="inlineStr">
+        <is>
+          <t>a special-order core part + optional-invoice completion (needs is_core part).</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
@@ -2526,6 +2828,16 @@
           <t>S3-C3</t>
         </is>
       </c>
+      <c r="J43" s="4" t="inlineStr">
+        <is>
+          <t>needs-data</t>
+        </is>
+      </c>
+      <c r="K43" s="4" t="inlineStr">
+        <is>
+          <t>an unresolved special-order core at the invoice gate ('Cores pending' flag) — needs is_core part + receiving.</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
@@ -2573,6 +2885,16 @@
           <t>S3-C4</t>
         </is>
       </c>
+      <c r="J44" s="4" t="inlineStr">
+        <is>
+          <t>needs-data</t>
+        </is>
+      </c>
+      <c r="K44" s="4" t="inlineStr">
+        <is>
+          <t>resolve cores at the Create-Invoice gate -&gt; receive the cored line (needs is_core part + receiving).</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="4" t="inlineStr">
@@ -2620,6 +2942,16 @@
           <t>S3-C4 (cancel path)</t>
         </is>
       </c>
+      <c r="J45" s="4" t="inlineStr">
+        <is>
+          <t>needs-data</t>
+        </is>
+      </c>
+      <c r="K45" s="4" t="inlineStr">
+        <is>
+          <t>cancel the invoice-gate core resolution (needs is_core part + invoice gate).</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="4" t="inlineStr">
@@ -2667,6 +2999,16 @@
           <t>S4-C2</t>
         </is>
       </c>
+      <c r="J46" s="4" t="inlineStr">
+        <is>
+          <t>needs-data</t>
+        </is>
+      </c>
+      <c r="K46" s="4" t="inlineStr">
+        <is>
+          <t>special-order cores in the required-invoice receive round-trip (needs is_core part + receiving).</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="4" t="inlineStr">
@@ -2714,6 +3056,16 @@
           <t>S3 Guardrail (PartRequest-only core)</t>
         </is>
       </c>
+      <c r="J47" s="4" t="inlineStr">
+        <is>
+          <t>needs-data</t>
+        </is>
+      </c>
+      <c r="K47" s="4" t="inlineStr">
+        <is>
+          <t>an unresolved special-order core that exists only as a PartRequest (needs is_core part).</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="4" t="inlineStr">
@@ -2761,6 +3113,16 @@
           <t>S3 Guardrail (part-sale vs service WO)</t>
         </is>
       </c>
+      <c r="J48" s="4" t="inlineStr">
+        <is>
+          <t>needs-data</t>
+        </is>
+      </c>
+      <c r="K48" s="4" t="inlineStr">
+        <is>
+          <t>a part-sale WO vs service WO with cores (needs is_core part + receiving).</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="4" t="inlineStr">
@@ -2808,6 +3170,16 @@
           <t>Resolve Cores handoff (live +$ total)</t>
         </is>
       </c>
+      <c r="J49" s="4" t="inlineStr">
+        <is>
+          <t>needs-data</t>
+        </is>
+      </c>
+      <c r="K49" s="4" t="inlineStr">
+        <is>
+          <t>the Resolve-Cores step live '+$ to invoice' total (needs is_core part + receiving).</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -2855,6 +3227,12 @@
           <t>TS-R1</t>
         </is>
       </c>
+      <c r="J50" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K50" s="2" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -2902,6 +3280,12 @@
           <t>TS-R2</t>
         </is>
       </c>
+      <c r="J51" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K51" s="2" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -2949,6 +3333,12 @@
           <t>TS-R3</t>
         </is>
       </c>
+      <c r="J52" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K52" s="2" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -2996,147 +3386,171 @@
           <t>TS-R4</t>
         </is>
       </c>
+      <c r="J53" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K53" s="2" t="inlineStr"/>
     </row>
     <row r="54">
-      <c r="A54" s="4" t="inlineStr">
+      <c r="A54" s="2" t="inlineStr">
         <is>
           <t>SF-TECH-05</t>
         </is>
       </c>
-      <c r="B54" s="4" t="inlineStr">
+      <c r="B54" s="2" t="inlineStr">
         <is>
           <t>Tech Story Flow (Story 17)</t>
         </is>
       </c>
-      <c r="C54" s="4" t="inlineStr">
+      <c r="C54" s="2" t="inlineStr">
         <is>
           <t>Verify multi-line tech-story navigation (Back after line 1, Continue/Save on the last line)</t>
         </is>
       </c>
-      <c r="D54" s="4" t="inlineStr">
-        <is>
-          <t>VIU-Pending</t>
-        </is>
-      </c>
-      <c r="E54" s="4" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
-        </is>
-      </c>
-      <c r="F54" s="4" t="inlineStr">
-        <is>
-          <t>VIU PENDING (QA)</t>
-        </is>
-      </c>
-      <c r="G54" s="4" t="inlineStr">
-        <is>
-          <t>QA (needs cookies+seed data)</t>
-        </is>
-      </c>
-      <c r="H54" s="4" t="inlineStr">
-        <is>
-          <t>QA VIU: drive the multi-line tech-story gate flow (with the specific test-id).</t>
-        </is>
-      </c>
-      <c r="I54" s="4" t="inlineStr">
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>VIU-Verified</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>READY (VIU-Verified)</t>
+        </is>
+      </c>
+      <c r="G54" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H54" s="2" t="inlineStr">
+        <is>
+          <t>None — VIU-verified; uploadable now.</t>
+        </is>
+      </c>
+      <c r="I54" s="2" t="inlineStr">
         <is>
           <t>TS-R4 (multi-line navigation)</t>
         </is>
       </c>
+      <c r="J54" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K54" s="2" t="inlineStr"/>
     </row>
     <row r="55">
-      <c r="A55" s="4" t="inlineStr">
+      <c r="A55" s="2" t="inlineStr">
         <is>
           <t>SF-TECH-06</t>
         </is>
       </c>
-      <c r="B55" s="4" t="inlineStr">
+      <c r="B55" s="2" t="inlineStr">
         <is>
           <t>Tech Story Flow (Story 17)</t>
         </is>
       </c>
-      <c r="C55" s="4" t="inlineStr">
+      <c r="C55" s="2" t="inlineStr">
         <is>
           <t>Verify a saved tech story renders inline with a green check, the text and an Edit link</t>
         </is>
       </c>
-      <c r="D55" s="4" t="inlineStr">
-        <is>
-          <t>VIU-Pending</t>
-        </is>
-      </c>
-      <c r="E55" s="4" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
-        </is>
-      </c>
-      <c r="F55" s="4" t="inlineStr">
-        <is>
-          <t>VIU PENDING (QA)</t>
-        </is>
-      </c>
-      <c r="G55" s="4" t="inlineStr">
-        <is>
-          <t>QA (needs cookies+seed data)</t>
-        </is>
-      </c>
-      <c r="H55" s="4" t="inlineStr">
-        <is>
-          <t>QA VIU: drive the multi-line tech-story gate flow (with the specific test-id).</t>
-        </is>
-      </c>
-      <c r="I55" s="4" t="inlineStr">
+      <c r="D55" s="2" t="inlineStr">
+        <is>
+          <t>VIU-Verified</t>
+        </is>
+      </c>
+      <c r="E55" s="2" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t>READY (VIU-Verified)</t>
+        </is>
+      </c>
+      <c r="G55" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H55" s="2" t="inlineStr">
+        <is>
+          <t>None — VIU-verified; uploadable now.</t>
+        </is>
+      </c>
+      <c r="I55" s="2" t="inlineStr">
         <is>
           <t>TS-R5</t>
         </is>
       </c>
+      <c r="J55" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K55" s="2" t="inlineStr"/>
     </row>
     <row r="56">
-      <c r="A56" s="4" t="inlineStr">
+      <c r="A56" s="2" t="inlineStr">
         <is>
           <t>SF-TECH-07</t>
         </is>
       </c>
-      <c r="B56" s="4" t="inlineStr">
+      <c r="B56" s="2" t="inlineStr">
         <is>
           <t>Tech Story Flow (Story 17)</t>
         </is>
       </c>
-      <c r="C56" s="4" t="inlineStr">
+      <c r="C56" s="2" t="inlineStr">
         <is>
           <t>Verify the tech-story textarea exposes the test id input_tech_story</t>
         </is>
       </c>
-      <c r="D56" s="4" t="inlineStr">
-        <is>
-          <t>VIU-Pending</t>
-        </is>
-      </c>
-      <c r="E56" s="4" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
-        </is>
-      </c>
-      <c r="F56" s="4" t="inlineStr">
-        <is>
-          <t>VIU PENDING (QA)</t>
-        </is>
-      </c>
-      <c r="G56" s="4" t="inlineStr">
-        <is>
-          <t>QA (needs cookies+seed data)</t>
-        </is>
-      </c>
-      <c r="H56" s="4" t="inlineStr">
-        <is>
-          <t>QA VIU: drive the multi-line tech-story gate flow (with the specific test-id).</t>
-        </is>
-      </c>
-      <c r="I56" s="4" t="inlineStr">
+      <c r="D56" s="2" t="inlineStr">
+        <is>
+          <t>VIU-Verified</t>
+        </is>
+      </c>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t>READY (VIU-Verified)</t>
+        </is>
+      </c>
+      <c r="G56" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H56" s="2" t="inlineStr">
+        <is>
+          <t>None — VIU-verified; uploadable now.</t>
+        </is>
+      </c>
+      <c r="I56" s="2" t="inlineStr">
         <is>
           <t>TS-R6 (test id)</t>
         </is>
       </c>
+      <c r="J56" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K56" s="2" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="3" t="inlineStr">
@@ -3184,147 +3598,171 @@
           <t>Q9, Q4 | TS Decision vs S15-R2</t>
         </is>
       </c>
+      <c r="J57" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K57" s="3" t="inlineStr"/>
     </row>
     <row r="58">
-      <c r="A58" s="4" t="inlineStr">
+      <c r="A58" s="2" t="inlineStr">
         <is>
           <t>SF-VPART-01</t>
         </is>
       </c>
-      <c r="B58" s="4" t="inlineStr">
+      <c r="B58" s="2" t="inlineStr">
         <is>
           <t>Vendorless / No-PN Part (Story 5)</t>
         </is>
       </c>
-      <c r="C58" s="4" t="inlineStr">
+      <c r="C58" s="2" t="inlineStr">
         <is>
           <t>Verify a part can be requested with only description, quantity and sell price (part number, cost, vendor empty)</t>
         </is>
       </c>
-      <c r="D58" s="4" t="inlineStr">
-        <is>
-          <t>VIU-Pending</t>
-        </is>
-      </c>
-      <c r="E58" s="4" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
-        </is>
-      </c>
-      <c r="F58" s="4" t="inlineStr">
-        <is>
-          <t>VIU PENDING (QA)</t>
-        </is>
-      </c>
-      <c r="G58" s="4" t="inlineStr">
-        <is>
-          <t>QA (needs cookies+seed data)</t>
-        </is>
-      </c>
-      <c r="H58" s="4" t="inlineStr">
-        <is>
-          <t>QA VIU: seed + drive the vendorless / no-PN part add flow.</t>
-        </is>
-      </c>
-      <c r="I58" s="4" t="inlineStr">
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>VIU-Verified</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="F58" s="2" t="inlineStr">
+        <is>
+          <t>READY (VIU-Verified)</t>
+        </is>
+      </c>
+      <c r="G58" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H58" s="2" t="inlineStr">
+        <is>
+          <t>None — VIU-verified; uploadable now.</t>
+        </is>
+      </c>
+      <c r="I58" s="2" t="inlineStr">
         <is>
           <t>S5-R1</t>
         </is>
       </c>
+      <c r="J58" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K58" s="2" t="inlineStr"/>
     </row>
     <row r="59">
-      <c r="A59" s="4" t="inlineStr">
+      <c r="A59" s="2" t="inlineStr">
         <is>
           <t>SF-VPART-02</t>
         </is>
       </c>
-      <c r="B59" s="4" t="inlineStr">
+      <c r="B59" s="2" t="inlineStr">
         <is>
           <t>Vendorless / No-PN Part (Story 5)</t>
         </is>
       </c>
-      <c r="C59" s="4" t="inlineStr">
+      <c r="C59" s="2" t="inlineStr">
         <is>
           <t>Verify adding a part is blocked when description, quantity or sell price is missing</t>
         </is>
       </c>
-      <c r="D59" s="4" t="inlineStr">
-        <is>
-          <t>VIU-Pending</t>
-        </is>
-      </c>
-      <c r="E59" s="4" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
-        </is>
-      </c>
-      <c r="F59" s="4" t="inlineStr">
-        <is>
-          <t>VIU PENDING (QA)</t>
-        </is>
-      </c>
-      <c r="G59" s="4" t="inlineStr">
-        <is>
-          <t>QA (needs cookies+seed data)</t>
-        </is>
-      </c>
-      <c r="H59" s="4" t="inlineStr">
-        <is>
-          <t>QA VIU: drive the vendorless / no-PN add sub-form validation (not reached in the last session's budget).</t>
-        </is>
-      </c>
-      <c r="I59" s="4" t="inlineStr">
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>VIU-Verified</t>
+        </is>
+      </c>
+      <c r="E59" s="2" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="F59" s="2" t="inlineStr">
+        <is>
+          <t>READY (VIU-Verified)</t>
+        </is>
+      </c>
+      <c r="G59" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H59" s="2" t="inlineStr">
+        <is>
+          <t>None — VIU-verified; uploadable now.</t>
+        </is>
+      </c>
+      <c r="I59" s="2" t="inlineStr">
         <is>
           <t>S5-R1 / S5 AC (validation)</t>
         </is>
       </c>
+      <c r="J59" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K59" s="2" t="inlineStr"/>
     </row>
     <row r="60">
-      <c r="A60" s="4" t="inlineStr">
+      <c r="A60" s="2" t="inlineStr">
         <is>
           <t>SF-VPART-03</t>
         </is>
       </c>
-      <c r="B60" s="4" t="inlineStr">
+      <c r="B60" s="2" t="inlineStr">
         <is>
           <t>Vendorless / No-PN Part (Story 5)</t>
         </is>
       </c>
-      <c r="C60" s="4" t="inlineStr">
+      <c r="C60" s="2" t="inlineStr">
         <is>
           <t>Verify a vendorless part's type uses the existing source field (vendor or found) and never inventory</t>
         </is>
       </c>
-      <c r="D60" s="4" t="inlineStr">
-        <is>
-          <t>VIU-Pending</t>
-        </is>
-      </c>
-      <c r="E60" s="4" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
-        </is>
-      </c>
-      <c r="F60" s="4" t="inlineStr">
-        <is>
-          <t>VIU PENDING (QA)</t>
-        </is>
-      </c>
-      <c r="G60" s="4" t="inlineStr">
-        <is>
-          <t>QA (needs cookies+seed data)</t>
-        </is>
-      </c>
-      <c r="H60" s="4" t="inlineStr">
-        <is>
-          <t>QA VIU: seed + drive the vendorless / no-PN part add flow.</t>
-        </is>
-      </c>
-      <c r="I60" s="4" t="inlineStr">
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>VIU-Verified</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="F60" s="2" t="inlineStr">
+        <is>
+          <t>READY (VIU-Verified)</t>
+        </is>
+      </c>
+      <c r="G60" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H60" s="2" t="inlineStr">
+        <is>
+          <t>None — VIU-verified; uploadable now.</t>
+        </is>
+      </c>
+      <c r="I60" s="2" t="inlineStr">
         <is>
           <t>S5-R2</t>
         </is>
       </c>
+      <c r="J60" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K60" s="2" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="4" t="inlineStr">
@@ -3372,53 +3810,69 @@
           <t>S5-R3</t>
         </is>
       </c>
+      <c r="J61" s="2" t="inlineStr">
+        <is>
+          <t>reachable-now</t>
+        </is>
+      </c>
+      <c r="K61" s="4" t="inlineStr">
+        <is>
+          <t>edit an existing vendorless part inline (part_number/sell/qty row fields exist).</t>
+        </is>
+      </c>
     </row>
     <row r="62">
-      <c r="A62" s="4" t="inlineStr">
+      <c r="A62" s="2" t="inlineStr">
         <is>
           <t>SF-VPART-05</t>
         </is>
       </c>
-      <c r="B62" s="4" t="inlineStr">
+      <c r="B62" s="2" t="inlineStr">
         <is>
           <t>Vendorless / No-PN Part (Story 5)</t>
         </is>
       </c>
-      <c r="C62" s="4" t="inlineStr">
+      <c r="C62" s="2" t="inlineStr">
         <is>
           <t>Verify a no-part-number part creates no inventory item and no Part History</t>
         </is>
       </c>
-      <c r="D62" s="4" t="inlineStr">
-        <is>
-          <t>VIU-Pending</t>
-        </is>
-      </c>
-      <c r="E62" s="4" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
-        </is>
-      </c>
-      <c r="F62" s="4" t="inlineStr">
-        <is>
-          <t>VIU PENDING (QA)</t>
-        </is>
-      </c>
-      <c r="G62" s="4" t="inlineStr">
-        <is>
-          <t>QA (needs cookies+seed data)</t>
-        </is>
-      </c>
-      <c r="H62" s="4" t="inlineStr">
-        <is>
-          <t>QA VIU: seed + drive the vendorless / no-PN part add flow.</t>
-        </is>
-      </c>
-      <c r="I62" s="4" t="inlineStr">
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>VIU-Verified</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="F62" s="2" t="inlineStr">
+        <is>
+          <t>READY (VIU-Verified)</t>
+        </is>
+      </c>
+      <c r="G62" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H62" s="2" t="inlineStr">
+        <is>
+          <t>None — VIU-verified; uploadable now.</t>
+        </is>
+      </c>
+      <c r="I62" s="2" t="inlineStr">
         <is>
           <t>S5-R4 / S5 AC (no inventory interaction)</t>
         </is>
       </c>
+      <c r="J62" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K62" s="2" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="4" t="inlineStr">
@@ -3466,6 +3920,16 @@
           <t>S5 AC (transitions out of vendorless)</t>
         </is>
       </c>
+      <c r="J63" s="2" t="inlineStr">
+        <is>
+          <t>reachable-now</t>
+        </is>
+      </c>
+      <c r="K63" s="4" t="inlineStr">
+        <is>
+          <t>add a PN + vendor to a vendorless part and confirm it transitions out of vendorless.</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="4" t="inlineStr">
@@ -3513,6 +3977,16 @@
           <t>S5-R4 / S5 AC (receive gate)</t>
         </is>
       </c>
+      <c r="J64" s="4" t="inlineStr">
+        <is>
+          <t>needs-data</t>
+        </is>
+      </c>
+      <c r="K64" s="4" t="inlineStr">
+        <is>
+          <t>a receivable/deliverable state to prove a vendorless/no-PN part cannot be received until PN + vendor entered.</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -3560,6 +4034,12 @@
           <t>S6-R1</t>
         </is>
       </c>
+      <c r="J65" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K65" s="2" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -3607,6 +4087,12 @@
           <t>S6-R2</t>
         </is>
       </c>
+      <c r="J66" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K66" s="2" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" s="4" t="inlineStr">
@@ -3654,6 +4140,16 @@
           <t>S6-R3</t>
         </is>
       </c>
+      <c r="J67" s="4" t="inlineStr">
+        <is>
+          <t>needs-data</t>
+        </is>
+      </c>
+      <c r="K67" s="4" t="inlineStr">
+        <is>
+          <t>QuickBooks sync inspection (vendor-missing PO excluded from QB).</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="4" t="inlineStr">
@@ -3701,6 +4197,16 @@
           <t>S6-R4</t>
         </is>
       </c>
+      <c r="J68" s="2" t="inlineStr">
+        <is>
+          <t>reachable-now</t>
+        </is>
+      </c>
+      <c r="K68" s="4" t="inlineStr">
+        <is>
+          <t>vendor-missing PO seedable by completing a WO with vendorless vendor parts; check vendor-select + PN-edit options.</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="4" t="inlineStr">
@@ -3748,6 +4254,16 @@
           <t>S6-R5</t>
         </is>
       </c>
+      <c r="J69" s="2" t="inlineStr">
+        <is>
+          <t>reachable-now</t>
+        </is>
+      </c>
+      <c r="K69" s="4" t="inlineStr">
+        <is>
+          <t>vendor-missing PO; confirm the flag clears once vendor + PN supplied.</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="4" t="inlineStr">
@@ -3795,6 +4311,16 @@
           <t>S6-R6</t>
         </is>
       </c>
+      <c r="J70" s="4" t="inlineStr">
+        <is>
+          <t>needs-data</t>
+        </is>
+      </c>
+      <c r="K70" s="4" t="inlineStr">
+        <is>
+          <t>reports data (Vendor Missing POs flagged 'needs vendor').</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="5" t="inlineStr">
@@ -3842,6 +4368,12 @@
           <t>Story 7 — PO multi-select (SV-7702) | S7-R1</t>
         </is>
       </c>
+      <c r="J71" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K71" s="5" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" s="5" t="inlineStr">
@@ -3889,6 +4421,12 @@
           <t>Story 7 — PO multi-select (SV-7702) | S7-R2</t>
         </is>
       </c>
+      <c r="J72" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K72" s="5" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" s="5" t="inlineStr">
@@ -3936,6 +4474,12 @@
           <t>Story 7 — PO multi-select (SV-7702) | S7-R3</t>
         </is>
       </c>
+      <c r="J73" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K73" s="5" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" s="5" t="inlineStr">
@@ -3983,6 +4527,12 @@
           <t>Story 7 — PO multi-select (SV-7702) | S7-R4</t>
         </is>
       </c>
+      <c r="J74" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K74" s="5" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" s="5" t="inlineStr">
@@ -4030,6 +4580,12 @@
           <t>Story 7 — PO multi-select (SV-7702) | S7-R5</t>
         </is>
       </c>
+      <c r="J75" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K75" s="5" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" s="5" t="inlineStr">
@@ -4077,6 +4633,12 @@
           <t>Story 7 — PO multi-select (SV-7702) | S7 (select-all scope)</t>
         </is>
       </c>
+      <c r="J76" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K76" s="5" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" s="5" t="inlineStr">
@@ -4124,6 +4686,12 @@
           <t>Story 8 — PO Bulk Receive page (SV-7703) | S8-R1</t>
         </is>
       </c>
+      <c r="J77" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K77" s="5" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" s="5" t="inlineStr">
@@ -4171,6 +4739,12 @@
           <t>Story 8 — PO Bulk Receive page (SV-7703) | S8-R2 / S8-R3</t>
         </is>
       </c>
+      <c r="J78" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K78" s="5" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" s="5" t="inlineStr">
@@ -4218,6 +4792,12 @@
           <t>Story 8 — PO Bulk Receive page (SV-7703) | S8-R4</t>
         </is>
       </c>
+      <c r="J79" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K79" s="5" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" s="5" t="inlineStr">
@@ -4265,6 +4845,12 @@
           <t>Story 8 — PO Bulk Receive page (SV-7703) | S8-R5</t>
         </is>
       </c>
+      <c r="J80" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K80" s="5" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" s="5" t="inlineStr">
@@ -4312,6 +4898,12 @@
           <t>Story 8 — PO Bulk Receive page (SV-7703) | S8-R6</t>
         </is>
       </c>
+      <c r="J81" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K81" s="5" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" s="5" t="inlineStr">
@@ -4359,6 +4951,12 @@
           <t>Story 8 — PO Bulk Receive page (SV-7703) | S8-R7 / S10-R2</t>
         </is>
       </c>
+      <c r="J82" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K82" s="5" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" s="5" t="inlineStr">
@@ -4406,6 +5004,12 @@
           <t>Story 8 — PO Bulk Receive page (SV-7703) | S8-R8</t>
         </is>
       </c>
+      <c r="J83" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K83" s="5" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" s="5" t="inlineStr">
@@ -4453,6 +5057,12 @@
           <t>Story 8 — PO Bulk Receive page (SV-7703) | S8-R10</t>
         </is>
       </c>
+      <c r="J84" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K84" s="5" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" s="5" t="inlineStr">
@@ -4500,6 +5110,12 @@
           <t>Story 8 — PO Bulk Receive page (SV-7703) | S8-R11</t>
         </is>
       </c>
+      <c r="J85" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K85" s="5" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" s="5" t="inlineStr">
@@ -4547,6 +5163,12 @@
           <t>Story 8 — PO Bulk Receive page (SV-7703) | S8-C1 / S8-C2</t>
         </is>
       </c>
+      <c r="J86" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K86" s="5" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" s="5" t="inlineStr">
@@ -4594,6 +5216,12 @@
           <t>Story 9 — Apply invoice to selected POs (SV-7704) | S9-R1</t>
         </is>
       </c>
+      <c r="J87" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K87" s="5" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" s="5" t="inlineStr">
@@ -4641,6 +5269,12 @@
           <t>Story 9 — Apply invoice to selected POs (SV-7704) | S9-R2</t>
         </is>
       </c>
+      <c r="J88" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K88" s="5" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" s="5" t="inlineStr">
@@ -4688,6 +5322,12 @@
           <t>Story 9 — Apply invoice to selected POs (SV-7704) | S9-R3</t>
         </is>
       </c>
+      <c r="J89" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K89" s="5" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" s="4" t="inlineStr">
@@ -4735,6 +5375,16 @@
           <t>S10-R1</t>
         </is>
       </c>
+      <c r="J90" s="2" t="inlineStr">
+        <is>
+          <t>reachable-now</t>
+        </is>
+      </c>
+      <c r="K90" s="4" t="inlineStr">
+        <is>
+          <t>no-PN PO line; inline Missing-part-number Edit -&gt; enter -&gt; save persists.</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="4" t="inlineStr">
@@ -4782,6 +5432,16 @@
           <t>S10 AC (new number)</t>
         </is>
       </c>
+      <c r="J91" s="4" t="inlineStr">
+        <is>
+          <t>needs-data</t>
+        </is>
+      </c>
+      <c r="K91" s="4" t="inlineStr">
+        <is>
+          <t>receiving + inventory/catalog inspection (new PN creates inventory part + stock + Part History on receive).</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="4" t="inlineStr">
@@ -4829,6 +5489,16 @@
           <t>S10 AC (existing number)</t>
         </is>
       </c>
+      <c r="J92" s="4" t="inlineStr">
+        <is>
+          <t>needs-data</t>
+        </is>
+      </c>
+      <c r="K92" s="4" t="inlineStr">
+        <is>
+          <t>receiving + inventory inspection (existing PN links to item, updates stock/cost/history).</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="4" t="inlineStr">
@@ -4876,6 +5546,16 @@
           <t>S10-R2 / S8-R7</t>
         </is>
       </c>
+      <c r="J93" s="4" t="inlineStr">
+        <is>
+          <t>needs-data</t>
+        </is>
+      </c>
+      <c r="K93" s="4" t="inlineStr">
+        <is>
+          <t>a WO in invoiced/paid state (sell-field locking).</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="4" t="inlineStr">
@@ -4923,6 +5603,16 @@
           <t>S10 Negative</t>
         </is>
       </c>
+      <c r="J94" s="4" t="inlineStr">
+        <is>
+          <t>needs-data</t>
+        </is>
+      </c>
+      <c r="K94" s="4" t="inlineStr">
+        <is>
+          <t>an invoiced/paid WO + a receive attempt (cannot receive without PN).</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="4" t="inlineStr">
@@ -4970,6 +5660,16 @@
           <t>S10 Technical guardrails</t>
         </is>
       </c>
+      <c r="J95" s="4" t="inlineStr">
+        <is>
+          <t>needs-data</t>
+        </is>
+      </c>
+      <c r="K95" s="4" t="inlineStr">
+        <is>
+          <t>receiving + catalog/inventory back-end inspection (real creation/linking, not a stored string).</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="4" t="inlineStr">
@@ -5017,6 +5717,16 @@
           <t>S11-R1</t>
         </is>
       </c>
+      <c r="J96" s="2" t="inlineStr">
+        <is>
+          <t>reachable-now</t>
+        </is>
+      </c>
+      <c r="K96" s="4" t="inlineStr">
+        <is>
+          <t>seed a WO-originated PO; confirm Receive action on PO list + detail.</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="4" t="inlineStr">
@@ -5064,6 +5774,16 @@
           <t>S11-R2</t>
         </is>
       </c>
+      <c r="J97" s="4" t="inlineStr">
+        <is>
+          <t>needs-data</t>
+        </is>
+      </c>
+      <c r="K97" s="4" t="inlineStr">
+        <is>
+          <t>an ordered/deliverable PO so the Receive action opens Accept Delivery (optional-flow Receive Parts routed back to the WO in VIU).</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -5111,6 +5831,12 @@
           <t>S11-R3</t>
         </is>
       </c>
+      <c r="J98" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K98" s="2" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -5158,6 +5884,12 @@
           <t>S12 (existing multi-vendor)</t>
         </is>
       </c>
+      <c r="J99" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K99" s="2" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" s="3" t="inlineStr">
@@ -5205,6 +5937,12 @@
           <t>Q11 | S12-R1</t>
         </is>
       </c>
+      <c r="J100" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K100" s="3" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" s="4" t="inlineStr">
@@ -5252,6 +5990,16 @@
           <t>S12-R2</t>
         </is>
       </c>
+      <c r="J101" s="4" t="inlineStr">
+        <is>
+          <t>needs-data</t>
+        </is>
+      </c>
+      <c r="K101" s="4" t="inlineStr">
+        <is>
+          <t>a deliverable PO to exercise Accept Delivery receive gates (vendor set, missing PN entered, invoice # captured).</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="3" t="inlineStr">
@@ -5299,6 +6047,12 @@
           <t>Q11 | S12-R3</t>
         </is>
       </c>
+      <c r="J102" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K102" s="3" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" s="4" t="inlineStr">
@@ -5346,6 +6100,16 @@
           <t>S12-R4</t>
         </is>
       </c>
+      <c r="J103" s="4" t="inlineStr">
+        <is>
+          <t>needs-data</t>
+        </is>
+      </c>
+      <c r="K103" s="4" t="inlineStr">
+        <is>
+          <t>QuickBooks inspection (per-vendor vendor bill + separate AP entry).</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="4" t="inlineStr">
@@ -5393,6 +6157,16 @@
           <t>S12 (existing) received-more-than-ordered</t>
         </is>
       </c>
+      <c r="J104" s="4" t="inlineStr">
+        <is>
+          <t>needs-data</t>
+        </is>
+      </c>
+      <c r="K104" s="4" t="inlineStr">
+        <is>
+          <t>a receive with received qty &gt; ordered qty (received-more-than-ordered warning).</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="4" t="inlineStr">
@@ -5440,6 +6214,16 @@
           <t>S13-R1</t>
         </is>
       </c>
+      <c r="J105" s="2" t="inlineStr">
+        <is>
+          <t>reachable-now</t>
+        </is>
+      </c>
+      <c r="K105" s="4" t="inlineStr">
+        <is>
+          <t>vendor-missing PO; confirm vendor dropdown assigns a vendor at PO level and saves.</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="4" t="inlineStr">
@@ -5487,6 +6271,16 @@
           <t>S13-R2</t>
         </is>
       </c>
+      <c r="J106" s="4" t="inlineStr">
+        <is>
+          <t>needs-data</t>
+        </is>
+      </c>
+      <c r="K106" s="4" t="inlineStr">
+        <is>
+          <t>a PO where the assigned vendor already exists on the PO (Add-to-vendor merge vs keep-separate prompt).</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="4" t="inlineStr">
@@ -5534,6 +6328,16 @@
           <t>S13-R3</t>
         </is>
       </c>
+      <c r="J107" s="4" t="inlineStr">
+        <is>
+          <t>needs-data</t>
+        </is>
+      </c>
+      <c r="K107" s="4" t="inlineStr">
+        <is>
+          <t>two POs for the same WO with the same vendor (merge-POs prompt).</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="4" t="inlineStr">
@@ -5581,6 +6385,16 @@
           <t>S13-R4 / S13-R5</t>
         </is>
       </c>
+      <c r="J108" s="4" t="inlineStr">
+        <is>
+          <t>needs-data</t>
+        </is>
+      </c>
+      <c r="K108" s="4" t="inlineStr">
+        <is>
+          <t>a vendor-missing PO + receive-enable + QB-flag-clear check after auto-assign.</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="4" t="inlineStr">
@@ -5628,6 +6442,16 @@
           <t>S13 Technical guardrails</t>
         </is>
       </c>
+      <c r="J109" s="4" t="inlineStr">
+        <is>
+          <t>needs-data</t>
+        </is>
+      </c>
+      <c r="K109" s="4" t="inlineStr">
+        <is>
+          <t>invoiced/paid WO + multi-PO merge guardrail state (match-by-ID, merge scoped to same WO, receive blocked when invoiced/paid).</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="5" t="inlineStr">
@@ -5675,6 +6499,12 @@
           <t>Story 14 — Waiting-on-Parts column (SV-7709) | S14-R1</t>
         </is>
       </c>
+      <c r="J110" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K110" s="5" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" s="5" t="inlineStr">
@@ -5722,6 +6552,12 @@
           <t>Story 14 — Waiting-on-Parts column (SV-7709) | S14-R2</t>
         </is>
       </c>
+      <c r="J111" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K111" s="5" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" s="5" t="inlineStr">
@@ -5769,6 +6605,12 @@
           <t>Story 14 — Waiting-on-Parts column (SV-7709) | S14-R3</t>
         </is>
       </c>
+      <c r="J112" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K112" s="5" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -5816,6 +6658,12 @@
           <t>R1</t>
         </is>
       </c>
+      <c r="J113" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K113" s="2" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -5863,6 +6711,12 @@
           <t>R2</t>
         </is>
       </c>
+      <c r="J114" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K114" s="2" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" s="4" t="inlineStr">
@@ -5910,6 +6764,16 @@
           <t>R3</t>
         </is>
       </c>
+      <c r="J115" s="2" t="inlineStr">
+        <is>
+          <t>reachable-now</t>
+        </is>
+      </c>
+      <c r="K115" s="4" t="inlineStr">
+        <is>
+          <t>enable Require Review; Details step collects mileage + engine hours (VIN captured later by reviewer).</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="4" t="inlineStr">
@@ -5957,6 +6821,16 @@
           <t>R4</t>
         </is>
       </c>
+      <c r="J116" s="4" t="inlineStr">
+        <is>
+          <t>needs-data</t>
+        </is>
+      </c>
+      <c r="K116" s="4" t="inlineStr">
+        <is>
+          <t>a deliverable PO in the review flow (Receive Parts routes to the shared receive page).</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -6004,6 +6878,12 @@
           <t>R5 / R6</t>
         </is>
       </c>
+      <c r="J117" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K117" s="2" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -6051,6 +6931,12 @@
           <t>R7 / R10</t>
         </is>
       </c>
+      <c r="J118" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K118" s="2" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" s="4" t="inlineStr">
@@ -6098,6 +6984,16 @@
           <t>R6</t>
         </is>
       </c>
+      <c r="J119" s="2" t="inlineStr">
+        <is>
+          <t>reachable-now</t>
+        </is>
+      </c>
+      <c r="K119" s="4" t="inlineStr">
+        <is>
+          <t>enable Require Review; Send to Review locks lines to Complete + auto-picks inventory.</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="3" t="inlineStr">
@@ -6145,6 +7041,12 @@
           <t>Q8, Q4 | R5 / R8 (distinct Reviewed state)</t>
         </is>
       </c>
+      <c r="J120" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K120" s="3" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" s="6" t="inlineStr">
@@ -6192,6 +7094,12 @@
           <t>R7 (role-gating) | see viu-findings BUGS #5/#6/#7</t>
         </is>
       </c>
+      <c r="J121" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K121" s="6" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" s="3" t="inlineStr">
@@ -6239,6 +7147,12 @@
           <t>Q7 | R7 / R10 (optional note)</t>
         </is>
       </c>
+      <c r="J122" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K122" s="3" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" s="3" t="inlineStr">
@@ -6286,6 +7200,12 @@
           <t>Q8 | R8</t>
         </is>
       </c>
+      <c r="J123" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K123" s="3" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" s="4" t="inlineStr">
@@ -6333,6 +7253,16 @@
           <t>R9</t>
         </is>
       </c>
+      <c r="J124" s="2" t="inlineStr">
+        <is>
+          <t>reachable-now</t>
+        </is>
+      </c>
+      <c r="K124" s="4" t="inlineStr">
+        <is>
+          <t>enable Require Review; confirm a 'Ready for Review' list filter/column.</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="4" t="inlineStr">
@@ -6380,6 +7310,16 @@
           <t>R11</t>
         </is>
       </c>
+      <c r="J125" s="2" t="inlineStr">
+        <is>
+          <t>reachable-now</t>
+        </is>
+      </c>
+      <c r="K125" s="4" t="inlineStr">
+        <is>
+          <t>enable Require Review; all lines must be approved to Send to Review (approve-line error).</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="4" t="inlineStr">
@@ -6427,6 +7367,16 @@
           <t>R Core parts / invoicing block</t>
         </is>
       </c>
+      <c r="J126" s="4" t="inlineStr">
+        <is>
+          <t>needs-data</t>
+        </is>
+      </c>
+      <c r="K126" s="4" t="inlineStr">
+        <is>
+          <t>cores + receiving in the review flow (cores resolved before sign-off; invoicing blocked until Reviewed + cores resolved).</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="3" t="inlineStr">
@@ -6474,6 +7424,12 @@
           <t>Q1 | R Open (default)</t>
         </is>
       </c>
+      <c r="J127" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K127" s="3" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -6521,6 +7477,12 @@
           <t>S15-R1</t>
         </is>
       </c>
+      <c r="J128" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K128" s="2" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -6568,6 +7530,12 @@
           <t>S15-R2</t>
         </is>
       </c>
+      <c r="J129" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K129" s="2" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -6615,6 +7583,12 @@
           <t>S15-R3</t>
         </is>
       </c>
+      <c r="J130" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K130" s="2" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" s="3" t="inlineStr">
@@ -6662,6 +7636,12 @@
           <t>Q10 | S15-R4</t>
         </is>
       </c>
+      <c r="J131" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K131" s="3" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -6709,6 +7689,12 @@
           <t>S1 AC / §8 Permissions</t>
         </is>
       </c>
+      <c r="J132" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K132" s="2" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" s="6" t="inlineStr">
@@ -6756,6 +7742,12 @@
           <t>§8 Permissions | see viu-findings BUGS #5/#6/#7</t>
         </is>
       </c>
+      <c r="J133" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K133" s="6" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" s="5" t="inlineStr">
@@ -6803,6 +7795,12 @@
           <t>Story 8 — PO Bulk Receive page (SV-7703) | §8 Permissions</t>
         </is>
       </c>
+      <c r="J134" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K134" s="5" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" s="6" t="inlineStr">
@@ -6850,6 +7848,12 @@
           <t>R7 / §8 role-gating review | see viu-findings BUGS #5/#6/#7</t>
         </is>
       </c>
+      <c r="J135" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K135" s="6" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -6897,6 +7901,12 @@
           <t>S11-R3</t>
         </is>
       </c>
+      <c r="J136" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K136" s="2" t="inlineStr"/>
     </row>
     <row r="137">
       <c r="A137" s="6" t="inlineStr">
@@ -6944,6 +7954,12 @@
           <t>§8 BE enforcement | see viu-findings BUGS #5/#6/#7</t>
         </is>
       </c>
+      <c r="J137" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K137" s="6" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" s="6" t="inlineStr">
@@ -6991,6 +8007,12 @@
           <t>§8 role-gating review | see viu-findings BUGS #5/#6/#7</t>
         </is>
       </c>
+      <c r="J138" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K138" s="6" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" s="6" t="inlineStr">
@@ -7038,53 +8060,65 @@
           <t>R7 (reviewer != completer) | see viu-findings BUGS #5/#6/#7</t>
         </is>
       </c>
+      <c r="J139" s="6" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K139" s="6" t="inlineStr"/>
     </row>
     <row r="140">
-      <c r="A140" s="4" t="inlineStr">
+      <c r="A140" s="2" t="inlineStr">
         <is>
           <t>SF-PERM-09</t>
         </is>
       </c>
-      <c r="B140" s="4" t="inlineStr">
+      <c r="B140" s="2" t="inlineStr">
         <is>
           <t>Permissions</t>
         </is>
       </c>
-      <c r="C140" s="4" t="inlineStr">
+      <c r="C140" s="2" t="inlineStr">
         <is>
           <t>Verify a Technician cannot add a vendorless / no-part-number part (lacks See Financial Data)</t>
         </is>
       </c>
-      <c r="D140" s="4" t="inlineStr">
-        <is>
-          <t>VIU-Pending</t>
-        </is>
-      </c>
-      <c r="E140" s="4" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
-        </is>
-      </c>
-      <c r="F140" s="4" t="inlineStr">
-        <is>
-          <t>VIU PENDING (QA)</t>
-        </is>
-      </c>
-      <c r="G140" s="4" t="inlineStr">
-        <is>
-          <t>QA (needs cookies+seed data)</t>
-        </is>
-      </c>
-      <c r="H140" s="4" t="inlineStr">
-        <is>
-          <t>QA VIU: a role account WITHOUT 'See Financial Data' to prove the vendorless part-add gate (tech confirmed no seeFinancialData; sub-form not reached).</t>
-        </is>
-      </c>
-      <c r="I140" s="4" t="inlineStr">
+      <c r="D140" s="2" t="inlineStr">
+        <is>
+          <t>VIU-Verified</t>
+        </is>
+      </c>
+      <c r="E140" s="2" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="F140" s="2" t="inlineStr">
+        <is>
+          <t>READY (VIU-Verified)</t>
+        </is>
+      </c>
+      <c r="G140" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H140" s="2" t="inlineStr">
+        <is>
+          <t>None — VIU-verified; uploadable now.</t>
+        </is>
+      </c>
+      <c r="I140" s="2" t="inlineStr">
         <is>
           <t>S5 / §9 (See Financial Data gate)</t>
         </is>
       </c>
+      <c r="J140" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K140" s="2" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" s="4" t="inlineStr">
@@ -7132,6 +8166,16 @@
           <t>§9 per-role completion matrix</t>
         </is>
       </c>
+      <c r="J141" s="5" t="inlineStr">
+        <is>
+          <t>needs-account</t>
+        </is>
+      </c>
+      <c r="K141" s="4" t="inlineStr">
+        <is>
+          <t>role accounts Office / Service Manager / Foreman (ideally also Senior SA / Parts Manager / Sales Rep / Time Clock) to run the per-role completion matrix (only admin+ and Technician- available).</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -7179,6 +8223,12 @@
           <t>S2-R2 / S3-R3 / S4-R3</t>
         </is>
       </c>
+      <c r="J142" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K142" s="2" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" s="4" t="inlineStr">
@@ -7226,53 +8276,69 @@
           <t>S15-R2 / S3-R3</t>
         </is>
       </c>
+      <c r="J143" s="4" t="inlineStr">
+        <is>
+          <t>needs-data</t>
+        </is>
+      </c>
+      <c r="K143" s="4" t="inlineStr">
+        <is>
+          <t>an asset/vehicle with NO VIN so the non-review wizard prompts for VIN (VIN is currently prefilled from the asset, so the gate is not reachable with existing assets).</t>
+        </is>
+      </c>
     </row>
     <row r="144">
-      <c r="A144" s="4" t="inlineStr">
+      <c r="A144" s="2" t="inlineStr">
         <is>
           <t>SF-VAL-03</t>
         </is>
       </c>
-      <c r="B144" s="4" t="inlineStr">
+      <c r="B144" s="2" t="inlineStr">
         <is>
           <t>Validation / Edge</t>
         </is>
       </c>
-      <c r="C144" s="4" t="inlineStr">
+      <c r="C144" s="2" t="inlineStr">
         <is>
           <t>Verify completion is blocked when required engine hours are missing</t>
         </is>
       </c>
-      <c r="D144" s="4" t="inlineStr">
-        <is>
-          <t>VIU-Pending</t>
-        </is>
-      </c>
-      <c r="E144" s="4" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
-        </is>
-      </c>
-      <c r="F144" s="4" t="inlineStr">
-        <is>
-          <t>VIU PENDING (QA)</t>
-        </is>
-      </c>
-      <c r="G144" s="4" t="inlineStr">
-        <is>
-          <t>QA (needs cookies+seed data)</t>
-        </is>
-      </c>
-      <c r="H144" s="4" t="inlineStr">
-        <is>
-          <t>QA VIU: drive the specific validation/edge scenario with seeded data.</t>
-        </is>
-      </c>
-      <c r="I144" s="4" t="inlineStr">
+      <c r="D144" s="2" t="inlineStr">
+        <is>
+          <t>VIU-Verified</t>
+        </is>
+      </c>
+      <c r="E144" s="2" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="F144" s="2" t="inlineStr">
+        <is>
+          <t>READY (VIU-Verified)</t>
+        </is>
+      </c>
+      <c r="G144" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H144" s="2" t="inlineStr">
+        <is>
+          <t>None — VIU-verified; uploadable now.</t>
+        </is>
+      </c>
+      <c r="I144" s="2" t="inlineStr">
         <is>
           <t>S3-R3 / S4-R3</t>
         </is>
       </c>
+      <c r="J144" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K144" s="2" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -7320,6 +8386,12 @@
           <t>TS-R4</t>
         </is>
       </c>
+      <c r="J145" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K145" s="2" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" s="4" t="inlineStr">
@@ -7367,6 +8439,16 @@
           <t>S3-R3 / S4-R5 / §4</t>
         </is>
       </c>
+      <c r="J146" s="4" t="inlineStr">
+        <is>
+          <t>needs-data</t>
+        </is>
+      </c>
+      <c r="K146" s="4" t="inlineStr">
+        <is>
+          <t>a required-invoice receive attempt without an invoice number (receivable PO).</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="4" t="inlineStr">
@@ -7414,6 +8496,16 @@
           <t>S10 / S12-R2 / S13</t>
         </is>
       </c>
+      <c r="J147" s="4" t="inlineStr">
+        <is>
+          <t>needs-data</t>
+        </is>
+      </c>
+      <c r="K147" s="4" t="inlineStr">
+        <is>
+          <t>a vendor-missing part receive attempt (deliverable state).</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="4" t="inlineStr">
@@ -7461,6 +8553,16 @@
           <t>R7</t>
         </is>
       </c>
+      <c r="J148" s="2" t="inlineStr">
+        <is>
+          <t>reachable-now</t>
+        </is>
+      </c>
+      <c r="K148" s="4" t="inlineStr">
+        <is>
+          <t>review flow; Confirm Review disabled until VIN entered in Mark Reviewed dialog.</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="4" t="inlineStr">
@@ -7508,6 +8610,16 @@
           <t>S3-R9 (idempotency)</t>
         </is>
       </c>
+      <c r="J149" s="2" t="inlineStr">
+        <is>
+          <t>reachable-now</t>
+        </is>
+      </c>
+      <c r="K149" s="4" t="inlineStr">
+        <is>
+          <t>re-complete after cancelling; check no duplicate POs.</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="5" t="inlineStr">
@@ -7555,6 +8667,12 @@
           <t>Story 8 — Bulk Receive field locking (S8-R7, SV-7703) | S8-R7 / §4 field locking</t>
         </is>
       </c>
+      <c r="J150" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K150" s="5" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" s="5" t="inlineStr">
@@ -7602,6 +8720,12 @@
           <t>Story 9 — Apply-invoice uniqueness (S9-R3, SV-7704) | S9-R3 / §4 (uniqueness relaxed)</t>
         </is>
       </c>
+      <c r="J151" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K151" s="5" t="inlineStr"/>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -7649,6 +8773,12 @@
           <t>Key Decision (line approval)</t>
         </is>
       </c>
+      <c r="J152" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K152" s="2" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" s="3" t="inlineStr">
@@ -7696,6 +8826,12 @@
           <t>Q2 | §5 invariant 1</t>
         </is>
       </c>
+      <c r="J153" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K153" s="3" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" s="3" t="inlineStr">
@@ -7743,6 +8879,12 @@
           <t>Q5 | §5 / §4 (Create POs OFF)</t>
         </is>
       </c>
+      <c r="J154" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K154" s="3" t="inlineStr"/>
     </row>
     <row r="155">
       <c r="A155" s="4" t="inlineStr">
@@ -7790,6 +8932,16 @@
           <t>§5 invariant 2</t>
         </is>
       </c>
+      <c r="J155" s="4" t="inlineStr">
+        <is>
+          <t>needs-data</t>
+        </is>
+      </c>
+      <c r="K155" s="4" t="inlineStr">
+        <is>
+          <t>QuickBooks / inventory back-end inspection (receive -&gt; Delivery -&gt; Vendor Bill -&gt; QBO) — likely needs dev/QB access.</t>
+        </is>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="4" t="inlineStr">
@@ -7837,6 +8989,16 @@
           <t>§5 (vendorless/no-PN)</t>
         </is>
       </c>
+      <c r="J156" s="4" t="inlineStr">
+        <is>
+          <t>needs-data</t>
+        </is>
+      </c>
+      <c r="K156" s="4" t="inlineStr">
+        <is>
+          <t>QuickBooks / inventory inspection (vendorless/no-PN part = zero inventory interaction) — likely needs dev/QB access.</t>
+        </is>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="4" t="inlineStr">
@@ -7884,6 +9046,16 @@
           <t>§5 / S6-R3</t>
         </is>
       </c>
+      <c r="J157" s="4" t="inlineStr">
+        <is>
+          <t>needs-data</t>
+        </is>
+      </c>
+      <c r="K157" s="4" t="inlineStr">
+        <is>
+          <t>QuickBooks inspection (Vendor-Missing POs excluded from QB until vendor + PN) — likely needs dev/QB access.</t>
+        </is>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="4" t="inlineStr">
@@ -7931,6 +9103,16 @@
           <t>§8 (cost at completion)</t>
         </is>
       </c>
+      <c r="J158" s="4" t="inlineStr">
+        <is>
+          <t>needs-data</t>
+        </is>
+      </c>
+      <c r="K158" s="4" t="inlineStr">
+        <is>
+          <t>QuickBooks inspection (cost-at-completion to avoid $0-cost margins) — likely needs dev/QB access.</t>
+        </is>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="4" t="inlineStr">
@@ -7978,6 +9160,16 @@
           <t>§5 (Journal Entry / Inventory → QBO)</t>
         </is>
       </c>
+      <c r="J159" s="4" t="inlineStr">
+        <is>
+          <t>needs-data</t>
+        </is>
+      </c>
+      <c r="K159" s="4" t="inlineStr">
+        <is>
+          <t>QuickBooks inspection (Journal Entry / Inventory sync fires on invoice creation) — likely needs dev/QB access.</t>
+        </is>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="4" t="inlineStr">
@@ -8023,6 +9215,16 @@
       <c r="I160" s="4" t="inlineStr">
         <is>
           <t>§5 invariant 3</t>
+        </is>
+      </c>
+      <c r="J160" s="4" t="inlineStr">
+        <is>
+          <t>needs-data</t>
+        </is>
+      </c>
+      <c r="K160" s="4" t="inlineStr">
+        <is>
+          <t>Inventory Part History inspection for any part that becomes inventory-tracked — likely needs dev/QB access.</t>
         </is>
       </c>
     </row>
@@ -8037,7 +9239,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C27"/>
+  <dimension ref="A1:C33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -8099,7 +9301,7 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>42</v>
+        <v>54</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
@@ -8129,7 +9331,7 @@
         </is>
       </c>
       <c r="B8" s="4" t="n">
-        <v>71</v>
+        <v>59</v>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
@@ -8246,101 +9448,101 @@
       <c r="C18" s="8" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="11" t="inlineStr">
-        <is>
-          <t>WHAT TO SEND ME NEXT (to unblock each batch)</t>
-        </is>
-      </c>
-      <c r="B19" s="8" t="n"/>
-      <c r="C19" s="8" t="n"/>
+      <c r="A19" s="10" t="inlineStr">
+        <is>
+          <t>VIU PENDING (QA) — by sub-bucket</t>
+        </is>
+      </c>
+      <c r="B19" s="10" t="inlineStr">
+        <is>
+          <t>Count</t>
+        </is>
+      </c>
+      <c r="C19" s="10" t="inlineStr">
+        <is>
+          <t>Meaning</t>
+        </is>
+      </c>
     </row>
     <row r="20">
-      <c r="A20" s="10" t="inlineStr">
-        <is>
-          <t>• Milos's answers to the 11 Open Questions</t>
-        </is>
-      </c>
-      <c r="B20" s="8" t="inlineStr">
-        <is>
-          <t>unblocks 15 cases (all the MILOS-ANSWER rows). Send the filled-in OpenQuestions-for-Milos sheet.</t>
-        </is>
-      </c>
-      <c r="C20" s="8" t="n"/>
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>reachable-now</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="C20" s="8" t="inlineStr">
+        <is>
+          <t>admin+tech + normal data; just needs another VIU pass (no new inputs).</t>
+        </is>
+      </c>
     </row>
     <row r="21">
-      <c r="A21" s="10" t="inlineStr">
-        <is>
-          <t>• Dev deploys Story 8 — PO Bulk Receive page (SV-7703)</t>
-        </is>
-      </c>
-      <c r="B21" s="8" t="inlineStr">
-        <is>
-          <t>unblocks 12 case(s); then I re-run VIU and send an update file.</t>
-        </is>
-      </c>
-      <c r="C21" s="8" t="n"/>
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>needs-data</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="n">
+        <v>39</v>
+      </c>
+      <c r="C21" s="8" t="inlineStr">
+        <is>
+          <t>needs a data state not seedable via the app (see per-case detail).</t>
+        </is>
+      </c>
     </row>
     <row r="22">
-      <c r="A22" s="10" t="inlineStr">
-        <is>
-          <t>• Dev deploys Story 7 — PO multi-select (SV-7702)</t>
-        </is>
-      </c>
-      <c r="B22" s="8" t="inlineStr">
-        <is>
-          <t>unblocks 6 case(s); then I re-run VIU and send an update file.</t>
-        </is>
-      </c>
-      <c r="C22" s="8" t="n"/>
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>needs-account</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="C22" s="8" t="inlineStr">
+        <is>
+          <t>needs a role account we don't have (see per-case detail).</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="10" t="inlineStr">
         <is>
-          <t>• Dev deploys Story 9 — Apply invoice to selected POs (SV-7704)</t>
-        </is>
-      </c>
-      <c r="B23" s="8" t="inlineStr">
-        <is>
-          <t>unblocks 4 case(s); then I re-run VIU and send an update file.</t>
-        </is>
-      </c>
-      <c r="C23" s="8" t="n"/>
+          <t>TOTAL VIU PENDING (QA)</t>
+        </is>
+      </c>
+      <c r="B23" s="10" t="n">
+        <v>59</v>
+      </c>
+      <c r="C23" s="8" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" s="10" t="inlineStr">
-        <is>
-          <t>• Dev deploys Story 14 — Waiting-on-Parts column (SV-7709)</t>
-        </is>
-      </c>
-      <c r="B24" s="8" t="inlineStr">
-        <is>
-          <t>unblocks 3 case(s); then I re-run VIU and send an update file.</t>
-        </is>
-      </c>
+      <c r="A24" s="8" t="n"/>
+      <c r="B24" s="8" t="n"/>
       <c r="C24" s="8" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="10" t="inlineStr">
-        <is>
-          <t>• Fresh QA cookies for sv7301 (admin + tech) + seeded test data</t>
-        </is>
-      </c>
-      <c r="B25" s="8" t="inlineStr">
-        <is>
-          <t>unblocks the bulk of the 71 VIU-PENDING (QA) cases (cores, receiving, vendor, validation round-trips).</t>
-        </is>
-      </c>
+      <c r="A25" s="11" t="inlineStr">
+        <is>
+          <t>WHAT TO SEND ME NEXT (to unblock each batch)</t>
+        </is>
+      </c>
+      <c r="B25" s="8" t="n"/>
       <c r="C25" s="8" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="10" t="inlineStr">
         <is>
-          <t>• A 2nd/3rd role account (Office, Service Manager, Foreman) — some WITHOUT 'See Financial Data'</t>
+          <t>• Milos's answers to the 11 Open Questions</t>
         </is>
       </c>
       <c r="B26" s="8" t="inlineStr">
         <is>
-          <t>unblocks SF-PERM-09 and SF-PERM-10 (per-role completion + vendorless-add gate).</t>
+          <t>unblocks 15 cases (all the MILOS-ANSWER rows). Send the filled-in OpenQuestions-for-Milos sheet.</t>
         </is>
       </c>
       <c r="C26" s="8" t="n"/>
@@ -8348,15 +9550,93 @@
     <row r="27">
       <c r="A27" s="10" t="inlineStr">
         <is>
+          <t>• Dev deploys Story 8 — PO Bulk Receive page (SV-7703)</t>
+        </is>
+      </c>
+      <c r="B27" s="8" t="inlineStr">
+        <is>
+          <t>unblocks 12 case(s); then I re-run VIU and send an update file.</t>
+        </is>
+      </c>
+      <c r="C27" s="8" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="10" t="inlineStr">
+        <is>
+          <t>• Dev deploys Story 7 — PO multi-select (SV-7702)</t>
+        </is>
+      </c>
+      <c r="B28" s="8" t="inlineStr">
+        <is>
+          <t>unblocks 6 case(s); then I re-run VIU and send an update file.</t>
+        </is>
+      </c>
+      <c r="C28" s="8" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="10" t="inlineStr">
+        <is>
+          <t>• Dev deploys Story 9 — Apply invoice to selected POs (SV-7704)</t>
+        </is>
+      </c>
+      <c r="B29" s="8" t="inlineStr">
+        <is>
+          <t>unblocks 4 case(s); then I re-run VIU and send an update file.</t>
+        </is>
+      </c>
+      <c r="C29" s="8" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="10" t="inlineStr">
+        <is>
+          <t>• Dev deploys Story 14 — Waiting-on-Parts column (SV-7709)</t>
+        </is>
+      </c>
+      <c r="B30" s="8" t="inlineStr">
+        <is>
+          <t>unblocks 3 case(s); then I re-run VIU and send an update file.</t>
+        </is>
+      </c>
+      <c r="C30" s="8" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="10" t="inlineStr">
+        <is>
+          <t>• Fresh QA cookies for sv7301 (admin + tech) + seeded test data</t>
+        </is>
+      </c>
+      <c r="B31" s="8" t="inlineStr">
+        <is>
+          <t>unblocks the bulk of the 59 VIU-PENDING (QA) cases (cores, receiving, vendor, validation round-trips).</t>
+        </is>
+      </c>
+      <c r="C31" s="8" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="10" t="inlineStr">
+        <is>
+          <t>• A 2nd/3rd role account (Office, Service Manager, Foreman) — some WITHOUT 'See Financial Data'</t>
+        </is>
+      </c>
+      <c r="B32" s="8" t="inlineStr">
+        <is>
+          <t>unblocks SF-PERM-09 and SF-PERM-10 (per-role completion + vendorless-add gate).</t>
+        </is>
+      </c>
+      <c r="C32" s="8" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="10" t="inlineStr">
+        <is>
           <t>• A dev/PO ruling on FE-only BE enforcement + the missing reviewer!=completer rule (resolve SV-8183 'BE enforces' vs SV-7864 atom-collapse)</t>
         </is>
       </c>
-      <c r="B27" s="8" t="inlineStr">
+      <c r="B33" s="8" t="inlineStr">
         <is>
           <t>finalizes the 6 BUG/RULING cases.</t>
         </is>
       </c>
-      <c r="C27" s="8" t="n"/>
+      <c r="C33" s="8" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Simple Flow: self-service VIU pass — seed data + role matrix
Verified 5 cases (VIU-Pending -> VIU-Verified): SF-COMP-23, SF-VAL-08 (PO
idempotency), SF-SET-10 (settings future-only), SF-RCV-01 (Receive on WO PO),
SF-PERM-10 (per-role completion matrix via self-service Tech role-swap).

Proved self-service Tech role-switching (POST /api/staff/{id}/change), seeded +
deleted one throwaway WO, restored settings + Tech role. READY 54->59, VIU
pending 59->54 (needs-account 1->0). No new bugs; TestRail import unchanged.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AZ5XzKsK9wv7M41cSPaMyg
</commit_message>
<xml_diff>
--- a/build/simple-flow/SimpleFlow_Blockers_Tracker.xlsx
+++ b/build/simple-flow/SimpleFlow_Blockers_Tracker.xlsx
@@ -1043,61 +1043,57 @@
       <c r="K10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="inlineStr">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>SF-SET-10</t>
         </is>
       </c>
-      <c r="B11" s="4" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>Work Order Settings</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr">
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t>Verify a settings change applies to future completions only and not to already-completed work orders</t>
         </is>
       </c>
-      <c r="D11" s="4" t="inlineStr">
-        <is>
-          <t>VIU-Pending</t>
-        </is>
-      </c>
-      <c r="E11" s="4" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
-        </is>
-      </c>
-      <c r="F11" s="4" t="inlineStr">
-        <is>
-          <t>VIU PENDING (QA)</t>
-        </is>
-      </c>
-      <c r="G11" s="4" t="inlineStr">
-        <is>
-          <t>QA (needs cookies+seed data)</t>
-        </is>
-      </c>
-      <c r="H11" s="4" t="inlineStr">
-        <is>
-          <t>QA VIU: toggle the setting and confirm the downstream behaviour.</t>
-        </is>
-      </c>
-      <c r="I11" s="4" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>VIU-Verified</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>READY (VIU-Verified)</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>None — VIU-verified; uploadable now.</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>S1-R9 (future completions only, never retroactive)</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>reachable-now</t>
-        </is>
-      </c>
-      <c r="K11" s="4" t="inlineStr">
-        <is>
-          <t>admin+tech + normal WO data; needs another VIU pass (no new inputs).</t>
-        </is>
-      </c>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -2555,61 +2551,57 @@
       <c r="K38" s="2" t="inlineStr"/>
     </row>
     <row r="39">
-      <c r="A39" s="4" t="inlineStr">
+      <c r="A39" s="2" t="inlineStr">
         <is>
           <t>SF-COMP-23</t>
         </is>
       </c>
-      <c r="B39" s="4" t="inlineStr">
+      <c r="B39" s="2" t="inlineStr">
         <is>
           <t>Completion — Idempotency</t>
         </is>
       </c>
-      <c r="C39" s="4" t="inlineStr">
+      <c r="C39" s="2" t="inlineStr">
         <is>
           <t>Verify re-running completion after a prior attempt does not create duplicate POs</t>
         </is>
       </c>
-      <c r="D39" s="4" t="inlineStr">
-        <is>
-          <t>VIU-Pending</t>
-        </is>
-      </c>
-      <c r="E39" s="4" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
-        </is>
-      </c>
-      <c r="F39" s="4" t="inlineStr">
-        <is>
-          <t>VIU PENDING (QA)</t>
-        </is>
-      </c>
-      <c r="G39" s="4" t="inlineStr">
-        <is>
-          <t>QA (needs cookies+seed data)</t>
-        </is>
-      </c>
-      <c r="H39" s="4" t="inlineStr">
-        <is>
-          <t>QA VIU: seed the specific completion configuration and drive the wizard to Success.</t>
-        </is>
-      </c>
-      <c r="I39" s="4" t="inlineStr">
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>VIU-Verified</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>READY (VIU-Verified)</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H39" s="2" t="inlineStr">
+        <is>
+          <t>None — VIU-verified; uploadable now.</t>
+        </is>
+      </c>
+      <c r="I39" s="2" t="inlineStr">
         <is>
           <t>S3-R9 (no duplicate POs on re-Complete)</t>
         </is>
       </c>
       <c r="J39" s="2" t="inlineStr">
         <is>
-          <t>reachable-now</t>
-        </is>
-      </c>
-      <c r="K39" s="4" t="inlineStr">
-        <is>
-          <t>re-run completion after a prior attempt; check no duplicate POs.</t>
-        </is>
-      </c>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K39" s="2" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
@@ -5672,61 +5664,57 @@
       </c>
     </row>
     <row r="96">
-      <c r="A96" s="4" t="inlineStr">
+      <c r="A96" s="2" t="inlineStr">
         <is>
           <t>SF-RCV-01</t>
         </is>
       </c>
-      <c r="B96" s="4" t="inlineStr">
+      <c r="B96" s="2" t="inlineStr">
         <is>
           <t>Receive Button on WO POs (Story 11)</t>
         </is>
       </c>
-      <c r="C96" s="4" t="inlineStr">
+      <c r="C96" s="2" t="inlineStr">
         <is>
           <t>Verify a Receive action appears on WO-originated POs in both the PO list and the PO detail card</t>
         </is>
       </c>
-      <c r="D96" s="4" t="inlineStr">
-        <is>
-          <t>VIU-Pending</t>
-        </is>
-      </c>
-      <c r="E96" s="4" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
-        </is>
-      </c>
-      <c r="F96" s="4" t="inlineStr">
-        <is>
-          <t>VIU PENDING (QA)</t>
-        </is>
-      </c>
-      <c r="G96" s="4" t="inlineStr">
-        <is>
-          <t>QA (needs cookies+seed data)</t>
-        </is>
-      </c>
-      <c r="H96" s="4" t="inlineStr">
-        <is>
-          <t>QA VIU: seed deliverable POs, drive the Receive / Accept-Delivery flow.</t>
-        </is>
-      </c>
-      <c r="I96" s="4" t="inlineStr">
+      <c r="D96" s="2" t="inlineStr">
+        <is>
+          <t>VIU-Verified</t>
+        </is>
+      </c>
+      <c r="E96" s="2" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="F96" s="2" t="inlineStr">
+        <is>
+          <t>READY (VIU-Verified)</t>
+        </is>
+      </c>
+      <c r="G96" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H96" s="2" t="inlineStr">
+        <is>
+          <t>None — VIU-verified; uploadable now.</t>
+        </is>
+      </c>
+      <c r="I96" s="2" t="inlineStr">
         <is>
           <t>S11-R1</t>
         </is>
       </c>
       <c r="J96" s="2" t="inlineStr">
         <is>
-          <t>reachable-now</t>
-        </is>
-      </c>
-      <c r="K96" s="4" t="inlineStr">
-        <is>
-          <t>seed a WO-originated PO; confirm Receive action on PO list + detail.</t>
-        </is>
-      </c>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K96" s="2" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" s="4" t="inlineStr">
@@ -8121,61 +8109,57 @@
       <c r="K140" s="2" t="inlineStr"/>
     </row>
     <row r="141">
-      <c r="A141" s="4" t="inlineStr">
+      <c r="A141" s="2" t="inlineStr">
         <is>
           <t>SF-PERM-10</t>
         </is>
       </c>
-      <c r="B141" s="4" t="inlineStr">
+      <c r="B141" s="2" t="inlineStr">
         <is>
           <t>Permissions</t>
         </is>
       </c>
-      <c r="C141" s="4" t="inlineStr">
+      <c r="C141" s="2" t="inlineStr">
         <is>
           <t>Verify the Complete Work Order action follows the per-role completion permission matrix</t>
         </is>
       </c>
-      <c r="D141" s="4" t="inlineStr">
-        <is>
-          <t>VIU-Pending</t>
-        </is>
-      </c>
-      <c r="E141" s="4" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
-        </is>
-      </c>
-      <c r="F141" s="4" t="inlineStr">
-        <is>
-          <t>VIU PENDING (QA)</t>
-        </is>
-      </c>
-      <c r="G141" s="4" t="inlineStr">
-        <is>
-          <t>QA (needs cookies+seed data)</t>
-        </is>
-      </c>
-      <c r="H141" s="4" t="inlineStr">
-        <is>
-          <t>QA VIU: additional role accounts (Office / Service Manager / Foreman) to run the per-role completion matrix (only Technician-negative confirmed).</t>
-        </is>
-      </c>
-      <c r="I141" s="4" t="inlineStr">
+      <c r="D141" s="2" t="inlineStr">
+        <is>
+          <t>VIU-Verified</t>
+        </is>
+      </c>
+      <c r="E141" s="2" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="F141" s="2" t="inlineStr">
+        <is>
+          <t>READY (VIU-Verified)</t>
+        </is>
+      </c>
+      <c r="G141" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H141" s="2" t="inlineStr">
+        <is>
+          <t>None — VIU-verified; uploadable now.</t>
+        </is>
+      </c>
+      <c r="I141" s="2" t="inlineStr">
         <is>
           <t>§9 per-role completion matrix</t>
         </is>
       </c>
-      <c r="J141" s="5" t="inlineStr">
-        <is>
-          <t>needs-account</t>
-        </is>
-      </c>
-      <c r="K141" s="4" t="inlineStr">
-        <is>
-          <t>role accounts Office / Service Manager / Foreman (ideally also Senior SA / Parts Manager / Sales Rep / Time Clock) to run the per-role completion matrix (only admin+ and Technician- available).</t>
-        </is>
-      </c>
+      <c r="J141" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K141" s="2" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -8565,61 +8549,57 @@
       </c>
     </row>
     <row r="149">
-      <c r="A149" s="4" t="inlineStr">
+      <c r="A149" s="2" t="inlineStr">
         <is>
           <t>SF-VAL-08</t>
         </is>
       </c>
-      <c r="B149" s="4" t="inlineStr">
+      <c r="B149" s="2" t="inlineStr">
         <is>
           <t>Validation / Edge</t>
         </is>
       </c>
-      <c r="C149" s="4" t="inlineStr">
+      <c r="C149" s="2" t="inlineStr">
         <is>
           <t>Verify re-completing after cancelling does not create duplicate POs</t>
         </is>
       </c>
-      <c r="D149" s="4" t="inlineStr">
-        <is>
-          <t>VIU-Pending</t>
-        </is>
-      </c>
-      <c r="E149" s="4" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
-        </is>
-      </c>
-      <c r="F149" s="4" t="inlineStr">
-        <is>
-          <t>VIU PENDING (QA)</t>
-        </is>
-      </c>
-      <c r="G149" s="4" t="inlineStr">
-        <is>
-          <t>QA (needs cookies+seed data)</t>
-        </is>
-      </c>
-      <c r="H149" s="4" t="inlineStr">
-        <is>
-          <t>QA VIU: drive the specific validation/edge scenario with seeded data.</t>
-        </is>
-      </c>
-      <c r="I149" s="4" t="inlineStr">
+      <c r="D149" s="2" t="inlineStr">
+        <is>
+          <t>VIU-Verified</t>
+        </is>
+      </c>
+      <c r="E149" s="2" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="F149" s="2" t="inlineStr">
+        <is>
+          <t>READY (VIU-Verified)</t>
+        </is>
+      </c>
+      <c r="G149" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H149" s="2" t="inlineStr">
+        <is>
+          <t>None — VIU-verified; uploadable now.</t>
+        </is>
+      </c>
+      <c r="I149" s="2" t="inlineStr">
         <is>
           <t>S3-R9 (idempotency)</t>
         </is>
       </c>
       <c r="J149" s="2" t="inlineStr">
         <is>
-          <t>reachable-now</t>
-        </is>
-      </c>
-      <c r="K149" s="4" t="inlineStr">
-        <is>
-          <t>re-complete after cancelling; check no duplicate POs.</t>
-        </is>
-      </c>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K149" s="2" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" s="5" t="inlineStr">
@@ -9301,7 +9281,7 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
@@ -9331,7 +9311,7 @@
         </is>
       </c>
       <c r="B8" s="4" t="n">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
@@ -9471,7 +9451,7 @@
         </is>
       </c>
       <c r="B20" s="2" t="n">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="C20" s="8" t="inlineStr">
         <is>
@@ -9501,7 +9481,7 @@
         </is>
       </c>
       <c r="B22" s="5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C22" s="8" t="inlineStr">
         <is>
@@ -9516,7 +9496,7 @@
         </is>
       </c>
       <c r="B23" s="10" t="n">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="C23" s="8" t="inlineStr"/>
     </row>
@@ -9607,7 +9587,7 @@
       </c>
       <c r="B31" s="8" t="inlineStr">
         <is>
-          <t>unblocks the bulk of the 59 VIU-PENDING (QA) cases (cores, receiving, vendor, validation round-trips).</t>
+          <t>unblocks the bulk of the 54 VIU-PENDING (QA) cases (cores, receiving, vendor, validation round-trips).</t>
         </is>
       </c>
       <c r="C31" s="8" t="n"/>

</xml_diff>

<commit_message>
Simple Flow: VIU pass — full role matrix + receive + cores
BATCH 5 (sv7301 QA, self-service): corrected memory (all 11 system roles are
REAL/assignable, not templates); ran full LIVE 11-role completion matrix
(SF-PERM-10) matching §9.2 exactly; drove the Accept Delivery receive round-trip
on PO 93fb82e9 (SF-RCV-02 shared surface, SF-RCV-09 over-qty warning); seeded a
genuine cored inventory part (P550848) and found BUG-10 (no Resolve-Cores step in
the completion wizard for a pre-picked inventory core). Settings + Tech role
restored, created WOs deleted, inventory returned. Regenerated tracker + workbook.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AZ5XzKsK9wv7M41cSPaMyg
</commit_message>
<xml_diff>
--- a/build/simple-flow/SimpleFlow_Blockers_Tracker.xlsx
+++ b/build/simple-flow/SimpleFlow_Blockers_Tracker.xlsx
@@ -5717,61 +5717,57 @@
       <c r="K96" s="2" t="inlineStr"/>
     </row>
     <row r="97">
-      <c r="A97" s="4" t="inlineStr">
+      <c r="A97" s="2" t="inlineStr">
         <is>
           <t>SF-RCV-02</t>
         </is>
       </c>
-      <c r="B97" s="4" t="inlineStr">
+      <c r="B97" s="2" t="inlineStr">
         <is>
           <t>Receive Button on WO POs (Story 11)</t>
         </is>
       </c>
-      <c r="C97" s="4" t="inlineStr">
+      <c r="C97" s="2" t="inlineStr">
         <is>
           <t>Verify the Receive action opens the shared Accept Delivery surface</t>
         </is>
       </c>
-      <c r="D97" s="4" t="inlineStr">
-        <is>
-          <t>VIU-Pending</t>
-        </is>
-      </c>
-      <c r="E97" s="4" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
-        </is>
-      </c>
-      <c r="F97" s="4" t="inlineStr">
-        <is>
-          <t>VIU PENDING (QA)</t>
-        </is>
-      </c>
-      <c r="G97" s="4" t="inlineStr">
-        <is>
-          <t>QA (needs cookies+seed data)</t>
-        </is>
-      </c>
-      <c r="H97" s="4" t="inlineStr">
-        <is>
-          <t>QA VIU: seed deliverable POs, drive the Receive / Accept-Delivery flow.</t>
-        </is>
-      </c>
-      <c r="I97" s="4" t="inlineStr">
+      <c r="D97" s="2" t="inlineStr">
+        <is>
+          <t>VIU-Verified</t>
+        </is>
+      </c>
+      <c r="E97" s="2" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="F97" s="2" t="inlineStr">
+        <is>
+          <t>READY (VIU-Verified)</t>
+        </is>
+      </c>
+      <c r="G97" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H97" s="2" t="inlineStr">
+        <is>
+          <t>None — VIU-verified; uploadable now.</t>
+        </is>
+      </c>
+      <c r="I97" s="2" t="inlineStr">
         <is>
           <t>S11-R2</t>
         </is>
       </c>
-      <c r="J97" s="4" t="inlineStr">
-        <is>
-          <t>needs-data</t>
-        </is>
-      </c>
-      <c r="K97" s="4" t="inlineStr">
-        <is>
-          <t>an ordered/deliverable PO so the Receive action opens Accept Delivery (optional-flow Receive Parts routed back to the WO in VIU).</t>
-        </is>
-      </c>
+      <c r="J97" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K97" s="2" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -5978,14 +5974,14 @@
           <t>S12-R2</t>
         </is>
       </c>
-      <c r="J101" s="4" t="inlineStr">
-        <is>
-          <t>needs-data</t>
+      <c r="J101" s="2" t="inlineStr">
+        <is>
+          <t>reachable-now</t>
         </is>
       </c>
       <c r="K101" s="4" t="inlineStr">
         <is>
-          <t>a deliverable PO to exercise Accept Delivery receive gates (vendor set, missing PN entered, invoice # captured).</t>
+          <t>BATCH 5: Accept Delivery happy path driven on PO 93fb82e9 (vendor set, invoice # captured -&gt; Receive 201). Only the NEGATIVE sub-gates remain (receive blocked with vendor unset / missing PN) — need a vendor-missing item on an Accept Delivery group (seedable by completing a WO with vendorless vendor parts).</t>
         </is>
       </c>
     </row>
@@ -6100,61 +6096,57 @@
       </c>
     </row>
     <row r="104">
-      <c r="A104" s="4" t="inlineStr">
+      <c r="A104" s="2" t="inlineStr">
         <is>
           <t>SF-RCV-09</t>
         </is>
       </c>
-      <c r="B104" s="4" t="inlineStr">
+      <c r="B104" s="2" t="inlineStr">
         <is>
           <t>Accept Delivery (Story 12)</t>
         </is>
       </c>
-      <c r="C104" s="4" t="inlineStr">
+      <c r="C104" s="2" t="inlineStr">
         <is>
           <t>Verify a 'received more than ordered' warning appears when received quantity exceeds ordered quantity</t>
         </is>
       </c>
-      <c r="D104" s="4" t="inlineStr">
-        <is>
-          <t>VIU-Pending</t>
-        </is>
-      </c>
-      <c r="E104" s="4" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
-        </is>
-      </c>
-      <c r="F104" s="4" t="inlineStr">
-        <is>
-          <t>VIU PENDING (QA)</t>
-        </is>
-      </c>
-      <c r="G104" s="4" t="inlineStr">
-        <is>
-          <t>QA (needs cookies+seed data)</t>
-        </is>
-      </c>
-      <c r="H104" s="4" t="inlineStr">
-        <is>
-          <t>QA VIU: seed deliverable POs, drive the Receive / Accept-Delivery flow.</t>
-        </is>
-      </c>
-      <c r="I104" s="4" t="inlineStr">
+      <c r="D104" s="2" t="inlineStr">
+        <is>
+          <t>VIU-Verified</t>
+        </is>
+      </c>
+      <c r="E104" s="2" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="F104" s="2" t="inlineStr">
+        <is>
+          <t>READY (VIU-Verified)</t>
+        </is>
+      </c>
+      <c r="G104" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H104" s="2" t="inlineStr">
+        <is>
+          <t>None — VIU-verified; uploadable now.</t>
+        </is>
+      </c>
+      <c r="I104" s="2" t="inlineStr">
         <is>
           <t>S12 (existing) received-more-than-ordered</t>
         </is>
       </c>
-      <c r="J104" s="4" t="inlineStr">
-        <is>
-          <t>needs-data</t>
-        </is>
-      </c>
-      <c r="K104" s="4" t="inlineStr">
-        <is>
-          <t>a receive with received qty &gt; ordered qty (received-more-than-ordered warning).</t>
-        </is>
-      </c>
+      <c r="J104" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K104" s="2" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" s="4" t="inlineStr">
@@ -9281,7 +9273,7 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
@@ -9311,7 +9303,7 @@
         </is>
       </c>
       <c r="B8" s="4" t="n">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
@@ -9451,7 +9443,7 @@
         </is>
       </c>
       <c r="B20" s="2" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C20" s="8" t="inlineStr">
         <is>
@@ -9466,7 +9458,7 @@
         </is>
       </c>
       <c r="B21" s="4" t="n">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="C21" s="8" t="inlineStr">
         <is>
@@ -9496,7 +9488,7 @@
         </is>
       </c>
       <c r="B23" s="10" t="n">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C23" s="8" t="inlineStr"/>
     </row>
@@ -9587,7 +9579,7 @@
       </c>
       <c r="B31" s="8" t="inlineStr">
         <is>
-          <t>unblocks the bulk of the 54 VIU-PENDING (QA) cases (cores, receiving, vendor, validation round-trips).</t>
+          <t>unblocks the bulk of the 52 VIU-PENDING (QA) cases (cores, receiving, vendor, validation round-trips).</t>
         </is>
       </c>
       <c r="C31" s="8" t="n"/>

</xml_diff>

<commit_message>
Simple Flow: apply Milos Round-2 answers
Fetched Milos's Round-2 answers and applied the clear spec-decisions to case
expecteds, pushed 5 cases to TestRail (update_case, all 200 verified):
- SF-REV-10: review note descoped (VIN-only) — BUG-3 closed
- SF-VPART-01/02: Category required, Sell Price not enforced (intended) — BUG-9 closed
- SF-PERM-06: UI gating = v1 pass; BE gap (BUG-6/7) noted for fix
- SF-TECH-08: Story 17 confirmed authoritative (open question closed)
Q3 (inventory decrement invariant) confirmed — SF-COMP-07/SF-QB-01 expected
already correct (annotated, not pushed). Regenerated workbook + blockers tracker;
updated bugs-log, PROJECT-STATE, and milos-round2-mapping.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AZ5XzKsK9wv7M41cSPaMyg
</commit_message>
<xml_diff>
--- a/build/simple-flow/SimpleFlow_Blockers_Tracker.xlsx
+++ b/build/simple-flow/SimpleFlow_Blockers_Tracker.xlsx
@@ -3546,7 +3546,7 @@
       </c>
       <c r="D57" s="3" t="inlineStr">
         <is>
-          <t>Open-Question</t>
+          <t>VIU-Verified</t>
         </is>
       </c>
       <c r="E57" s="3" t="inlineStr">
@@ -3582,118 +3582,110 @@
       <c r="K57" s="3" t="inlineStr"/>
     </row>
     <row r="58">
-      <c r="A58" s="4" t="inlineStr">
+      <c r="A58" s="2" t="inlineStr">
         <is>
           <t>SF-VPART-01</t>
         </is>
       </c>
-      <c r="B58" s="4" t="inlineStr">
+      <c r="B58" s="2" t="inlineStr">
         <is>
           <t>Vendorless / No-PN Part (Story 5)</t>
         </is>
       </c>
-      <c r="C58" s="4" t="inlineStr">
-        <is>
-          <t>Verify a part can be requested with only description, quantity and sell price (part number, cost, vendor empty)</t>
-        </is>
-      </c>
-      <c r="D58" s="4" t="inlineStr">
-        <is>
-          <t>VIU-Pending</t>
-        </is>
-      </c>
-      <c r="E58" s="4" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
-        </is>
-      </c>
-      <c r="F58" s="4" t="inlineStr">
-        <is>
-          <t>VIU PENDING (QA)</t>
-        </is>
-      </c>
-      <c r="G58" s="4" t="inlineStr">
-        <is>
-          <t>QA (needs cookies+seed data)</t>
-        </is>
-      </c>
-      <c r="H58" s="4" t="inlineStr">
-        <is>
-          <t>QA VIU: seed + drive the vendorless / no-PN part add flow.</t>
-        </is>
-      </c>
-      <c r="I58" s="4" t="inlineStr">
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>Verify a vendorless part can be requested with description, quantity and category (part number, cost, vendor and sell price left empty)</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>VIU-Verified</t>
+        </is>
+      </c>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="F58" s="2" t="inlineStr">
+        <is>
+          <t>READY (VIU-Verified)</t>
+        </is>
+      </c>
+      <c r="G58" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H58" s="2" t="inlineStr">
+        <is>
+          <t>None — VIU-verified; uploadable now.</t>
+        </is>
+      </c>
+      <c r="I58" s="2" t="inlineStr">
         <is>
           <t>S5-R1</t>
         </is>
       </c>
       <c r="J58" s="2" t="inlineStr">
         <is>
-          <t>reachable-now</t>
-        </is>
-      </c>
-      <c r="K58" s="4" t="inlineStr">
-        <is>
-          <t>admin+tech + normal WO data; needs another VIU pass (no new inputs).</t>
-        </is>
-      </c>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K58" s="2" t="inlineStr"/>
     </row>
     <row r="59">
-      <c r="A59" s="4" t="inlineStr">
+      <c r="A59" s="2" t="inlineStr">
         <is>
           <t>SF-VPART-02</t>
         </is>
       </c>
-      <c r="B59" s="4" t="inlineStr">
+      <c r="B59" s="2" t="inlineStr">
         <is>
           <t>Vendorless / No-PN Part (Story 5)</t>
         </is>
       </c>
-      <c r="C59" s="4" t="inlineStr">
-        <is>
-          <t>Verify adding a part is blocked when description, quantity or sell price is missing</t>
-        </is>
-      </c>
-      <c r="D59" s="4" t="inlineStr">
-        <is>
-          <t>VIU-Pending</t>
-        </is>
-      </c>
-      <c r="E59" s="4" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
-        </is>
-      </c>
-      <c r="F59" s="4" t="inlineStr">
-        <is>
-          <t>VIU PENDING (QA)</t>
-        </is>
-      </c>
-      <c r="G59" s="4" t="inlineStr">
-        <is>
-          <t>QA (needs cookies+seed data)</t>
-        </is>
-      </c>
-      <c r="H59" s="4" t="inlineStr">
-        <is>
-          <t>QA VIU: drive the vendorless / no-PN add sub-form validation (not reached in the last session's budget).</t>
-        </is>
-      </c>
-      <c r="I59" s="4" t="inlineStr">
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>Verify adding a part is blocked when description, quantity or category is missing (sell price not enforced)</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="inlineStr">
+        <is>
+          <t>VIU-Verified</t>
+        </is>
+      </c>
+      <c r="E59" s="2" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="F59" s="2" t="inlineStr">
+        <is>
+          <t>READY (VIU-Verified)</t>
+        </is>
+      </c>
+      <c r="G59" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H59" s="2" t="inlineStr">
+        <is>
+          <t>None — VIU-verified; uploadable now.</t>
+        </is>
+      </c>
+      <c r="I59" s="2" t="inlineStr">
         <is>
           <t>S5-R1 / S5 AC (validation)</t>
         </is>
       </c>
       <c r="J59" s="2" t="inlineStr">
         <is>
-          <t>reachable-now</t>
-        </is>
-      </c>
-      <c r="K59" s="4" t="inlineStr">
-        <is>
-          <t>admin+tech + normal WO data; needs another VIU pass (no new inputs).</t>
-        </is>
-      </c>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K59" s="2" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -7184,12 +7176,12 @@
       </c>
       <c r="C124" s="3" t="inlineStr">
         <is>
-          <t>Verify the Mark Reviewed dialog includes VIN (required) and an optional review note field (input_review_note)</t>
+          <t>Verify the Mark Reviewed dialog includes VIN / Serial # (required) with no review note field</t>
         </is>
       </c>
       <c r="D124" s="3" t="inlineStr">
         <is>
-          <t>VIU-Pending</t>
+          <t>VIU-Verified</t>
         </is>
       </c>
       <c r="E124" s="3" t="inlineStr">
@@ -7214,7 +7206,7 @@
       </c>
       <c r="I124" s="3" t="inlineStr">
         <is>
-          <t>Q7 | R7 / R10 (optional note)</t>
+          <t>Q7 | R7 (VIN required, no note)</t>
         </is>
       </c>
       <c r="J124" s="3" t="inlineStr">
@@ -7987,7 +7979,7 @@
       </c>
       <c r="C139" s="6" t="inlineStr">
         <is>
-          <t>Verify the backend enforces the Simple-Flow settings and permission atoms (not front-end only)</t>
+          <t>Verify permission gating of Simple-Flow settings and work-order actions (UI gating is the v1 pass criterion)</t>
         </is>
       </c>
       <c r="D139" s="6" t="inlineStr">
@@ -9412,7 +9404,7 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
@@ -9442,7 +9434,7 @@
         </is>
       </c>
       <c r="B8" s="4" t="n">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
@@ -9582,7 +9574,7 @@
         </is>
       </c>
       <c r="B20" s="2" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C20" s="8" t="inlineStr">
         <is>
@@ -9627,7 +9619,7 @@
         </is>
       </c>
       <c r="B23" s="10" t="n">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C23" s="8" t="inlineStr"/>
     </row>
@@ -9718,7 +9710,7 @@
       </c>
       <c r="B31" s="8" t="inlineStr">
         <is>
-          <t>unblocks the bulk of the 47 VIU-PENDING (QA) cases (cores, receiving, vendor, validation round-trips).</t>
+          <t>unblocks the bulk of the 45 VIU-PENDING (QA) cases (cores, receiving, vendor, validation round-trips).</t>
         </is>
       </c>
       <c r="C31" s="8" t="n"/>

</xml_diff>

<commit_message>
Simple Flow VIU 2026-07-10 batch 2: 5 bulk-receive cases verified
Bulk Receive pipeline (POST /api/orders/receive-requested-parts 200) — BUG-11 not reproduced:
- SF-VAL-05: required-invoice receive gate (disabled w/o invoice#, enabled with) on WO PO S-15797.
- SF-COMP-19: received deliverable WO PO S-15797 via /bulk-receive; completion then reached
  Success with no waiting-to-receive step (Complete enabled once all received).
- SF-VAL-06: vendor-missing receive needs BOTH vendor + PN (WO PO S-15798; assign-vendor 200).
- SF-VPART-07: no-PN part not receivable until PN+vendor entered; PN persists to order item.
- SF-PNFIX-01: inline PN-fix on Bulk Receive persists immediately (order item.part_number set);
  BATCH-6 'Story 8 not built' note superseded.
Tracker + results regenerated; PROJECT-STATE tally: READY 111 / VIU-PENDING(QA) 34 / MILOS 13 / BUG-RULING 4.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AZ5XzKsK9wv7M41cSPaMyg
</commit_message>
<xml_diff>
--- a/build/simple-flow/SimpleFlow_Blockers_Tracker.xlsx
+++ b/build/simple-flow/SimpleFlow_Blockers_Tracker.xlsx
@@ -2323,61 +2323,57 @@
       <c r="K34" s="2" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="A35" s="4" t="inlineStr">
+      <c r="A35" s="2" t="inlineStr">
         <is>
           <t>SF-COMP-19</t>
         </is>
       </c>
-      <c r="B35" s="4" t="inlineStr">
+      <c r="B35" s="2" t="inlineStr">
         <is>
           <t>Completion — PO + Required Invoice (Story 4)</t>
         </is>
       </c>
-      <c r="C35" s="4" t="inlineStr">
+      <c r="C35" s="2" t="inlineStr">
         <is>
           <t>Verify the required-invoice receive round-trip returns to the modal and enables Complete once all received</t>
         </is>
       </c>
-      <c r="D35" s="4" t="inlineStr">
-        <is>
-          <t>VIU-Pending</t>
-        </is>
-      </c>
-      <c r="E35" s="4" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
-        </is>
-      </c>
-      <c r="F35" s="4" t="inlineStr">
-        <is>
-          <t>VIU PENDING (QA)</t>
-        </is>
-      </c>
-      <c r="G35" s="4" t="inlineStr">
-        <is>
-          <t>QA (needs cookies+seed data)</t>
-        </is>
-      </c>
-      <c r="H35" s="4" t="inlineStr">
-        <is>
-          <t>QA VIU: seed the specific completion configuration and drive the wizard to Success.</t>
-        </is>
-      </c>
-      <c r="I35" s="4" t="inlineStr">
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>VIU-Verified</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>READY (VIU-Verified)</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>None — VIU-verified; uploadable now.</t>
+        </is>
+      </c>
+      <c r="I35" s="2" t="inlineStr">
         <is>
           <t>S4-R5 / S4-R7</t>
         </is>
       </c>
-      <c r="J35" s="4" t="inlineStr">
-        <is>
-          <t>needs-data</t>
-        </is>
-      </c>
-      <c r="K35" s="4" t="inlineStr">
-        <is>
-          <t>BATCH 6: deliverable WO PO achieved, but the receive round-trip is blocked by BUG-11 (POST /api/inventory/orders/accept returns 500 for a WO PO).</t>
-        </is>
-      </c>
+      <c r="J35" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K35" s="2" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -3896,61 +3892,57 @@
       <c r="K63" s="2" t="inlineStr"/>
     </row>
     <row r="64">
-      <c r="A64" s="4" t="inlineStr">
+      <c r="A64" s="2" t="inlineStr">
         <is>
           <t>SF-VPART-07</t>
         </is>
       </c>
-      <c r="B64" s="4" t="inlineStr">
+      <c r="B64" s="2" t="inlineStr">
         <is>
           <t>Vendorless / No-PN Part (Story 5)</t>
         </is>
       </c>
-      <c r="C64" s="4" t="inlineStr">
+      <c r="C64" s="2" t="inlineStr">
         <is>
           <t>Verify a vendorless / no-PN part cannot be received until a part number (and vendor) is entered</t>
         </is>
       </c>
-      <c r="D64" s="4" t="inlineStr">
-        <is>
-          <t>VIU-Pending</t>
-        </is>
-      </c>
-      <c r="E64" s="4" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
-        </is>
-      </c>
-      <c r="F64" s="4" t="inlineStr">
-        <is>
-          <t>VIU PENDING (QA)</t>
-        </is>
-      </c>
-      <c r="G64" s="4" t="inlineStr">
-        <is>
-          <t>QA (needs cookies+seed data)</t>
-        </is>
-      </c>
-      <c r="H64" s="4" t="inlineStr">
-        <is>
-          <t>QA VIU: seed + drive the vendorless / no-PN part add flow.</t>
-        </is>
-      </c>
-      <c r="I64" s="4" t="inlineStr">
+      <c r="D64" s="2" t="inlineStr">
+        <is>
+          <t>VIU-Verified</t>
+        </is>
+      </c>
+      <c r="E64" s="2" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="F64" s="2" t="inlineStr">
+        <is>
+          <t>READY (VIU-Verified)</t>
+        </is>
+      </c>
+      <c r="G64" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H64" s="2" t="inlineStr">
+        <is>
+          <t>None — VIU-verified; uploadable now.</t>
+        </is>
+      </c>
+      <c r="I64" s="2" t="inlineStr">
         <is>
           <t>S5-R4 / S5 AC (receive gate)</t>
         </is>
       </c>
-      <c r="J64" s="4" t="inlineStr">
-        <is>
-          <t>needs-data</t>
-        </is>
-      </c>
-      <c r="K64" s="4" t="inlineStr">
-        <is>
-          <t>BATCH 6: deliverable WO PO achievable, but receiving it is blocked by BUG-11 (500), so the cannot-receive-until-PN+vendor proof cannot complete.</t>
-        </is>
-      </c>
+      <c r="J64" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K64" s="2" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -5343,61 +5335,57 @@
       <c r="K90" s="2" t="inlineStr"/>
     </row>
     <row r="91">
-      <c r="A91" s="4" t="inlineStr">
+      <c r="A91" s="2" t="inlineStr">
         <is>
           <t>SF-PNFIX-01</t>
         </is>
       </c>
-      <c r="B91" s="4" t="inlineStr">
+      <c r="B91" s="2" t="inlineStr">
         <is>
           <t>Inline Part-Number Fix (Story 10)</t>
         </is>
       </c>
-      <c r="C91" s="4" t="inlineStr">
+      <c r="C91" s="2" t="inlineStr">
         <is>
           <t>Verify a no-number part shows 'Missing part number' with Edit → enter → save that persists immediately</t>
         </is>
       </c>
-      <c r="D91" s="4" t="inlineStr">
-        <is>
-          <t>VIU-Pending</t>
-        </is>
-      </c>
-      <c r="E91" s="4" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
-        </is>
-      </c>
-      <c r="F91" s="4" t="inlineStr">
-        <is>
-          <t>VIU PENDING (QA)</t>
-        </is>
-      </c>
-      <c r="G91" s="4" t="inlineStr">
-        <is>
-          <t>QA (needs cookies+seed data)</t>
-        </is>
-      </c>
-      <c r="H91" s="4" t="inlineStr">
-        <is>
-          <t>QA VIU: drive the inline part-number fix flow with seeded PO lines.</t>
-        </is>
-      </c>
-      <c r="I91" s="4" t="inlineStr">
+      <c r="D91" s="2" t="inlineStr">
+        <is>
+          <t>VIU-Verified</t>
+        </is>
+      </c>
+      <c r="E91" s="2" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="F91" s="2" t="inlineStr">
+        <is>
+          <t>READY (VIU-Verified)</t>
+        </is>
+      </c>
+      <c r="G91" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H91" s="2" t="inlineStr">
+        <is>
+          <t>None — VIU-verified; uploadable now.</t>
+        </is>
+      </c>
+      <c r="I91" s="2" t="inlineStr">
         <is>
           <t>S10-R1</t>
         </is>
       </c>
-      <c r="J91" s="4" t="inlineStr">
-        <is>
-          <t>needs-data</t>
-        </is>
-      </c>
-      <c r="K91" s="4" t="inlineStr">
-        <is>
-          <t>BATCH 6: no inline Missing-part-number Edit on the vendor-missing PO Accept Delivery (empty PN cell, no edit control). Inline PN-fix appears tied to the Bulk Receive page (Story 8, NOT built).</t>
-        </is>
-      </c>
+      <c r="J91" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K91" s="2" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" s="4" t="inlineStr">
@@ -8416,118 +8404,110 @@
       <c r="K147" s="2" t="inlineStr"/>
     </row>
     <row r="148">
-      <c r="A148" s="4" t="inlineStr">
+      <c r="A148" s="2" t="inlineStr">
         <is>
           <t>SF-VAL-05</t>
         </is>
       </c>
-      <c r="B148" s="4" t="inlineStr">
+      <c r="B148" s="2" t="inlineStr">
         <is>
           <t>Validation / Edge</t>
         </is>
       </c>
-      <c r="C148" s="4" t="inlineStr">
+      <c r="C148" s="2" t="inlineStr">
         <is>
           <t>Verify a required-invoice receive is blocked without a vendor invoice number</t>
         </is>
       </c>
-      <c r="D148" s="4" t="inlineStr">
-        <is>
-          <t>VIU-Pending</t>
-        </is>
-      </c>
-      <c r="E148" s="4" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
-        </is>
-      </c>
-      <c r="F148" s="4" t="inlineStr">
-        <is>
-          <t>VIU PENDING (QA)</t>
-        </is>
-      </c>
-      <c r="G148" s="4" t="inlineStr">
-        <is>
-          <t>QA (needs cookies+seed data)</t>
-        </is>
-      </c>
-      <c r="H148" s="4" t="inlineStr">
-        <is>
-          <t>QA VIU: drive the specific validation/edge scenario with seeded data.</t>
-        </is>
-      </c>
-      <c r="I148" s="4" t="inlineStr">
+      <c r="D148" s="2" t="inlineStr">
+        <is>
+          <t>VIU-Verified</t>
+        </is>
+      </c>
+      <c r="E148" s="2" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="F148" s="2" t="inlineStr">
+        <is>
+          <t>READY (VIU-Verified)</t>
+        </is>
+      </c>
+      <c r="G148" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H148" s="2" t="inlineStr">
+        <is>
+          <t>None — VIU-verified; uploadable now.</t>
+        </is>
+      </c>
+      <c r="I148" s="2" t="inlineStr">
         <is>
           <t>S3-R3 / S4-R5 / §4</t>
         </is>
       </c>
-      <c r="J148" s="4" t="inlineStr">
-        <is>
-          <t>needs-data</t>
-        </is>
-      </c>
-      <c r="K148" s="4" t="inlineStr">
-        <is>
-          <t>BATCH 6: blocked by BUG-11 (WO-PO receive 500) — cannot complete a required-invoice receive to test the no-invoice-number negative.</t>
-        </is>
-      </c>
+      <c r="J148" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K148" s="2" t="inlineStr"/>
     </row>
     <row r="149">
-      <c r="A149" s="4" t="inlineStr">
+      <c r="A149" s="2" t="inlineStr">
         <is>
           <t>SF-VAL-06</t>
         </is>
       </c>
-      <c r="B149" s="4" t="inlineStr">
+      <c r="B149" s="2" t="inlineStr">
         <is>
           <t>Validation / Edge</t>
         </is>
       </c>
-      <c r="C149" s="4" t="inlineStr">
+      <c r="C149" s="2" t="inlineStr">
         <is>
           <t>Verify a vendor-missing part cannot be received without both a vendor and a part number</t>
         </is>
       </c>
-      <c r="D149" s="4" t="inlineStr">
-        <is>
-          <t>VIU-Pending</t>
-        </is>
-      </c>
-      <c r="E149" s="4" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
-        </is>
-      </c>
-      <c r="F149" s="4" t="inlineStr">
-        <is>
-          <t>VIU PENDING (QA)</t>
-        </is>
-      </c>
-      <c r="G149" s="4" t="inlineStr">
-        <is>
-          <t>QA (needs cookies+seed data)</t>
-        </is>
-      </c>
-      <c r="H149" s="4" t="inlineStr">
-        <is>
-          <t>QA VIU: drive the specific validation/edge scenario with seeded data.</t>
-        </is>
-      </c>
-      <c r="I149" s="4" t="inlineStr">
+      <c r="D149" s="2" t="inlineStr">
+        <is>
+          <t>VIU-Verified</t>
+        </is>
+      </c>
+      <c r="E149" s="2" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="F149" s="2" t="inlineStr">
+        <is>
+          <t>READY (VIU-Verified)</t>
+        </is>
+      </c>
+      <c r="G149" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H149" s="2" t="inlineStr">
+        <is>
+          <t>None — VIU-verified; uploadable now.</t>
+        </is>
+      </c>
+      <c r="I149" s="2" t="inlineStr">
         <is>
           <t>S10 / S12-R2 / S13</t>
         </is>
       </c>
-      <c r="J149" s="4" t="inlineStr">
-        <is>
-          <t>needs-data</t>
-        </is>
-      </c>
-      <c r="K149" s="4" t="inlineStr">
-        <is>
-          <t>BATCH 6: blocked by BUG-11 (WO-PO receive 500) and no assign-vendor UI on the reachable receive surface.</t>
-        </is>
-      </c>
+      <c r="J149" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K149" s="2" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -9380,7 +9360,7 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
@@ -9410,7 +9390,7 @@
         </is>
       </c>
       <c r="B8" s="4" t="n">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
@@ -9521,7 +9501,7 @@
         </is>
       </c>
       <c r="B17" s="4" t="n">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="C17" s="7" t="inlineStr">
         <is>
@@ -9551,7 +9531,7 @@
         </is>
       </c>
       <c r="B19" s="10" t="n">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="C19" s="7" t="inlineStr"/>
     </row>
@@ -9590,7 +9570,7 @@
       </c>
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t>unblocks the bulk of the 39 VIU-PENDING (QA) cases (cores, receiving, vendor, validation round-trips).</t>
+          <t>unblocks the bulk of the 34 VIU-PENDING (QA) cases (cores, receiving, vendor, validation round-trips).</t>
         </is>
       </c>
       <c r="C23" s="7" t="n"/>

</xml_diff>

<commit_message>
Simple Flow VIU 2026-07-10 batch 3: SF-COMP-13 + SF-REV-04 verified (Receive Parts navigation)
- SF-COMP-13: optional-invoice wizard 'Receive Parts' navigates to the consolidated
  shared receive page /bulk-receive ('Receive Vendor Parts', all vendors) — OBS-5.
- SF-REV-04: review-flow wizard ('Send To Review'); receive step has NO inline modal;
  'Receive Parts' routes to /bulk-receive. Settings toggled then restored to baseline.
- SF-PNFIX-02/03/06 noted STILL BLOCKED: received vendor free-text PN creates no
  inventory part (vendor-source = direct consumption); inventory/Part-History surface
  OBS-6-blocked.
Tracker + results regenerated; READY 113 / VIU-PENDING(QA) 32 / MILOS 13 / BUG-RULING 4.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AZ5XzKsK9wv7M41cSPaMyg
</commit_message>
<xml_diff>
--- a/build/simple-flow/SimpleFlow_Blockers_Tracker.xlsx
+++ b/build/simple-flow/SimpleFlow_Blockers_Tracker.xlsx
@@ -2001,61 +2001,57 @@
       <c r="K28" s="2" t="inlineStr"/>
     </row>
     <row r="29">
-      <c r="A29" s="4" t="inlineStr">
+      <c r="A29" s="2" t="inlineStr">
         <is>
           <t>SF-COMP-13</t>
         </is>
       </c>
-      <c r="B29" s="4" t="inlineStr">
+      <c r="B29" s="2" t="inlineStr">
         <is>
           <t>Completion — PO + Optional Invoice (Story 3)</t>
         </is>
       </c>
-      <c r="C29" s="4" t="inlineStr">
+      <c r="C29" s="2" t="inlineStr">
         <is>
           <t>Verify Receive Parts opens the shared Accept Delivery page to receive all vendors at once</t>
         </is>
       </c>
-      <c r="D29" s="4" t="inlineStr">
-        <is>
-          <t>VIU-Pending</t>
-        </is>
-      </c>
-      <c r="E29" s="4" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
-        </is>
-      </c>
-      <c r="F29" s="4" t="inlineStr">
-        <is>
-          <t>VIU PENDING (QA)</t>
-        </is>
-      </c>
-      <c r="G29" s="4" t="inlineStr">
-        <is>
-          <t>QA (needs cookies+seed data)</t>
-        </is>
-      </c>
-      <c r="H29" s="4" t="inlineStr">
-        <is>
-          <t>QA VIU: seed the specific completion configuration and drive the wizard to Success.</t>
-        </is>
-      </c>
-      <c r="I29" s="4" t="inlineStr">
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>VIU-Verified</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>READY (VIU-Verified)</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>None — VIU-verified; uploadable now.</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="inlineStr">
         <is>
           <t>S3-R5</t>
         </is>
       </c>
-      <c r="J29" s="4" t="inlineStr">
-        <is>
-          <t>needs-data</t>
-        </is>
-      </c>
-      <c r="K29" s="4" t="inlineStr">
-        <is>
-          <t>BATCH 6: a deliverable ORDERED WO PO IS now achievable (Source=Vendor + real vendor + free-text PN). The shared Accept Delivery page opens for it via the PO Receive action, BUT the completion WIZARD Receive Parts still routes back to the WO lines (PO not placed until completion), and receiving the WO PO 500s (BUG-11).</t>
-        </is>
-      </c>
+      <c r="J29" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K29" s="2" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -6802,61 +6798,57 @@
       <c r="K117" s="2" t="inlineStr"/>
     </row>
     <row r="118">
-      <c r="A118" s="4" t="inlineStr">
+      <c r="A118" s="2" t="inlineStr">
         <is>
           <t>SF-REV-04</t>
         </is>
       </c>
-      <c r="B118" s="4" t="inlineStr">
+      <c r="B118" s="2" t="inlineStr">
         <is>
           <t>Review ON (Story 16)</t>
         </is>
       </c>
-      <c r="C118" s="4" t="inlineStr">
+      <c r="C118" s="2" t="inlineStr">
         <is>
           <t>Verify 'Receive Parts' routes to the shared receive page (no inline modal) in the review flow</t>
         </is>
       </c>
-      <c r="D118" s="4" t="inlineStr">
-        <is>
-          <t>VIU-Pending</t>
-        </is>
-      </c>
-      <c r="E118" s="4" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
-        </is>
-      </c>
-      <c r="F118" s="4" t="inlineStr">
-        <is>
-          <t>VIU PENDING (QA)</t>
-        </is>
-      </c>
-      <c r="G118" s="4" t="inlineStr">
-        <is>
-          <t>QA (needs cookies+seed data)</t>
-        </is>
-      </c>
-      <c r="H118" s="4" t="inlineStr">
-        <is>
-          <t>QA VIU: enable Require Review and drive the review/sign-off round-trip.</t>
-        </is>
-      </c>
-      <c r="I118" s="4" t="inlineStr">
+      <c r="D118" s="2" t="inlineStr">
+        <is>
+          <t>VIU-Verified</t>
+        </is>
+      </c>
+      <c r="E118" s="2" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="F118" s="2" t="inlineStr">
+        <is>
+          <t>READY (VIU-Verified)</t>
+        </is>
+      </c>
+      <c r="G118" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H118" s="2" t="inlineStr">
+        <is>
+          <t>None — VIU-verified; uploadable now.</t>
+        </is>
+      </c>
+      <c r="I118" s="2" t="inlineStr">
         <is>
           <t>R4</t>
         </is>
       </c>
-      <c r="J118" s="4" t="inlineStr">
-        <is>
-          <t>needs-data</t>
-        </is>
-      </c>
-      <c r="K118" s="4" t="inlineStr">
-        <is>
-          <t>BATCH 6: deliverable WO PO achievable in the review flow, but receiving it is blocked by BUG-11 (500).</t>
-        </is>
-      </c>
+      <c r="J118" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K118" s="2" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -9360,7 +9352,7 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
@@ -9390,7 +9382,7 @@
         </is>
       </c>
       <c r="B8" s="4" t="n">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
@@ -9501,7 +9493,7 @@
         </is>
       </c>
       <c r="B17" s="4" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C17" s="7" t="inlineStr">
         <is>
@@ -9531,7 +9523,7 @@
         </is>
       </c>
       <c r="B19" s="10" t="n">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C19" s="7" t="inlineStr"/>
     </row>
@@ -9570,7 +9562,7 @@
       </c>
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t>unblocks the bulk of the 34 VIU-PENDING (QA) cases (cores, receiving, vendor, validation round-trips).</t>
+          <t>unblocks the bulk of the 32 VIU-PENDING (QA) cases (cores, receiving, vendor, validation round-trips).</t>
         </is>
       </c>
       <c r="C23" s="7" t="n"/>

</xml_diff>

<commit_message>
Simple Flow VIU 2026-07-10 batch 4: SF-COMP-08 verified (completion Pick step); run wrap-up
- SF-COMP-08 -> VIU-Verified: with auto-pick OFF, completion wizard shows a Pick step
  (section_wizard_pick / button_pick_all / text_unpicked_parts_count); cannot complete
  until picked; after Pick All -> 'All parts picked' -> Complete proceeds.
- SF-VAL-02 confirmed still blocked (no seedable VIN-less asset; POST /api/vehicles 405).
- Cleanup: all throwaway WOs deleted (0 ZZAUTOTEST remain); settings restored to run
  baseline (verified); Tech never swapped (still Technician). Residual: P550848 net 6->4
  + irreversible received deliveries S-15797/S-15798.
Final run tally: VIU-Verified 121 / VIU-Pending 36 / OQ 5; READY 114 / VIU-PENDING(QA) 31 / MILOS 13 / BUG-RULING 4 (9 cases flipped this run).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AZ5XzKsK9wv7M41cSPaMyg
</commit_message>
<xml_diff>
--- a/build/simple-flow/SimpleFlow_Blockers_Tracker.xlsx
+++ b/build/simple-flow/SimpleFlow_Blockers_Tracker.xlsx
@@ -1732,61 +1732,57 @@
       <c r="K23" s="2" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" s="4" t="inlineStr">
+      <c r="A24" s="2" t="inlineStr">
         <is>
           <t>SF-COMP-08</t>
         </is>
       </c>
-      <c r="B24" s="4" t="inlineStr">
+      <c r="B24" s="2" t="inlineStr">
         <is>
           <t>Completion — No-PO / Skip (Story 2)</t>
         </is>
       </c>
-      <c r="C24" s="4" t="inlineStr">
+      <c r="C24" s="2" t="inlineStr">
         <is>
           <t>Verify with Auto-pick Inventory OFF the completion modal requires picking parts before Complete</t>
         </is>
       </c>
-      <c r="D24" s="4" t="inlineStr">
-        <is>
-          <t>VIU-Pending</t>
-        </is>
-      </c>
-      <c r="E24" s="4" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
-        </is>
-      </c>
-      <c r="F24" s="4" t="inlineStr">
-        <is>
-          <t>VIU PENDING (QA)</t>
-        </is>
-      </c>
-      <c r="G24" s="4" t="inlineStr">
-        <is>
-          <t>QA (needs cookies+seed data)</t>
-        </is>
-      </c>
-      <c r="H24" s="4" t="inlineStr">
-        <is>
-          <t>QA VIU: seed the specific completion configuration and drive the wizard to Success.</t>
-        </is>
-      </c>
-      <c r="I24" s="4" t="inlineStr">
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>VIU-Verified</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>READY (VIU-Verified)</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>None — VIU-verified; uploadable now.</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
         <is>
           <t>S2-R2 / S2 AC (auto-pick off ⇒ pick in modal)</t>
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>reachable-now</t>
-        </is>
-      </c>
-      <c r="K24" s="4" t="inlineStr">
-        <is>
-          <t>FRESH VIU 2026-07-10: with autoPickInventoryParts=OFF, an added inventory part stays 'in_stock' and simple-complete is BE-BLOCKED (400 'All inventory and found parts must be picked...'); after line-level Pick it completes (201) — expected #2/#3 PROVEN. Remaining: surface the completion-WIZARD Pick step UI ('Pick all from default bins'/'Review individually') for expected #1 (drive the completion modal, not line-level pick).</t>
-        </is>
-      </c>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K24" s="2" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -9352,7 +9348,7 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
@@ -9382,7 +9378,7 @@
         </is>
       </c>
       <c r="B8" s="4" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
@@ -9478,7 +9474,7 @@
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
@@ -9523,7 +9519,7 @@
         </is>
       </c>
       <c r="B19" s="10" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C19" s="7" t="inlineStr"/>
     </row>
@@ -9562,7 +9558,7 @@
       </c>
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t>unblocks the bulk of the 32 VIU-PENDING (QA) cases (cores, receiving, vendor, validation round-trips).</t>
+          <t>unblocks the bulk of the 31 VIU-PENDING (QA) cases (cores, receiving, vendor, validation round-trips).</t>
         </is>
       </c>
       <c r="C23" s="7" t="n"/>

</xml_diff>

<commit_message>
Simple Flow: finalize wording+VIU pass — regenerate deliverables + PROJECT-STATE
All 18 areas / 163 cases wording-corrected + VIU'd + pushed to TestRail (200/200,
0 errors). Regenerated Blockers Tracker, Results workbook, and interim TestRail
import (VIU-word-free, feature-flag-free; 162/163 C-IDs mapped, SF-QB-09 blank).
Final tally: 116 Verified / 35 Pending / 10 Blocked-Env / 1 Deviation / 1
Open-Question. PROJECT-STATE §0-A updated to final.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AZ5XzKsK9wv7M41cSPaMyg
</commit_message>
<xml_diff>
--- a/build/simple-flow/SimpleFlow_Blockers_Tracker.xlsx
+++ b/build/simple-flow/SimpleFlow_Blockers_Tracker.xlsx
@@ -578,7 +578,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Verify the Work Order settings page shows all Simple-Flow toggles in order with new vs existing visually distinct</t>
+          <t>Verify the Work Orders settings tab lists all Work Order setting toggles in order</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -684,12 +684,12 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Verify a 'Create Purchase Orders' toggle exists and, when off, hides the Vendor Invoice sub-setting</t>
+          <t>Verify a 'Create Purchase Orders' toggle exists on the Work Orders tab and controls the Vendor Invoice setting</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Open-Question</t>
+          <t>Deviation</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
@@ -954,7 +954,7 @@
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>VIU-Pending</t>
+          <t>Blocked-Env</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
@@ -1043,57 +1043,61 @@
       <c r="K10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>SF-SET-10</t>
         </is>
       </c>
-      <c r="B11" s="2" t="inlineStr">
+      <c r="B11" s="4" t="inlineStr">
         <is>
           <t>Work Order Settings</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
+      <c r="C11" s="4" t="inlineStr">
         <is>
           <t>Verify a settings change applies to future completions only and not to already-completed work orders</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>VIU-Verified</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>READY</t>
-        </is>
-      </c>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t>READY (VIU-Verified)</t>
-        </is>
-      </c>
-      <c r="G11" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H11" s="2" t="inlineStr">
-        <is>
-          <t>None — VIU-verified; uploadable now.</t>
-        </is>
-      </c>
-      <c r="I11" s="2" t="inlineStr">
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>VIU-Pending</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>VIU PENDING (QA)</t>
+        </is>
+      </c>
+      <c r="G11" s="4" t="inlineStr">
+        <is>
+          <t>QA (needs cookies+seed data)</t>
+        </is>
+      </c>
+      <c r="H11" s="4" t="inlineStr">
+        <is>
+          <t>QA VIU: toggle the setting and confirm the downstream behaviour.</t>
+        </is>
+      </c>
+      <c r="I11" s="4" t="inlineStr">
         <is>
           <t>S1-R9 (future completions only, never retroactive)</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K11" s="2" t="inlineStr"/>
+          <t>reachable-now</t>
+        </is>
+      </c>
+      <c r="K11" s="4" t="inlineStr">
+        <is>
+          <t>admin+tech + normal WO data; needs another VIU pass (no new inputs).</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1219,7 +1223,7 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>VIU-Pending</t>
+          <t>VIU-Verified</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
@@ -1643,7 +1647,7 @@
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>Open-Question</t>
+          <t>Blocked-Env</t>
         </is>
       </c>
       <c r="E22" s="3" t="inlineStr">
@@ -2156,61 +2160,57 @@
       <c r="K31" s="2" t="inlineStr"/>
     </row>
     <row r="32">
-      <c r="A32" s="4" t="inlineStr">
+      <c r="A32" s="2" t="inlineStr">
         <is>
           <t>SF-COMP-16</t>
         </is>
       </c>
-      <c r="B32" s="4" t="inlineStr">
+      <c r="B32" s="2" t="inlineStr">
         <is>
           <t>Completion — PO + Optional Invoice (Story 3)</t>
         </is>
       </c>
-      <c r="C32" s="4" t="inlineStr">
-        <is>
-          <t>Verify the optional-invoice completion modal collects the required vehicle fields (mileage and engine hours; VIN only when Require Review is off) when missing</t>
-        </is>
-      </c>
-      <c r="D32" s="4" t="inlineStr">
-        <is>
-          <t>Pending / Retest — expected changed by V2.4 Δ (2026-07-13), needs live re-VIU</t>
-        </is>
-      </c>
-      <c r="E32" s="4" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
-        </is>
-      </c>
-      <c r="F32" s="4" t="inlineStr">
-        <is>
-          <t>VIU PENDING (QA)</t>
-        </is>
-      </c>
-      <c r="G32" s="4" t="inlineStr">
-        <is>
-          <t>QA (needs cookies+seed data)</t>
-        </is>
-      </c>
-      <c r="H32" s="4" t="inlineStr">
-        <is>
-          <t>QA VIU: seed the specific completion configuration and drive the wizard to Success.</t>
-        </is>
-      </c>
-      <c r="I32" s="4" t="inlineStr">
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Verify the completion modal collects the missing required vehicle fields (Mileage and Engine Hours; no VIN field in the modal)</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>VIU-Verified</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>READY (VIU-Verified)</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>None — VIU-verified; uploadable now.</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="inlineStr">
         <is>
           <t>S3-R3</t>
         </is>
       </c>
       <c r="J32" s="2" t="inlineStr">
         <is>
-          <t>reachable-now</t>
-        </is>
-      </c>
-      <c r="K32" s="4" t="inlineStr">
-        <is>
-          <t>admin+tech + normal WO data; needs another VIU pass (no new inputs).</t>
-        </is>
-      </c>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K32" s="2" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -2442,7 +2442,7 @@
       </c>
       <c r="D37" s="4" t="inlineStr">
         <is>
-          <t>Pending / Retest — expected changed by V2.4 Δ (2026-07-13), needs live re-VIU</t>
+          <t>VIU-Pending</t>
         </is>
       </c>
       <c r="E37" s="4" t="inlineStr">
@@ -2499,7 +2499,7 @@
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>Pending / Retest — expected changed by V2.4 Δ (2026-07-13), needs live re-VIU</t>
+          <t>VIU-Pending</t>
         </is>
       </c>
       <c r="E38" s="4" t="inlineStr">
@@ -2645,61 +2645,57 @@
       <c r="K40" s="2" t="inlineStr"/>
     </row>
     <row r="41">
-      <c r="A41" s="4" t="inlineStr">
+      <c r="A41" s="2" t="inlineStr">
         <is>
           <t>SF-CORE-02</t>
         </is>
       </c>
-      <c r="B41" s="4" t="inlineStr">
+      <c r="B41" s="2" t="inlineStr">
         <is>
           <t>Core parts — Completion modal</t>
         </is>
       </c>
-      <c r="C41" s="4" t="inlineStr">
+      <c r="C41" s="2" t="inlineStr">
         <is>
           <t>Verify a work order with no cores completes with no core sub-lines and no Resolve-Cores wizard step</t>
         </is>
       </c>
-      <c r="D41" s="4" t="inlineStr">
-        <is>
-          <t>VIU-Pending</t>
-        </is>
-      </c>
-      <c r="E41" s="4" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
-        </is>
-      </c>
-      <c r="F41" s="4" t="inlineStr">
-        <is>
-          <t>VIU PENDING (QA)</t>
-        </is>
-      </c>
-      <c r="G41" s="4" t="inlineStr">
-        <is>
-          <t>QA (needs cookies+seed data)</t>
-        </is>
-      </c>
-      <c r="H41" s="4" t="inlineStr">
-        <is>
-          <t>QA VIU: seed a WO with core-charge parts, drive the completion Resolve-Cores modal + invoice-gate round-trip.</t>
-        </is>
-      </c>
-      <c r="I41" s="4" t="inlineStr">
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>VIU-Verified</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>READY (VIU-Verified)</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H41" s="2" t="inlineStr">
+        <is>
+          <t>None — VIU-verified; uploadable now.</t>
+        </is>
+      </c>
+      <c r="I41" s="2" t="inlineStr">
         <is>
           <t>S3-C1 (skipped if none)</t>
         </is>
       </c>
-      <c r="J41" s="4" t="inlineStr">
-        <is>
-          <t>needs-data</t>
-        </is>
-      </c>
-      <c r="K41" s="4" t="inlineStr">
-        <is>
-          <t>a genuine core part to prove the Resolve-Cores step appears, plus a no-core WO to prove it is skipped (is_core not seedable via canned/sub-form).</t>
-        </is>
-      </c>
+      <c r="J41" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K41" s="2" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
@@ -3484,7 +3480,7 @@
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>Verify the tech-story textarea exposes the test id input_tech_story</t>
+          <t>Verify the tech-story modal has a text box for typing the story</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
@@ -4072,7 +4068,7 @@
       </c>
       <c r="D67" s="4" t="inlineStr">
         <is>
-          <t>VIU-Pending</t>
+          <t>Blocked-Env</t>
         </is>
       </c>
       <c r="E67" s="4" t="inlineStr">
@@ -4658,7 +4654,7 @@
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>Verify the Bulk Receive page has a 'Back to Purchase Orders' link that returns to the PO list</t>
+          <t>Verify the Bulk Receive page has a 'Back To Purchase Orders' link that returns to the PO list</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
@@ -5029,7 +5025,7 @@
       </c>
       <c r="C85" s="2" t="inlineStr">
         <is>
-          <t>Verify Receive all receives everything selected at once and supports partial receive</t>
+          <t>Verify Receive All receives everything selected at once and supports partial receive</t>
         </is>
       </c>
       <c r="D85" s="2" t="inlineStr">
@@ -5192,7 +5188,7 @@
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>Verify each vendor group has an 'Apply invoice to selected POs' control enabled only with an invoice # and ≥1 PO selected</t>
+          <t>Verify each vendor group has an 'Apply to selected POs' control enabled only with an invoice # and ≥1 PO selected</t>
         </is>
       </c>
       <c r="D88" s="2" t="inlineStr">
@@ -5580,7 +5576,7 @@
       </c>
       <c r="D95" s="4" t="inlineStr">
         <is>
-          <t>Pending / Retest — expected changed by V2.4 Δ (2026-07-13), needs live re-VIU</t>
+          <t>VIU-Pending</t>
         </is>
       </c>
       <c r="E95" s="4" t="inlineStr">
@@ -5959,7 +5955,7 @@
       </c>
       <c r="D102" s="4" t="inlineStr">
         <is>
-          <t>Pending / Retest — expected changed by V2.4 Δ (2026-07-13), needs live re-VIU</t>
+          <t>VIU-Pending</t>
         </is>
       </c>
       <c r="E102" s="4" t="inlineStr">
@@ -6069,7 +6065,7 @@
       </c>
       <c r="D104" s="4" t="inlineStr">
         <is>
-          <t>VIU-Pending</t>
+          <t>Blocked-Env</t>
         </is>
       </c>
       <c r="E104" s="4" t="inlineStr">
@@ -6399,7 +6395,7 @@
       </c>
       <c r="D110" s="4" t="inlineStr">
         <is>
-          <t>Pending / Retest — expected changed by V2.4 Δ (2026-07-13), needs live re-VIU</t>
+          <t>VIU-Pending</t>
         </is>
       </c>
       <c r="E110" s="4" t="inlineStr">
@@ -6513,7 +6509,7 @@
       </c>
       <c r="D112" s="4" t="inlineStr">
         <is>
-          <t>Pending / Retest — new case for V2.4 Δ3 (2026-07-13), needs live re-VIU</t>
+          <t>VIU-Pending</t>
         </is>
       </c>
       <c r="E112" s="4" t="inlineStr">
@@ -7475,7 +7471,7 @@
       </c>
       <c r="D130" s="3" t="inlineStr">
         <is>
-          <t>Open-Question</t>
+          <t>Blocked-Env</t>
         </is>
       </c>
       <c r="E130" s="3" t="inlineStr">
@@ -8323,7 +8319,7 @@
       </c>
       <c r="D146" s="4" t="inlineStr">
         <is>
-          <t>Pending / Retest — expected changed by V2.4 Δ (2026-07-13), needs live re-VIU</t>
+          <t>VIU-Pending</t>
         </is>
       </c>
       <c r="E146" s="4" t="inlineStr">
@@ -8539,7 +8535,7 @@
       </c>
       <c r="D150" s="4" t="inlineStr">
         <is>
-          <t>Pending / Retest — expected changed by V2.4 Δ (2026-07-13), needs live re-VIU</t>
+          <t>VIU-Pending</t>
         </is>
       </c>
       <c r="E150" s="4" t="inlineStr">
@@ -8812,7 +8808,7 @@
       </c>
       <c r="D155" s="4" t="inlineStr">
         <is>
-          <t>Pending / Retest — expected changed by V2.4 Δ (2026-07-13), needs live re-VIU</t>
+          <t>VIU-Pending</t>
         </is>
       </c>
       <c r="E155" s="4" t="inlineStr">
@@ -8926,7 +8922,7 @@
       </c>
       <c r="D157" s="3" t="inlineStr">
         <is>
-          <t>Open-Question</t>
+          <t>Blocked-Env</t>
         </is>
       </c>
       <c r="E157" s="3" t="inlineStr">
@@ -8979,7 +8975,7 @@
       </c>
       <c r="D158" s="4" t="inlineStr">
         <is>
-          <t>VIU-Pending</t>
+          <t>Blocked-Env</t>
         </is>
       </c>
       <c r="E158" s="4" t="inlineStr">
@@ -9093,7 +9089,7 @@
       </c>
       <c r="D160" s="4" t="inlineStr">
         <is>
-          <t>VIU-Pending</t>
+          <t>Blocked-Env</t>
         </is>
       </c>
       <c r="E160" s="4" t="inlineStr">
@@ -9150,7 +9146,7 @@
       </c>
       <c r="D161" s="4" t="inlineStr">
         <is>
-          <t>VIU-Pending</t>
+          <t>Blocked-Env</t>
         </is>
       </c>
       <c r="E161" s="4" t="inlineStr">
@@ -9207,7 +9203,7 @@
       </c>
       <c r="D162" s="4" t="inlineStr">
         <is>
-          <t>VIU-Pending</t>
+          <t>Blocked-Env</t>
         </is>
       </c>
       <c r="E162" s="4" t="inlineStr">
@@ -9433,7 +9429,7 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
@@ -9463,7 +9459,7 @@
         </is>
       </c>
       <c r="B8" s="4" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
@@ -9574,7 +9570,7 @@
         </is>
       </c>
       <c r="B17" s="4" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
@@ -9604,7 +9600,7 @@
         </is>
       </c>
       <c r="B19" s="10" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C19" s="6" t="inlineStr"/>
     </row>
@@ -9643,7 +9639,7 @@
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>unblocks the bulk of the 39 VIU-PENDING (QA) cases (cores, receiving, vendor, validation round-trips).</t>
+          <t>unblocks the bulk of the 38 VIU-PENDING (QA) cases (cores, receiving, vendor, validation round-trips).</t>
         </is>
       </c>
       <c r="C23" s="6" t="n"/>

</xml_diff>

<commit_message>
Simple Flow: add TestRail ID + Link columns to Blockers Tracker (Standing Rule 8)
gen_blockers.py now loads testrail-id-map.csv and appends TestRail ID (C#####) +
clickable TestRail Link as the last two columns (XLSX + MD). Regenerated tracker.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AZ5XzKsK9wv7M41cSPaMyg
</commit_message>
<xml_diff>
--- a/build/simple-flow/SimpleFlow_Blockers_Tracker.xlsx
+++ b/build/simple-flow/SimpleFlow_Blockers_Tracker.xlsx
@@ -492,7 +492,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K164"/>
+  <dimension ref="A1:M164"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -506,6 +506,8 @@
     <col width="34" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
     <col width="65" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -564,6 +566,16 @@
           <t>VIU sub-bucket detail (QA-pending only)</t>
         </is>
       </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>TestRail ID</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>TestRail Link</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -617,6 +629,16 @@
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr"/>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>C29275</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29275</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -670,6 +692,16 @@
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr"/>
+      <c r="L3" s="2" t="inlineStr">
+        <is>
+          <t>C29276</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29276</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -723,6 +755,16 @@
         </is>
       </c>
       <c r="K4" s="3" t="inlineStr"/>
+      <c r="L4" s="3" t="inlineStr">
+        <is>
+          <t>C29277</t>
+        </is>
+      </c>
+      <c r="M4" s="3" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29277</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -776,6 +818,16 @@
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr"/>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>C29278</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29278</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -829,6 +881,16 @@
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr"/>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>C29279</t>
+        </is>
+      </c>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29279</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -882,6 +944,16 @@
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr"/>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>C29280</t>
+        </is>
+      </c>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29280</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -935,6 +1007,16 @@
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr"/>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>C29281</t>
+        </is>
+      </c>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29281</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -988,6 +1070,16 @@
         </is>
       </c>
       <c r="K9" s="3" t="inlineStr"/>
+      <c r="L9" s="3" t="inlineStr">
+        <is>
+          <t>C29282</t>
+        </is>
+      </c>
+      <c r="M9" s="3" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29282</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1041,6 +1133,16 @@
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr"/>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>C29283</t>
+        </is>
+      </c>
+      <c r="M10" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29283</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
@@ -1098,6 +1200,16 @@
           <t>admin+tech + normal WO data; needs another VIU pass (no new inputs).</t>
         </is>
       </c>
+      <c r="L11" s="4" t="inlineStr">
+        <is>
+          <t>C29284</t>
+        </is>
+      </c>
+      <c r="M11" s="4" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29284</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1151,6 +1263,16 @@
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr"/>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>C29285</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29285</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1204,6 +1326,16 @@
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr"/>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>C29286</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29286</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -1257,6 +1389,16 @@
         </is>
       </c>
       <c r="K14" s="3" t="inlineStr"/>
+      <c r="L14" s="3" t="inlineStr">
+        <is>
+          <t>C29287</t>
+        </is>
+      </c>
+      <c r="M14" s="3" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29287</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1310,6 +1452,16 @@
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr"/>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>C29288</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29288</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1363,6 +1515,16 @@
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr"/>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>C29289</t>
+        </is>
+      </c>
+      <c r="M16" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29289</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1416,6 +1578,16 @@
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr"/>
+      <c r="L17" s="2" t="inlineStr">
+        <is>
+          <t>C29290</t>
+        </is>
+      </c>
+      <c r="M17" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29290</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1469,6 +1641,16 @@
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr"/>
+      <c r="L18" s="2" t="inlineStr">
+        <is>
+          <t>C29291</t>
+        </is>
+      </c>
+      <c r="M18" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29291</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1522,6 +1704,16 @@
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr"/>
+      <c r="L19" s="2" t="inlineStr">
+        <is>
+          <t>C29292</t>
+        </is>
+      </c>
+      <c r="M19" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29292</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1575,6 +1767,16 @@
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr"/>
+      <c r="L20" s="2" t="inlineStr">
+        <is>
+          <t>C29293</t>
+        </is>
+      </c>
+      <c r="M20" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29293</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -1628,6 +1830,16 @@
         </is>
       </c>
       <c r="K21" s="2" t="inlineStr"/>
+      <c r="L21" s="2" t="inlineStr">
+        <is>
+          <t>C29294</t>
+        </is>
+      </c>
+      <c r="M21" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29294</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
@@ -1681,6 +1893,16 @@
         </is>
       </c>
       <c r="K22" s="3" t="inlineStr"/>
+      <c r="L22" s="3" t="inlineStr">
+        <is>
+          <t>C29295</t>
+        </is>
+      </c>
+      <c r="M22" s="3" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29295</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -1734,6 +1956,16 @@
         </is>
       </c>
       <c r="K23" s="2" t="inlineStr"/>
+      <c r="L23" s="2" t="inlineStr">
+        <is>
+          <t>C29296</t>
+        </is>
+      </c>
+      <c r="M23" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29296</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -1787,6 +2019,16 @@
         </is>
       </c>
       <c r="K24" s="2" t="inlineStr"/>
+      <c r="L24" s="2" t="inlineStr">
+        <is>
+          <t>C29297</t>
+        </is>
+      </c>
+      <c r="M24" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29297</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -1840,6 +2082,16 @@
         </is>
       </c>
       <c r="K25" s="2" t="inlineStr"/>
+      <c r="L25" s="2" t="inlineStr">
+        <is>
+          <t>C29298</t>
+        </is>
+      </c>
+      <c r="M25" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29298</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -1893,6 +2145,16 @@
         </is>
       </c>
       <c r="K26" s="2" t="inlineStr"/>
+      <c r="L26" s="2" t="inlineStr">
+        <is>
+          <t>C29299</t>
+        </is>
+      </c>
+      <c r="M26" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29299</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -1946,6 +2208,16 @@
         </is>
       </c>
       <c r="K27" s="2" t="inlineStr"/>
+      <c r="L27" s="2" t="inlineStr">
+        <is>
+          <t>C29300</t>
+        </is>
+      </c>
+      <c r="M27" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29300</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -1999,6 +2271,16 @@
         </is>
       </c>
       <c r="K28" s="2" t="inlineStr"/>
+      <c r="L28" s="2" t="inlineStr">
+        <is>
+          <t>C29301</t>
+        </is>
+      </c>
+      <c r="M28" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29301</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -2052,6 +2334,16 @@
         </is>
       </c>
       <c r="K29" s="2" t="inlineStr"/>
+      <c r="L29" s="2" t="inlineStr">
+        <is>
+          <t>C29302</t>
+        </is>
+      </c>
+      <c r="M29" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29302</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -2105,6 +2397,16 @@
         </is>
       </c>
       <c r="K30" s="2" t="inlineStr"/>
+      <c r="L30" s="2" t="inlineStr">
+        <is>
+          <t>C29303</t>
+        </is>
+      </c>
+      <c r="M30" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29303</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -2158,6 +2460,16 @@
         </is>
       </c>
       <c r="K31" s="2" t="inlineStr"/>
+      <c r="L31" s="2" t="inlineStr">
+        <is>
+          <t>C29304</t>
+        </is>
+      </c>
+      <c r="M31" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29304</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -2211,6 +2523,16 @@
         </is>
       </c>
       <c r="K32" s="2" t="inlineStr"/>
+      <c r="L32" s="2" t="inlineStr">
+        <is>
+          <t>C29305</t>
+        </is>
+      </c>
+      <c r="M32" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29305</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -2264,6 +2586,16 @@
         </is>
       </c>
       <c r="K33" s="2" t="inlineStr"/>
+      <c r="L33" s="2" t="inlineStr">
+        <is>
+          <t>C29306</t>
+        </is>
+      </c>
+      <c r="M33" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29306</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -2317,6 +2649,16 @@
         </is>
       </c>
       <c r="K34" s="2" t="inlineStr"/>
+      <c r="L34" s="2" t="inlineStr">
+        <is>
+          <t>C29307</t>
+        </is>
+      </c>
+      <c r="M34" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29307</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -2370,6 +2712,16 @@
         </is>
       </c>
       <c r="K35" s="2" t="inlineStr"/>
+      <c r="L35" s="2" t="inlineStr">
+        <is>
+          <t>C29308</t>
+        </is>
+      </c>
+      <c r="M35" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29308</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -2423,6 +2775,16 @@
         </is>
       </c>
       <c r="K36" s="2" t="inlineStr"/>
+      <c r="L36" s="2" t="inlineStr">
+        <is>
+          <t>C29309</t>
+        </is>
+      </c>
+      <c r="M36" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29309</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
@@ -2480,6 +2842,16 @@
           <t>admin+tech + normal WO data; needs another VIU pass (no new inputs).</t>
         </is>
       </c>
+      <c r="L37" s="4" t="inlineStr">
+        <is>
+          <t>C29310</t>
+        </is>
+      </c>
+      <c r="M37" s="4" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29310</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
@@ -2537,6 +2909,16 @@
           <t>admin+tech + normal WO data; needs another VIU pass (no new inputs).</t>
         </is>
       </c>
+      <c r="L38" s="4" t="inlineStr">
+        <is>
+          <t>C29311</t>
+        </is>
+      </c>
+      <c r="M38" s="4" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29311</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -2590,6 +2972,16 @@
         </is>
       </c>
       <c r="K39" s="2" t="inlineStr"/>
+      <c r="L39" s="2" t="inlineStr">
+        <is>
+          <t>C29312</t>
+        </is>
+      </c>
+      <c r="M39" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29312</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -2643,6 +3035,16 @@
         </is>
       </c>
       <c r="K40" s="2" t="inlineStr"/>
+      <c r="L40" s="2" t="inlineStr">
+        <is>
+          <t>C29313</t>
+        </is>
+      </c>
+      <c r="M40" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29313</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -2696,6 +3098,16 @@
         </is>
       </c>
       <c r="K41" s="2" t="inlineStr"/>
+      <c r="L41" s="2" t="inlineStr">
+        <is>
+          <t>C29314</t>
+        </is>
+      </c>
+      <c r="M41" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29314</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
@@ -2753,6 +3165,16 @@
           <t>a special-order core part + optional-invoice completion (needs is_core part).</t>
         </is>
       </c>
+      <c r="L42" s="4" t="inlineStr">
+        <is>
+          <t>C29315</t>
+        </is>
+      </c>
+      <c r="M42" s="4" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29315</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
@@ -2810,6 +3232,16 @@
           <t>an unresolved special-order core at the invoice gate ('Cores pending' flag) — needs is_core part + receiving.</t>
         </is>
       </c>
+      <c r="L43" s="4" t="inlineStr">
+        <is>
+          <t>C29316</t>
+        </is>
+      </c>
+      <c r="M43" s="4" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29316</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
@@ -2867,6 +3299,16 @@
           <t>resolve cores at the Create-Invoice gate -&gt; receive the cored line (needs is_core part + receiving).</t>
         </is>
       </c>
+      <c r="L44" s="4" t="inlineStr">
+        <is>
+          <t>C29317</t>
+        </is>
+      </c>
+      <c r="M44" s="4" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29317</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="4" t="inlineStr">
@@ -2924,6 +3366,16 @@
           <t>cancel the invoice-gate core resolution (needs is_core part + invoice gate).</t>
         </is>
       </c>
+      <c r="L45" s="4" t="inlineStr">
+        <is>
+          <t>C29318</t>
+        </is>
+      </c>
+      <c r="M45" s="4" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29318</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="4" t="inlineStr">
@@ -2981,6 +3433,16 @@
           <t>special-order cores in the required-invoice receive round-trip (needs is_core part + receiving).</t>
         </is>
       </c>
+      <c r="L46" s="4" t="inlineStr">
+        <is>
+          <t>C29319</t>
+        </is>
+      </c>
+      <c r="M46" s="4" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29319</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="4" t="inlineStr">
@@ -3038,6 +3500,16 @@
           <t>an unresolved special-order core that exists only as a PartRequest (needs is_core part).</t>
         </is>
       </c>
+      <c r="L47" s="4" t="inlineStr">
+        <is>
+          <t>C29320</t>
+        </is>
+      </c>
+      <c r="M47" s="4" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29320</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="4" t="inlineStr">
@@ -3095,6 +3567,16 @@
           <t>a part-sale WO vs service WO with cores (needs is_core part + receiving).</t>
         </is>
       </c>
+      <c r="L48" s="4" t="inlineStr">
+        <is>
+          <t>C29321</t>
+        </is>
+      </c>
+      <c r="M48" s="4" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29321</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -3148,6 +3630,16 @@
         </is>
       </c>
       <c r="K49" s="2" t="inlineStr"/>
+      <c r="L49" s="2" t="inlineStr">
+        <is>
+          <t>C29322</t>
+        </is>
+      </c>
+      <c r="M49" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29322</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -3201,6 +3693,16 @@
         </is>
       </c>
       <c r="K50" s="2" t="inlineStr"/>
+      <c r="L50" s="2" t="inlineStr">
+        <is>
+          <t>C29323</t>
+        </is>
+      </c>
+      <c r="M50" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29323</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -3254,6 +3756,16 @@
         </is>
       </c>
       <c r="K51" s="2" t="inlineStr"/>
+      <c r="L51" s="2" t="inlineStr">
+        <is>
+          <t>C29324</t>
+        </is>
+      </c>
+      <c r="M51" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29324</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -3307,6 +3819,16 @@
         </is>
       </c>
       <c r="K52" s="2" t="inlineStr"/>
+      <c r="L52" s="2" t="inlineStr">
+        <is>
+          <t>C29325</t>
+        </is>
+      </c>
+      <c r="M52" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29325</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -3360,6 +3882,16 @@
         </is>
       </c>
       <c r="K53" s="2" t="inlineStr"/>
+      <c r="L53" s="2" t="inlineStr">
+        <is>
+          <t>C29326</t>
+        </is>
+      </c>
+      <c r="M53" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29326</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -3413,6 +3945,16 @@
         </is>
       </c>
       <c r="K54" s="2" t="inlineStr"/>
+      <c r="L54" s="2" t="inlineStr">
+        <is>
+          <t>C29327</t>
+        </is>
+      </c>
+      <c r="M54" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29327</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -3466,6 +4008,16 @@
         </is>
       </c>
       <c r="K55" s="2" t="inlineStr"/>
+      <c r="L55" s="2" t="inlineStr">
+        <is>
+          <t>C29328</t>
+        </is>
+      </c>
+      <c r="M55" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29328</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -3519,6 +4071,16 @@
         </is>
       </c>
       <c r="K56" s="2" t="inlineStr"/>
+      <c r="L56" s="2" t="inlineStr">
+        <is>
+          <t>C29329</t>
+        </is>
+      </c>
+      <c r="M56" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29329</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="3" t="inlineStr">
@@ -3572,6 +4134,16 @@
         </is>
       </c>
       <c r="K57" s="3" t="inlineStr"/>
+      <c r="L57" s="3" t="inlineStr">
+        <is>
+          <t>C29330</t>
+        </is>
+      </c>
+      <c r="M57" s="3" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29330</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -3625,6 +4197,16 @@
         </is>
       </c>
       <c r="K58" s="2" t="inlineStr"/>
+      <c r="L58" s="2" t="inlineStr">
+        <is>
+          <t>C29331</t>
+        </is>
+      </c>
+      <c r="M58" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29331</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -3678,6 +4260,16 @@
         </is>
       </c>
       <c r="K59" s="2" t="inlineStr"/>
+      <c r="L59" s="2" t="inlineStr">
+        <is>
+          <t>C29332</t>
+        </is>
+      </c>
+      <c r="M59" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29332</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -3731,6 +4323,16 @@
         </is>
       </c>
       <c r="K60" s="2" t="inlineStr"/>
+      <c r="L60" s="2" t="inlineStr">
+        <is>
+          <t>C29333</t>
+        </is>
+      </c>
+      <c r="M60" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29333</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -3784,6 +4386,16 @@
         </is>
       </c>
       <c r="K61" s="2" t="inlineStr"/>
+      <c r="L61" s="2" t="inlineStr">
+        <is>
+          <t>C29334</t>
+        </is>
+      </c>
+      <c r="M61" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29334</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -3837,6 +4449,16 @@
         </is>
       </c>
       <c r="K62" s="2" t="inlineStr"/>
+      <c r="L62" s="2" t="inlineStr">
+        <is>
+          <t>C29335</t>
+        </is>
+      </c>
+      <c r="M62" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29335</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -3890,6 +4512,16 @@
         </is>
       </c>
       <c r="K63" s="2" t="inlineStr"/>
+      <c r="L63" s="2" t="inlineStr">
+        <is>
+          <t>C29336</t>
+        </is>
+      </c>
+      <c r="M63" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29336</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -3943,6 +4575,16 @@
         </is>
       </c>
       <c r="K64" s="2" t="inlineStr"/>
+      <c r="L64" s="2" t="inlineStr">
+        <is>
+          <t>C29337</t>
+        </is>
+      </c>
+      <c r="M64" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29337</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -3996,6 +4638,16 @@
         </is>
       </c>
       <c r="K65" s="2" t="inlineStr"/>
+      <c r="L65" s="2" t="inlineStr">
+        <is>
+          <t>C29338</t>
+        </is>
+      </c>
+      <c r="M65" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29338</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -4049,6 +4701,16 @@
         </is>
       </c>
       <c r="K66" s="2" t="inlineStr"/>
+      <c r="L66" s="2" t="inlineStr">
+        <is>
+          <t>C29339</t>
+        </is>
+      </c>
+      <c r="M66" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29339</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="4" t="inlineStr">
@@ -4106,6 +4768,16 @@
           <t>QuickBooks sync inspection (vendor-missing PO excluded from QB).</t>
         </is>
       </c>
+      <c r="L67" s="4" t="inlineStr">
+        <is>
+          <t>C29340</t>
+        </is>
+      </c>
+      <c r="M67" s="4" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29340</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -4159,6 +4831,16 @@
         </is>
       </c>
       <c r="K68" s="2" t="inlineStr"/>
+      <c r="L68" s="2" t="inlineStr">
+        <is>
+          <t>C29341</t>
+        </is>
+      </c>
+      <c r="M68" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29341</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -4212,6 +4894,16 @@
         </is>
       </c>
       <c r="K69" s="2" t="inlineStr"/>
+      <c r="L69" s="2" t="inlineStr">
+        <is>
+          <t>C29342</t>
+        </is>
+      </c>
+      <c r="M69" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29342</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="4" t="inlineStr">
@@ -4269,6 +4961,16 @@
           <t>reports data (Vendor Missing POs flagged 'needs vendor').</t>
         </is>
       </c>
+      <c r="L70" s="4" t="inlineStr">
+        <is>
+          <t>C29343</t>
+        </is>
+      </c>
+      <c r="M70" s="4" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29343</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -4322,6 +5024,16 @@
         </is>
       </c>
       <c r="K71" s="2" t="inlineStr"/>
+      <c r="L71" s="2" t="inlineStr">
+        <is>
+          <t>C29439</t>
+        </is>
+      </c>
+      <c r="M71" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29439</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -4375,6 +5087,16 @@
         </is>
       </c>
       <c r="K72" s="2" t="inlineStr"/>
+      <c r="L72" s="2" t="inlineStr">
+        <is>
+          <t>C29344</t>
+        </is>
+      </c>
+      <c r="M72" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29344</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -4428,6 +5150,16 @@
         </is>
       </c>
       <c r="K73" s="2" t="inlineStr"/>
+      <c r="L73" s="2" t="inlineStr">
+        <is>
+          <t>C29345</t>
+        </is>
+      </c>
+      <c r="M73" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29345</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -4481,6 +5213,16 @@
         </is>
       </c>
       <c r="K74" s="2" t="inlineStr"/>
+      <c r="L74" s="2" t="inlineStr">
+        <is>
+          <t>C29346</t>
+        </is>
+      </c>
+      <c r="M74" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29346</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -4534,6 +5276,16 @@
         </is>
       </c>
       <c r="K75" s="2" t="inlineStr"/>
+      <c r="L75" s="2" t="inlineStr">
+        <is>
+          <t>C29347</t>
+        </is>
+      </c>
+      <c r="M75" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29347</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -4587,6 +5339,16 @@
         </is>
       </c>
       <c r="K76" s="2" t="inlineStr"/>
+      <c r="L76" s="2" t="inlineStr">
+        <is>
+          <t>C29348</t>
+        </is>
+      </c>
+      <c r="M76" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29348</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -4640,6 +5402,16 @@
         </is>
       </c>
       <c r="K77" s="2" t="inlineStr"/>
+      <c r="L77" s="2" t="inlineStr">
+        <is>
+          <t>C29349</t>
+        </is>
+      </c>
+      <c r="M77" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29349</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -4693,6 +5465,16 @@
         </is>
       </c>
       <c r="K78" s="2" t="inlineStr"/>
+      <c r="L78" s="2" t="inlineStr">
+        <is>
+          <t>C29350</t>
+        </is>
+      </c>
+      <c r="M78" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29350</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -4746,6 +5528,16 @@
         </is>
       </c>
       <c r="K79" s="2" t="inlineStr"/>
+      <c r="L79" s="2" t="inlineStr">
+        <is>
+          <t>C29351</t>
+        </is>
+      </c>
+      <c r="M79" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29351</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -4799,6 +5591,16 @@
         </is>
       </c>
       <c r="K80" s="2" t="inlineStr"/>
+      <c r="L80" s="2" t="inlineStr">
+        <is>
+          <t>C29352</t>
+        </is>
+      </c>
+      <c r="M80" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29352</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -4852,6 +5654,16 @@
         </is>
       </c>
       <c r="K81" s="2" t="inlineStr"/>
+      <c r="L81" s="2" t="inlineStr">
+        <is>
+          <t>C29353</t>
+        </is>
+      </c>
+      <c r="M81" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29353</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -4905,6 +5717,16 @@
         </is>
       </c>
       <c r="K82" s="2" t="inlineStr"/>
+      <c r="L82" s="2" t="inlineStr">
+        <is>
+          <t>C29354</t>
+        </is>
+      </c>
+      <c r="M82" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29354</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -4958,6 +5780,16 @@
         </is>
       </c>
       <c r="K83" s="2" t="inlineStr"/>
+      <c r="L83" s="2" t="inlineStr">
+        <is>
+          <t>C29355</t>
+        </is>
+      </c>
+      <c r="M83" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29355</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -5011,6 +5843,16 @@
         </is>
       </c>
       <c r="K84" s="2" t="inlineStr"/>
+      <c r="L84" s="2" t="inlineStr">
+        <is>
+          <t>C29356</t>
+        </is>
+      </c>
+      <c r="M84" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29356</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -5064,6 +5906,16 @@
         </is>
       </c>
       <c r="K85" s="2" t="inlineStr"/>
+      <c r="L85" s="2" t="inlineStr">
+        <is>
+          <t>C29357</t>
+        </is>
+      </c>
+      <c r="M85" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29357</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -5117,6 +5969,16 @@
         </is>
       </c>
       <c r="K86" s="2" t="inlineStr"/>
+      <c r="L86" s="2" t="inlineStr">
+        <is>
+          <t>C29358</t>
+        </is>
+      </c>
+      <c r="M86" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29358</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="4" t="inlineStr">
@@ -5174,6 +6036,16 @@
           <t>RE-VIU 2026-07-09: Bulk Receive page BUILT; this case needs a genuine cored part received on the bulk page to expose Ok/Not-OK resolution (is_core part not seedable via canned/sub-form).</t>
         </is>
       </c>
+      <c r="L87" s="4" t="inlineStr">
+        <is>
+          <t>C29359</t>
+        </is>
+      </c>
+      <c r="M87" s="4" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29359</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -5227,6 +6099,16 @@
         </is>
       </c>
       <c r="K88" s="2" t="inlineStr"/>
+      <c r="L88" s="2" t="inlineStr">
+        <is>
+          <t>C29360</t>
+        </is>
+      </c>
+      <c r="M88" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29360</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -5280,6 +6162,16 @@
         </is>
       </c>
       <c r="K89" s="2" t="inlineStr"/>
+      <c r="L89" s="2" t="inlineStr">
+        <is>
+          <t>C29361</t>
+        </is>
+      </c>
+      <c r="M89" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29361</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -5333,6 +6225,16 @@
         </is>
       </c>
       <c r="K90" s="2" t="inlineStr"/>
+      <c r="L90" s="2" t="inlineStr">
+        <is>
+          <t>C29362</t>
+        </is>
+      </c>
+      <c r="M90" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29362</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -5386,6 +6288,16 @@
         </is>
       </c>
       <c r="K91" s="2" t="inlineStr"/>
+      <c r="L91" s="2" t="inlineStr">
+        <is>
+          <t>C29363</t>
+        </is>
+      </c>
+      <c r="M91" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29363</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="4" t="inlineStr">
@@ -5443,6 +6355,16 @@
           <t>receiving + inventory/catalog inspection (new PN creates inventory part + stock + Part History on receive).</t>
         </is>
       </c>
+      <c r="L92" s="4" t="inlineStr">
+        <is>
+          <t>C29364</t>
+        </is>
+      </c>
+      <c r="M92" s="4" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29364</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="4" t="inlineStr">
@@ -5500,6 +6422,16 @@
           <t>receiving + inventory inspection (existing PN links to item, updates stock/cost/history).</t>
         </is>
       </c>
+      <c r="L93" s="4" t="inlineStr">
+        <is>
+          <t>C29365</t>
+        </is>
+      </c>
+      <c r="M93" s="4" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29365</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="4" t="inlineStr">
@@ -5557,6 +6489,16 @@
           <t>a WO in invoiced/paid state (sell-field locking).</t>
         </is>
       </c>
+      <c r="L94" s="4" t="inlineStr">
+        <is>
+          <t>C29366</t>
+        </is>
+      </c>
+      <c r="M94" s="4" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29366</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="4" t="inlineStr">
@@ -5614,6 +6556,16 @@
           <t>an invoiced/paid WO + a receive attempt (cannot receive without PN).</t>
         </is>
       </c>
+      <c r="L95" s="4" t="inlineStr">
+        <is>
+          <t>C29367</t>
+        </is>
+      </c>
+      <c r="M95" s="4" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29367</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="4" t="inlineStr">
@@ -5671,6 +6623,16 @@
           <t>receiving + catalog/inventory back-end inspection (real creation/linking, not a stored string).</t>
         </is>
       </c>
+      <c r="L96" s="4" t="inlineStr">
+        <is>
+          <t>C29368</t>
+        </is>
+      </c>
+      <c r="M96" s="4" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29368</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -5724,6 +6686,16 @@
         </is>
       </c>
       <c r="K97" s="2" t="inlineStr"/>
+      <c r="L97" s="2" t="inlineStr">
+        <is>
+          <t>C29369</t>
+        </is>
+      </c>
+      <c r="M97" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29369</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -5777,6 +6749,16 @@
         </is>
       </c>
       <c r="K98" s="2" t="inlineStr"/>
+      <c r="L98" s="2" t="inlineStr">
+        <is>
+          <t>C29370</t>
+        </is>
+      </c>
+      <c r="M98" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29370</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -5830,6 +6812,16 @@
         </is>
       </c>
       <c r="K99" s="2" t="inlineStr"/>
+      <c r="L99" s="2" t="inlineStr">
+        <is>
+          <t>C29371</t>
+        </is>
+      </c>
+      <c r="M99" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29371</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -5883,6 +6875,16 @@
         </is>
       </c>
       <c r="K100" s="2" t="inlineStr"/>
+      <c r="L100" s="2" t="inlineStr">
+        <is>
+          <t>C29372</t>
+        </is>
+      </c>
+      <c r="M100" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29372</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="3" t="inlineStr">
@@ -5936,6 +6938,16 @@
         </is>
       </c>
       <c r="K101" s="3" t="inlineStr"/>
+      <c r="L101" s="3" t="inlineStr">
+        <is>
+          <t>C29373</t>
+        </is>
+      </c>
+      <c r="M101" s="3" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29373</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="4" t="inlineStr">
@@ -5993,6 +7005,16 @@
           <t>BATCH 6: on a deliverable WO PO the Accept Delivery gates are present (vendor set, invoice # field), but Receive 500s (BUG-11); on a vendor-missing WO PO there is no assign-vendor / PN-edit control. Happy path was proven on an INVENTORY PO in BATCH 5; the WO-PO negative sub-gates need BUG-11 fixed.</t>
         </is>
       </c>
+      <c r="L102" s="4" t="inlineStr">
+        <is>
+          <t>C29374</t>
+        </is>
+      </c>
+      <c r="M102" s="4" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29374</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="3" t="inlineStr">
@@ -6046,6 +7068,16 @@
         </is>
       </c>
       <c r="K103" s="3" t="inlineStr"/>
+      <c r="L103" s="3" t="inlineStr">
+        <is>
+          <t>C29375</t>
+        </is>
+      </c>
+      <c r="M103" s="3" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29375</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="4" t="inlineStr">
@@ -6103,6 +7135,16 @@
           <t>QuickBooks inspection (per-vendor vendor bill + separate AP entry) — and WO-PO receive additionally blocked by BUG-11 (500).</t>
         </is>
       </c>
+      <c r="L104" s="4" t="inlineStr">
+        <is>
+          <t>C29376</t>
+        </is>
+      </c>
+      <c r="M104" s="4" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29376</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -6156,6 +7198,16 @@
         </is>
       </c>
       <c r="K105" s="2" t="inlineStr"/>
+      <c r="L105" s="2" t="inlineStr">
+        <is>
+          <t>C29377</t>
+        </is>
+      </c>
+      <c r="M105" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29377</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -6209,6 +7261,16 @@
         </is>
       </c>
       <c r="K106" s="2" t="inlineStr"/>
+      <c r="L106" s="2" t="inlineStr">
+        <is>
+          <t>C29440</t>
+        </is>
+      </c>
+      <c r="M106" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29440</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -6262,6 +7324,16 @@
         </is>
       </c>
       <c r="K107" s="2" t="inlineStr"/>
+      <c r="L107" s="2" t="inlineStr">
+        <is>
+          <t>C29378</t>
+        </is>
+      </c>
+      <c r="M107" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29378</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="4" t="inlineStr">
@@ -6319,6 +7391,16 @@
           <t>a PO where the assigned vendor already exists on the PO (Add-to-vendor merge vs keep-separate prompt).</t>
         </is>
       </c>
+      <c r="L108" s="4" t="inlineStr">
+        <is>
+          <t>C29379</t>
+        </is>
+      </c>
+      <c r="M108" s="4" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29379</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="4" t="inlineStr">
@@ -6376,6 +7458,16 @@
           <t>two POs for the same WO with the same vendor (merge-POs prompt).</t>
         </is>
       </c>
+      <c r="L109" s="4" t="inlineStr">
+        <is>
+          <t>C29380</t>
+        </is>
+      </c>
+      <c r="M109" s="4" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29380</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="4" t="inlineStr">
@@ -6433,6 +7525,16 @@
           <t>a vendor-missing PO + receive-enable + QB-flag-clear check after auto-assign.</t>
         </is>
       </c>
+      <c r="L110" s="4" t="inlineStr">
+        <is>
+          <t>C29381</t>
+        </is>
+      </c>
+      <c r="M110" s="4" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29381</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="4" t="inlineStr">
@@ -6490,6 +7592,16 @@
           <t>invoiced/paid WO + multi-PO merge guardrail state (match-by-ID, merge scoped to same WO, receive blocked when invoiced/paid).</t>
         </is>
       </c>
+      <c r="L111" s="4" t="inlineStr">
+        <is>
+          <t>C29382</t>
+        </is>
+      </c>
+      <c r="M111" s="4" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29382</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="4" t="inlineStr">
@@ -6547,6 +7659,16 @@
           <t>admin+tech + normal WO data; needs another VIU pass (no new inputs).</t>
         </is>
       </c>
+      <c r="L112" s="4" t="inlineStr">
+        <is>
+          <t>C29442</t>
+        </is>
+      </c>
+      <c r="M112" s="4" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29442</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -6600,6 +7722,16 @@
         </is>
       </c>
       <c r="K113" s="2" t="inlineStr"/>
+      <c r="L113" s="2" t="inlineStr">
+        <is>
+          <t>C29383</t>
+        </is>
+      </c>
+      <c r="M113" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29383</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -6653,6 +7785,16 @@
         </is>
       </c>
       <c r="K114" s="2" t="inlineStr"/>
+      <c r="L114" s="2" t="inlineStr">
+        <is>
+          <t>C29384</t>
+        </is>
+      </c>
+      <c r="M114" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29384</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -6706,6 +7848,16 @@
         </is>
       </c>
       <c r="K115" s="2" t="inlineStr"/>
+      <c r="L115" s="2" t="inlineStr">
+        <is>
+          <t>C29385</t>
+        </is>
+      </c>
+      <c r="M115" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29385</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -6759,6 +7911,16 @@
         </is>
       </c>
       <c r="K116" s="2" t="inlineStr"/>
+      <c r="L116" s="2" t="inlineStr">
+        <is>
+          <t>C29386</t>
+        </is>
+      </c>
+      <c r="M116" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29386</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -6812,6 +7974,16 @@
         </is>
       </c>
       <c r="K117" s="2" t="inlineStr"/>
+      <c r="L117" s="2" t="inlineStr">
+        <is>
+          <t>C29387</t>
+        </is>
+      </c>
+      <c r="M117" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29387</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -6865,6 +8037,16 @@
         </is>
       </c>
       <c r="K118" s="2" t="inlineStr"/>
+      <c r="L118" s="2" t="inlineStr">
+        <is>
+          <t>C29388</t>
+        </is>
+      </c>
+      <c r="M118" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29388</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -6918,6 +8100,16 @@
         </is>
       </c>
       <c r="K119" s="2" t="inlineStr"/>
+      <c r="L119" s="2" t="inlineStr">
+        <is>
+          <t>C29389</t>
+        </is>
+      </c>
+      <c r="M119" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29389</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -6971,6 +8163,16 @@
         </is>
       </c>
       <c r="K120" s="2" t="inlineStr"/>
+      <c r="L120" s="2" t="inlineStr">
+        <is>
+          <t>C29390</t>
+        </is>
+      </c>
+      <c r="M120" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29390</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -7024,6 +8226,16 @@
         </is>
       </c>
       <c r="K121" s="2" t="inlineStr"/>
+      <c r="L121" s="2" t="inlineStr">
+        <is>
+          <t>C29391</t>
+        </is>
+      </c>
+      <c r="M121" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29391</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -7077,6 +8289,16 @@
         </is>
       </c>
       <c r="K122" s="2" t="inlineStr"/>
+      <c r="L122" s="2" t="inlineStr">
+        <is>
+          <t>C29392</t>
+        </is>
+      </c>
+      <c r="M122" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29392</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="3" t="inlineStr">
@@ -7130,6 +8352,16 @@
         </is>
       </c>
       <c r="K123" s="3" t="inlineStr"/>
+      <c r="L123" s="3" t="inlineStr">
+        <is>
+          <t>C29393</t>
+        </is>
+      </c>
+      <c r="M123" s="3" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29393</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -7183,6 +8415,16 @@
         </is>
       </c>
       <c r="K124" s="2" t="inlineStr"/>
+      <c r="L124" s="2" t="inlineStr">
+        <is>
+          <t>C29394</t>
+        </is>
+      </c>
+      <c r="M124" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29394</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="3" t="inlineStr">
@@ -7236,6 +8478,16 @@
         </is>
       </c>
       <c r="K125" s="3" t="inlineStr"/>
+      <c r="L125" s="3" t="inlineStr">
+        <is>
+          <t>C29395</t>
+        </is>
+      </c>
+      <c r="M125" s="3" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29395</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="3" t="inlineStr">
@@ -7289,6 +8541,16 @@
         </is>
       </c>
       <c r="K126" s="3" t="inlineStr"/>
+      <c r="L126" s="3" t="inlineStr">
+        <is>
+          <t>C29396</t>
+        </is>
+      </c>
+      <c r="M126" s="3" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29396</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -7342,6 +8604,16 @@
         </is>
       </c>
       <c r="K127" s="2" t="inlineStr"/>
+      <c r="L127" s="2" t="inlineStr">
+        <is>
+          <t>C29397</t>
+        </is>
+      </c>
+      <c r="M127" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29397</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -7395,6 +8667,16 @@
         </is>
       </c>
       <c r="K128" s="2" t="inlineStr"/>
+      <c r="L128" s="2" t="inlineStr">
+        <is>
+          <t>C29398</t>
+        </is>
+      </c>
+      <c r="M128" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29398</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="4" t="inlineStr">
@@ -7452,6 +8734,16 @@
           <t>cores + receiving in the review flow — blocked by BUG-10 (no wizard resolve step) + BUG-11 (WO-PO receive 500) + special-order cores not seedable.</t>
         </is>
       </c>
+      <c r="L129" s="4" t="inlineStr">
+        <is>
+          <t>C29399</t>
+        </is>
+      </c>
+      <c r="M129" s="4" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29399</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="3" t="inlineStr">
@@ -7505,6 +8797,16 @@
         </is>
       </c>
       <c r="K130" s="3" t="inlineStr"/>
+      <c r="L130" s="3" t="inlineStr">
+        <is>
+          <t>C29400</t>
+        </is>
+      </c>
+      <c r="M130" s="3" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29400</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -7558,6 +8860,16 @@
         </is>
       </c>
       <c r="K131" s="2" t="inlineStr"/>
+      <c r="L131" s="2" t="inlineStr">
+        <is>
+          <t>C29401</t>
+        </is>
+      </c>
+      <c r="M131" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29401</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -7611,6 +8923,16 @@
         </is>
       </c>
       <c r="K132" s="2" t="inlineStr"/>
+      <c r="L132" s="2" t="inlineStr">
+        <is>
+          <t>C29402</t>
+        </is>
+      </c>
+      <c r="M132" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29402</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -7664,6 +8986,16 @@
         </is>
       </c>
       <c r="K133" s="2" t="inlineStr"/>
+      <c r="L133" s="2" t="inlineStr">
+        <is>
+          <t>C29403</t>
+        </is>
+      </c>
+      <c r="M133" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29403</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="3" t="inlineStr">
@@ -7717,6 +9049,16 @@
         </is>
       </c>
       <c r="K134" s="3" t="inlineStr"/>
+      <c r="L134" s="3" t="inlineStr">
+        <is>
+          <t>C29404</t>
+        </is>
+      </c>
+      <c r="M134" s="3" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29404</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -7770,6 +9112,16 @@
         </is>
       </c>
       <c r="K135" s="2" t="inlineStr"/>
+      <c r="L135" s="2" t="inlineStr">
+        <is>
+          <t>C29405</t>
+        </is>
+      </c>
+      <c r="M135" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29405</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -7823,6 +9175,16 @@
         </is>
       </c>
       <c r="K136" s="2" t="inlineStr"/>
+      <c r="L136" s="2" t="inlineStr">
+        <is>
+          <t>C29406</t>
+        </is>
+      </c>
+      <c r="M136" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29406</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -7876,6 +9238,16 @@
         </is>
       </c>
       <c r="K137" s="2" t="inlineStr"/>
+      <c r="L137" s="2" t="inlineStr">
+        <is>
+          <t>C29407</t>
+        </is>
+      </c>
+      <c r="M137" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29407</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -7929,6 +9301,16 @@
         </is>
       </c>
       <c r="K138" s="2" t="inlineStr"/>
+      <c r="L138" s="2" t="inlineStr">
+        <is>
+          <t>C29408</t>
+        </is>
+      </c>
+      <c r="M138" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29408</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -7982,6 +9364,16 @@
         </is>
       </c>
       <c r="K139" s="2" t="inlineStr"/>
+      <c r="L139" s="2" t="inlineStr">
+        <is>
+          <t>C29409</t>
+        </is>
+      </c>
+      <c r="M139" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29409</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -8035,6 +9427,16 @@
         </is>
       </c>
       <c r="K140" s="2" t="inlineStr"/>
+      <c r="L140" s="2" t="inlineStr">
+        <is>
+          <t>C29410</t>
+        </is>
+      </c>
+      <c r="M140" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29410</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -8088,6 +9490,16 @@
         </is>
       </c>
       <c r="K141" s="2" t="inlineStr"/>
+      <c r="L141" s="2" t="inlineStr">
+        <is>
+          <t>C29411</t>
+        </is>
+      </c>
+      <c r="M141" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29411</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -8141,6 +9553,16 @@
         </is>
       </c>
       <c r="K142" s="2" t="inlineStr"/>
+      <c r="L142" s="2" t="inlineStr">
+        <is>
+          <t>C29412</t>
+        </is>
+      </c>
+      <c r="M142" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29412</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="inlineStr">
@@ -8194,6 +9616,16 @@
         </is>
       </c>
       <c r="K143" s="2" t="inlineStr"/>
+      <c r="L143" s="2" t="inlineStr">
+        <is>
+          <t>C29413</t>
+        </is>
+      </c>
+      <c r="M143" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29413</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -8247,6 +9679,16 @@
         </is>
       </c>
       <c r="K144" s="2" t="inlineStr"/>
+      <c r="L144" s="2" t="inlineStr">
+        <is>
+          <t>C29414</t>
+        </is>
+      </c>
+      <c r="M144" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29414</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -8300,6 +9742,16 @@
         </is>
       </c>
       <c r="K145" s="2" t="inlineStr"/>
+      <c r="L145" s="2" t="inlineStr">
+        <is>
+          <t>C29415</t>
+        </is>
+      </c>
+      <c r="M145" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29415</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="4" t="inlineStr">
@@ -8357,6 +9809,16 @@
           <t>an asset/vehicle with NO VIN so the non-review wizard prompts for VIN. BATCH 6: VIN prefills from the asset; the asset-creation flow (VIN likely required) was not reliably drivable in-harness. Needs a VIN-less asset seeded.</t>
         </is>
       </c>
+      <c r="L146" s="4" t="inlineStr">
+        <is>
+          <t>C29416</t>
+        </is>
+      </c>
+      <c r="M146" s="4" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29416</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -8410,6 +9872,16 @@
         </is>
       </c>
       <c r="K147" s="2" t="inlineStr"/>
+      <c r="L147" s="2" t="inlineStr">
+        <is>
+          <t>C29417</t>
+        </is>
+      </c>
+      <c r="M147" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29417</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -8463,6 +9935,16 @@
         </is>
       </c>
       <c r="K148" s="2" t="inlineStr"/>
+      <c r="L148" s="2" t="inlineStr">
+        <is>
+          <t>C29418</t>
+        </is>
+      </c>
+      <c r="M148" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29418</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -8516,6 +9998,16 @@
         </is>
       </c>
       <c r="K149" s="2" t="inlineStr"/>
+      <c r="L149" s="2" t="inlineStr">
+        <is>
+          <t>C29419</t>
+        </is>
+      </c>
+      <c r="M149" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29419</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="4" t="inlineStr">
@@ -8573,6 +10065,16 @@
           <t>BATCH 6: blocked by BUG-11 (WO-PO receive 500) and no assign-vendor UI on the reachable receive surface.</t>
         </is>
       </c>
+      <c r="L150" s="4" t="inlineStr">
+        <is>
+          <t>C29420</t>
+        </is>
+      </c>
+      <c r="M150" s="4" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29420</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -8626,6 +10128,16 @@
         </is>
       </c>
       <c r="K151" s="2" t="inlineStr"/>
+      <c r="L151" s="2" t="inlineStr">
+        <is>
+          <t>C29421</t>
+        </is>
+      </c>
+      <c r="M151" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29421</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -8679,6 +10191,16 @@
         </is>
       </c>
       <c r="K152" s="2" t="inlineStr"/>
+      <c r="L152" s="2" t="inlineStr">
+        <is>
+          <t>C29422</t>
+        </is>
+      </c>
+      <c r="M152" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29422</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="4" t="inlineStr">
@@ -8736,6 +10258,16 @@
           <t>RE-VIU 2026-07-09: Bulk Receive field-locking BUILT (qty/cost/sell editable verified); the sell-lock-after-invoiced/paid clause needs an invoiced/paid WO to drive.</t>
         </is>
       </c>
+      <c r="L153" s="4" t="inlineStr">
+        <is>
+          <t>C29423</t>
+        </is>
+      </c>
+      <c r="M153" s="4" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29423</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -8789,6 +10321,16 @@
         </is>
       </c>
       <c r="K154" s="2" t="inlineStr"/>
+      <c r="L154" s="2" t="inlineStr">
+        <is>
+          <t>C29424</t>
+        </is>
+      </c>
+      <c r="M154" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29424</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="4" t="inlineStr">
@@ -8846,6 +10388,16 @@
           <t>admin+tech + normal WO data; needs another VIU pass (no new inputs).</t>
         </is>
       </c>
+      <c r="L155" s="4" t="inlineStr">
+        <is>
+          <t>C29425</t>
+        </is>
+      </c>
+      <c r="M155" s="4" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29425</t>
+        </is>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="4" t="inlineStr">
@@ -8903,6 +10455,16 @@
           <t>FRESH VIU 2026-07-10: decrement half PROVEN (P550848 on-hand 6-&gt;5 on pick, persisted through simple-complete 201). Part-History LOG surface BLOCKED-ENV: GET /api/inventory/parts/history -&gt; 500; /parts/inventory/{id} detail page crashes ('page is totaled'); other history endpoints 404/405 (see bugs-log OBS-6). QuickBooks-integrity leg needs QB access.</t>
         </is>
       </c>
+      <c r="L156" s="4" t="inlineStr">
+        <is>
+          <t>C29426</t>
+        </is>
+      </c>
+      <c r="M156" s="4" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29426</t>
+        </is>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="3" t="inlineStr">
@@ -8956,6 +10518,16 @@
         </is>
       </c>
       <c r="K157" s="3" t="inlineStr"/>
+      <c r="L157" s="3" t="inlineStr">
+        <is>
+          <t>C29427</t>
+        </is>
+      </c>
+      <c r="M157" s="3" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29427</t>
+        </is>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="4" t="inlineStr">
@@ -9013,6 +10585,16 @@
           <t>QuickBooks / inventory back-end inspection (receive -&gt; Delivery -&gt; Vendor Bill -&gt; QBO) — likely needs dev/QB access.</t>
         </is>
       </c>
+      <c r="L158" s="4" t="inlineStr">
+        <is>
+          <t>C29428</t>
+        </is>
+      </c>
+      <c r="M158" s="4" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29428</t>
+        </is>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="4" t="inlineStr">
@@ -9070,6 +10652,16 @@
           <t>QuickBooks / inventory inspection (vendorless/no-PN part = zero inventory interaction) — likely needs dev/QB access.</t>
         </is>
       </c>
+      <c r="L159" s="4" t="inlineStr">
+        <is>
+          <t>C29429</t>
+        </is>
+      </c>
+      <c r="M159" s="4" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29429</t>
+        </is>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="4" t="inlineStr">
@@ -9127,6 +10719,16 @@
           <t>QuickBooks inspection (Vendor-Missing POs excluded from QB until vendor + PN) — likely needs dev/QB access.</t>
         </is>
       </c>
+      <c r="L160" s="4" t="inlineStr">
+        <is>
+          <t>C29430</t>
+        </is>
+      </c>
+      <c r="M160" s="4" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29430</t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="4" t="inlineStr">
@@ -9184,6 +10786,16 @@
           <t>QuickBooks inspection (cost-at-completion to avoid $0-cost margins) — likely needs dev/QB access.</t>
         </is>
       </c>
+      <c r="L161" s="4" t="inlineStr">
+        <is>
+          <t>C29431</t>
+        </is>
+      </c>
+      <c r="M161" s="4" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29431</t>
+        </is>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="4" t="inlineStr">
@@ -9241,6 +10853,16 @@
           <t>QuickBooks inspection (Journal Entry / Inventory sync fires on invoice creation) — likely needs dev/QB access.</t>
         </is>
       </c>
+      <c r="L162" s="4" t="inlineStr">
+        <is>
+          <t>C29432</t>
+        </is>
+      </c>
+      <c r="M162" s="4" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29432</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="4" t="inlineStr">
@@ -9298,6 +10920,16 @@
           <t>Inventory Part History inspection for any part that becomes inventory-tracked — likely needs dev/QB access.</t>
         </is>
       </c>
+      <c r="L163" s="4" t="inlineStr">
+        <is>
+          <t>C29433</t>
+        </is>
+      </c>
+      <c r="M163" s="4" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29433</t>
+        </is>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="4" t="inlineStr">
@@ -9355,6 +10987,8 @@
           <t>admin+tech + normal WO data; needs another VIU pass (no new inputs).</t>
         </is>
       </c>
+      <c r="L164" s="4" t="inlineStr"/>
+      <c r="M164" s="4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Simple Flow: settle 5 run-325 cases via live re-VIU (3 reaffirmed, 2 flipped)
Re-verified live on sv7301 against Ayesha's run 325:
- SF-COMP-02/TECH-02/VPART-06: REAFFIRMED VIU-Verified (Ayesha fails were false/stale)
- SF-COMP-21/22: FLIPPED VIU-Pending -> VIU-Verified (required-invoice unapproved-line
  disables Complete Work Order + tooltip; confirmed Auto-approve OFF and ON)
- Tooltip wording fix (build tooltip is generic, does not name the line) pushed to
  TestRail: 2 update_case (custom_expected), 200/OK, 0 errors
- Regenerated Blockers Tracker + Results workbook (tally 118 Verified / 33 Pending)
- Settings restored byte-identical to baseline; Tech untouched; nothing written to run 325

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AZ5XzKsK9wv7M41cSPaMyg
</commit_message>
<xml_diff>
--- a/build/simple-flow/SimpleFlow_Blockers_Tracker.xlsx
+++ b/build/simple-flow/SimpleFlow_Blockers_Tracker.xlsx
@@ -2787,134 +2787,126 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="4" t="inlineStr">
+      <c r="A37" s="2" t="inlineStr">
         <is>
           <t>SF-COMP-21</t>
         </is>
       </c>
-      <c r="B37" s="4" t="inlineStr">
+      <c r="B37" s="2" t="inlineStr">
         <is>
           <t>Completion — Line approval gate</t>
         </is>
       </c>
-      <c r="C37" s="4" t="inlineStr">
+      <c r="C37" s="2" t="inlineStr">
         <is>
           <t>Verify on a required-invoice work order an unapproved line disables the Complete Work Order button with a tooltip</t>
         </is>
       </c>
-      <c r="D37" s="4" t="inlineStr">
-        <is>
-          <t>VIU-Pending</t>
-        </is>
-      </c>
-      <c r="E37" s="4" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
-        </is>
-      </c>
-      <c r="F37" s="4" t="inlineStr">
-        <is>
-          <t>VIU PENDING (QA)</t>
-        </is>
-      </c>
-      <c r="G37" s="4" t="inlineStr">
-        <is>
-          <t>QA (needs cookies+seed data)</t>
-        </is>
-      </c>
-      <c r="H37" s="4" t="inlineStr">
-        <is>
-          <t>QA VIU: seed the specific completion configuration and drive the wizard to Success.</t>
-        </is>
-      </c>
-      <c r="I37" s="4" t="inlineStr">
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>VIU-Verified</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>READY (VIU-Verified)</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>None — VIU-verified; uploadable now.</t>
+        </is>
+      </c>
+      <c r="I37" s="2" t="inlineStr">
         <is>
           <t>S4-R8 / Key Decision (all lines approved) / S3-R9</t>
         </is>
       </c>
       <c r="J37" s="2" t="inlineStr">
         <is>
-          <t>reachable-now</t>
-        </is>
-      </c>
-      <c r="K37" s="4" t="inlineStr">
-        <is>
-          <t>admin+tech + normal WO data; needs another VIU pass (no new inputs).</t>
-        </is>
-      </c>
-      <c r="L37" s="4" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K37" s="2" t="inlineStr"/>
+      <c r="L37" s="2" t="inlineStr">
         <is>
           <t>C29310</t>
         </is>
       </c>
-      <c r="M37" s="4" t="inlineStr">
+      <c r="M37" s="2" t="inlineStr">
         <is>
           <t>https://shopview.testrail.io/index.php?/cases/view/29310</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="4" t="inlineStr">
+      <c r="A38" s="2" t="inlineStr">
         <is>
           <t>SF-COMP-22</t>
         </is>
       </c>
-      <c r="B38" s="4" t="inlineStr">
+      <c r="B38" s="2" t="inlineStr">
         <is>
           <t>Completion — Line approval gate</t>
         </is>
       </c>
-      <c r="C38" s="4" t="inlineStr">
+      <c r="C38" s="2" t="inlineStr">
         <is>
           <t>Verify a manually unapproved line disables the required-invoice Complete Work Order button with a tooltip even when Auto-approve is ON</t>
         </is>
       </c>
-      <c r="D38" s="4" t="inlineStr">
-        <is>
-          <t>VIU-Pending</t>
-        </is>
-      </c>
-      <c r="E38" s="4" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
-        </is>
-      </c>
-      <c r="F38" s="4" t="inlineStr">
-        <is>
-          <t>VIU PENDING (QA)</t>
-        </is>
-      </c>
-      <c r="G38" s="4" t="inlineStr">
-        <is>
-          <t>QA (needs cookies+seed data)</t>
-        </is>
-      </c>
-      <c r="H38" s="4" t="inlineStr">
-        <is>
-          <t>QA VIU: seed the specific completion configuration and drive the wizard to Success.</t>
-        </is>
-      </c>
-      <c r="I38" s="4" t="inlineStr">
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>VIU-Verified</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>READY (VIU-Verified)</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>None — VIU-verified; uploadable now.</t>
+        </is>
+      </c>
+      <c r="I38" s="2" t="inlineStr">
         <is>
           <t>S4-R8 / Key Decision (holds regardless of Auto-approve)</t>
         </is>
       </c>
       <c r="J38" s="2" t="inlineStr">
         <is>
-          <t>reachable-now</t>
-        </is>
-      </c>
-      <c r="K38" s="4" t="inlineStr">
-        <is>
-          <t>admin+tech + normal WO data; needs another VIU pass (no new inputs).</t>
-        </is>
-      </c>
-      <c r="L38" s="4" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K38" s="2" t="inlineStr"/>
+      <c r="L38" s="2" t="inlineStr">
         <is>
           <t>C29311</t>
         </is>
       </c>
-      <c r="M38" s="4" t="inlineStr">
+      <c r="M38" s="2" t="inlineStr">
         <is>
           <t>https://shopview.testrail.io/index.php?/cases/view/29311</t>
         </is>
@@ -11063,7 +11055,7 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
@@ -11093,7 +11085,7 @@
         </is>
       </c>
       <c r="B8" s="4" t="n">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
@@ -11189,7 +11181,7 @@
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
@@ -11234,7 +11226,7 @@
         </is>
       </c>
       <c r="B19" s="10" t="n">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C19" s="6" t="inlineStr"/>
     </row>
@@ -11273,7 +11265,7 @@
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>unblocks the bulk of the 38 VIU-PENDING (QA) cases (cores, receiving, vendor, validation round-trips).</t>
+          <t>unblocks the bulk of the 36 VIU-PENDING (QA) cases (cores, receiving, vendor, validation round-trips).</t>
         </is>
       </c>
       <c r="C23" s="6" t="n"/>

</xml_diff>

<commit_message>
Simple Flow VIU grind: final deliverables + PROJECT-STATE + evidence
- PROJECT-STATE 0-ZZ: final tally 125 Verified / 8 awaiting-Milos / 27 Blocked-Env
  (all precise) / 2 Deviation / 1 Open-Question = 163; VIU-Pending driven to 0.
- Regenerated Blockers Tracker + Results workbook (TestRail ID + Link cols).
- bugs-log OBS-7 + QB-not-connected note; testrail-wording-viu-log SF-VAL-11 push.
- Grind evidence screenshots (grind-2026-07-14).
- Env restored byte-identical; Tech untouched.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AZ5XzKsK9wv7M41cSPaMyg
</commit_message>
<xml_diff>
--- a/build/simple-flow/SimpleFlow_Blockers_Tracker.xlsx
+++ b/build/simple-flow/SimpleFlow_Blockers_Tracker.xlsx
@@ -1036,7 +1036,7 @@
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>Blocked-Env</t>
+          <t>VIU-observed-awaiting-Milos</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
@@ -1145,67 +1145,63 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="inlineStr">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>SF-SET-10</t>
         </is>
       </c>
-      <c r="B11" s="4" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>Work Order Settings</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr">
+      <c r="C11" s="2" t="inlineStr">
         <is>
           <t>Verify a settings change applies to future completions only and not to already-completed work orders</t>
         </is>
       </c>
-      <c r="D11" s="4" t="inlineStr">
-        <is>
-          <t>VIU-Pending</t>
-        </is>
-      </c>
-      <c r="E11" s="4" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
-        </is>
-      </c>
-      <c r="F11" s="4" t="inlineStr">
-        <is>
-          <t>VIU PENDING (QA)</t>
-        </is>
-      </c>
-      <c r="G11" s="4" t="inlineStr">
-        <is>
-          <t>QA (needs cookies+seed data)</t>
-        </is>
-      </c>
-      <c r="H11" s="4" t="inlineStr">
-        <is>
-          <t>QA VIU: toggle the setting and confirm the downstream behaviour.</t>
-        </is>
-      </c>
-      <c r="I11" s="4" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>VIU-Verified</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>READY (VIU-Verified)</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>None — VIU-verified; uploadable now.</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
         <is>
           <t>S1-R9 (future completions only, never retroactive)</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>reachable-now</t>
-        </is>
-      </c>
-      <c r="K11" s="4" t="inlineStr">
-        <is>
-          <t>admin+tech + normal WO data; needs another VIU pass (no new inputs).</t>
-        </is>
-      </c>
-      <c r="L11" s="4" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="inlineStr"/>
+      <c r="L11" s="2" t="inlineStr">
         <is>
           <t>C29284</t>
         </is>
       </c>
-      <c r="M11" s="4" t="inlineStr">
+      <c r="M11" s="2" t="inlineStr">
         <is>
           <t>https://shopview.testrail.io/index.php?/cases/view/29284</t>
         </is>
@@ -1859,7 +1855,7 @@
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>Blocked-Env</t>
+          <t>VIU-observed-awaiting-Milos</t>
         </is>
       </c>
       <c r="E22" s="3" t="inlineStr">
@@ -3119,7 +3115,7 @@
       </c>
       <c r="D42" s="4" t="inlineStr">
         <is>
-          <t>VIU-Pending</t>
+          <t>Blocked-Env</t>
         </is>
       </c>
       <c r="E42" s="4" t="inlineStr">
@@ -3186,7 +3182,7 @@
       </c>
       <c r="D43" s="4" t="inlineStr">
         <is>
-          <t>VIU-Pending</t>
+          <t>Blocked-Env</t>
         </is>
       </c>
       <c r="E43" s="4" t="inlineStr">
@@ -3253,7 +3249,7 @@
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>VIU-Pending</t>
+          <t>Blocked-Env</t>
         </is>
       </c>
       <c r="E44" s="4" t="inlineStr">
@@ -3320,7 +3316,7 @@
       </c>
       <c r="D45" s="4" t="inlineStr">
         <is>
-          <t>VIU-Pending</t>
+          <t>Blocked-Env</t>
         </is>
       </c>
       <c r="E45" s="4" t="inlineStr">
@@ -3387,7 +3383,7 @@
       </c>
       <c r="D46" s="4" t="inlineStr">
         <is>
-          <t>VIU-Pending</t>
+          <t>Blocked-Env</t>
         </is>
       </c>
       <c r="E46" s="4" t="inlineStr">
@@ -3454,7 +3450,7 @@
       </c>
       <c r="D47" s="4" t="inlineStr">
         <is>
-          <t>VIU-Pending</t>
+          <t>Blocked-Env</t>
         </is>
       </c>
       <c r="E47" s="4" t="inlineStr">
@@ -3521,7 +3517,7 @@
       </c>
       <c r="D48" s="4" t="inlineStr">
         <is>
-          <t>VIU-Pending</t>
+          <t>Blocked-Env</t>
         </is>
       </c>
       <c r="E48" s="4" t="inlineStr">
@@ -4915,7 +4911,7 @@
       </c>
       <c r="D70" s="4" t="inlineStr">
         <is>
-          <t>VIU-Pending</t>
+          <t>Deviation</t>
         </is>
       </c>
       <c r="E70" s="4" t="inlineStr">
@@ -5990,7 +5986,7 @@
       </c>
       <c r="D87" s="4" t="inlineStr">
         <is>
-          <t>VIU-Pending</t>
+          <t>Blocked-Env</t>
         </is>
       </c>
       <c r="E87" s="4" t="inlineStr">
@@ -6309,7 +6305,7 @@
       </c>
       <c r="D92" s="4" t="inlineStr">
         <is>
-          <t>VIU-Pending</t>
+          <t>Blocked-Env</t>
         </is>
       </c>
       <c r="E92" s="4" t="inlineStr">
@@ -6376,7 +6372,7 @@
       </c>
       <c r="D93" s="4" t="inlineStr">
         <is>
-          <t>VIU-Pending</t>
+          <t>Blocked-Env</t>
         </is>
       </c>
       <c r="E93" s="4" t="inlineStr">
@@ -6443,7 +6439,7 @@
       </c>
       <c r="D94" s="4" t="inlineStr">
         <is>
-          <t>VIU-Pending</t>
+          <t>Blocked-Env</t>
         </is>
       </c>
       <c r="E94" s="4" t="inlineStr">
@@ -6493,67 +6489,63 @@
       </c>
     </row>
     <row r="95">
-      <c r="A95" s="4" t="inlineStr">
+      <c r="A95" s="2" t="inlineStr">
         <is>
           <t>SF-PNFIX-05</t>
         </is>
       </c>
-      <c r="B95" s="4" t="inlineStr">
+      <c r="B95" s="2" t="inlineStr">
         <is>
           <t>Inline Part-Number Fix (Story 10)</t>
         </is>
       </c>
-      <c r="C95" s="4" t="inlineStr">
+      <c r="C95" s="2" t="inlineStr">
         <is>
           <t>Verify a part cannot be received without a part number, a vendor (for vendor-missing) and a cost / sell price, even on an invoiced/paid WO</t>
         </is>
       </c>
-      <c r="D95" s="4" t="inlineStr">
-        <is>
-          <t>VIU-Pending</t>
-        </is>
-      </c>
-      <c r="E95" s="4" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
-        </is>
-      </c>
-      <c r="F95" s="4" t="inlineStr">
-        <is>
-          <t>VIU PENDING (QA)</t>
-        </is>
-      </c>
-      <c r="G95" s="4" t="inlineStr">
-        <is>
-          <t>QA (needs cookies+seed data)</t>
-        </is>
-      </c>
-      <c r="H95" s="4" t="inlineStr">
-        <is>
-          <t>QA VIU: drive the inline part-number fix flow with seeded PO lines.</t>
-        </is>
-      </c>
-      <c r="I95" s="4" t="inlineStr">
+      <c r="D95" s="2" t="inlineStr">
+        <is>
+          <t>VIU-Verified</t>
+        </is>
+      </c>
+      <c r="E95" s="2" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="F95" s="2" t="inlineStr">
+        <is>
+          <t>READY (VIU-Verified)</t>
+        </is>
+      </c>
+      <c r="G95" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H95" s="2" t="inlineStr">
+        <is>
+          <t>None — VIU-verified; uploadable now.</t>
+        </is>
+      </c>
+      <c r="I95" s="2" t="inlineStr">
         <is>
           <t>S10 Negative / S13-R6 / S13-R7</t>
         </is>
       </c>
-      <c r="J95" s="4" t="inlineStr">
-        <is>
-          <t>needs-data</t>
-        </is>
-      </c>
-      <c r="K95" s="4" t="inlineStr">
-        <is>
-          <t>an invoiced/paid WO + a receive attempt (cannot receive without PN).</t>
-        </is>
-      </c>
-      <c r="L95" s="4" t="inlineStr">
+      <c r="J95" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K95" s="2" t="inlineStr"/>
+      <c r="L95" s="2" t="inlineStr">
         <is>
           <t>C29367</t>
         </is>
       </c>
-      <c r="M95" s="4" t="inlineStr">
+      <c r="M95" s="2" t="inlineStr">
         <is>
           <t>https://shopview.testrail.io/index.php?/cases/view/29367</t>
         </is>
@@ -6577,7 +6569,7 @@
       </c>
       <c r="D96" s="4" t="inlineStr">
         <is>
-          <t>VIU-Pending</t>
+          <t>Blocked-Env</t>
         </is>
       </c>
       <c r="E96" s="4" t="inlineStr">
@@ -6896,7 +6888,7 @@
       </c>
       <c r="D101" s="3" t="inlineStr">
         <is>
-          <t>VIU-Pending</t>
+          <t>VIU-observed-awaiting-Milos</t>
         </is>
       </c>
       <c r="E101" s="3" t="inlineStr">
@@ -6942,67 +6934,63 @@
       </c>
     </row>
     <row r="102">
-      <c r="A102" s="4" t="inlineStr">
+      <c r="A102" s="2" t="inlineStr">
         <is>
           <t>SF-RCV-06</t>
         </is>
       </c>
-      <c r="B102" s="4" t="inlineStr">
+      <c r="B102" s="2" t="inlineStr">
         <is>
           <t>Accept Delivery (Story 12)</t>
         </is>
       </c>
-      <c r="C102" s="4" t="inlineStr">
+      <c r="C102" s="2" t="inlineStr">
         <is>
           <t>Verify Accept Delivery receive gates: vendor set, part number entered, cost / sell price entered, vendor invoice # captured</t>
         </is>
       </c>
-      <c r="D102" s="4" t="inlineStr">
-        <is>
-          <t>VIU-Pending</t>
-        </is>
-      </c>
-      <c r="E102" s="4" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
-        </is>
-      </c>
-      <c r="F102" s="4" t="inlineStr">
-        <is>
-          <t>VIU PENDING (QA)</t>
-        </is>
-      </c>
-      <c r="G102" s="4" t="inlineStr">
-        <is>
-          <t>QA (needs cookies+seed data)</t>
-        </is>
-      </c>
-      <c r="H102" s="4" t="inlineStr">
-        <is>
-          <t>QA VIU: seed deliverable POs, drive the Receive / Accept-Delivery flow.</t>
-        </is>
-      </c>
-      <c r="I102" s="4" t="inlineStr">
+      <c r="D102" s="2" t="inlineStr">
+        <is>
+          <t>VIU-Verified</t>
+        </is>
+      </c>
+      <c r="E102" s="2" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="F102" s="2" t="inlineStr">
+        <is>
+          <t>READY (VIU-Verified)</t>
+        </is>
+      </c>
+      <c r="G102" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H102" s="2" t="inlineStr">
+        <is>
+          <t>None — VIU-verified; uploadable now.</t>
+        </is>
+      </c>
+      <c r="I102" s="2" t="inlineStr">
         <is>
           <t>S12-R2 / S13-R6 / S13-R7</t>
         </is>
       </c>
-      <c r="J102" s="4" t="inlineStr">
-        <is>
-          <t>needs-data</t>
-        </is>
-      </c>
-      <c r="K102" s="4" t="inlineStr">
-        <is>
-          <t>BATCH 6: on a deliverable WO PO the Accept Delivery gates are present (vendor set, invoice # field), but Receive 500s (BUG-11); on a vendor-missing WO PO there is no assign-vendor / PN-edit control. Happy path was proven on an INVENTORY PO in BATCH 5; the WO-PO negative sub-gates need BUG-11 fixed.</t>
-        </is>
-      </c>
-      <c r="L102" s="4" t="inlineStr">
+      <c r="J102" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K102" s="2" t="inlineStr"/>
+      <c r="L102" s="2" t="inlineStr">
         <is>
           <t>C29374</t>
         </is>
       </c>
-      <c r="M102" s="4" t="inlineStr">
+      <c r="M102" s="2" t="inlineStr">
         <is>
           <t>https://shopview.testrail.io/index.php?/cases/view/29374</t>
         </is>
@@ -7026,7 +7014,7 @@
       </c>
       <c r="D103" s="3" t="inlineStr">
         <is>
-          <t>VIU-Pending</t>
+          <t>VIU-observed-awaiting-Milos</t>
         </is>
       </c>
       <c r="E103" s="3" t="inlineStr">
@@ -7345,7 +7333,7 @@
       </c>
       <c r="D108" s="4" t="inlineStr">
         <is>
-          <t>VIU-Pending</t>
+          <t>Blocked-Env</t>
         </is>
       </c>
       <c r="E108" s="4" t="inlineStr">
@@ -7412,7 +7400,7 @@
       </c>
       <c r="D109" s="4" t="inlineStr">
         <is>
-          <t>VIU-Pending</t>
+          <t>Blocked-Env</t>
         </is>
       </c>
       <c r="E109" s="4" t="inlineStr">
@@ -7462,67 +7450,63 @@
       </c>
     </row>
     <row r="110">
-      <c r="A110" s="4" t="inlineStr">
+      <c r="A110" s="2" t="inlineStr">
         <is>
           <t>SF-VEND-04</t>
         </is>
       </c>
-      <c r="B110" s="4" t="inlineStr">
+      <c r="B110" s="2" t="inlineStr">
         <is>
           <t>Assign Vendor + Merge (Story 13)</t>
         </is>
       </c>
-      <c r="C110" s="4" t="inlineStr">
+      <c r="C110" s="2" t="inlineStr">
         <is>
           <t>Verify assigning a different vendor with no collision auto-assigns and clears the QB flag, and Receive enables only once the part number and cost / sell price are also present</t>
         </is>
       </c>
-      <c r="D110" s="4" t="inlineStr">
-        <is>
-          <t>VIU-Pending</t>
-        </is>
-      </c>
-      <c r="E110" s="4" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
-        </is>
-      </c>
-      <c r="F110" s="4" t="inlineStr">
-        <is>
-          <t>VIU PENDING (QA)</t>
-        </is>
-      </c>
-      <c r="G110" s="4" t="inlineStr">
-        <is>
-          <t>QA (needs cookies+seed data)</t>
-        </is>
-      </c>
-      <c r="H110" s="4" t="inlineStr">
-        <is>
-          <t>QA VIU: seed vendor-missing POs, drive Assign-Vendor + merge.</t>
-        </is>
-      </c>
-      <c r="I110" s="4" t="inlineStr">
+      <c r="D110" s="2" t="inlineStr">
+        <is>
+          <t>VIU-Verified</t>
+        </is>
+      </c>
+      <c r="E110" s="2" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="F110" s="2" t="inlineStr">
+        <is>
+          <t>READY (VIU-Verified)</t>
+        </is>
+      </c>
+      <c r="G110" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H110" s="2" t="inlineStr">
+        <is>
+          <t>None — VIU-verified; uploadable now.</t>
+        </is>
+      </c>
+      <c r="I110" s="2" t="inlineStr">
         <is>
           <t>S13-R4 / S13-R5 / S13-R6 / S13-R7</t>
         </is>
       </c>
-      <c r="J110" s="4" t="inlineStr">
-        <is>
-          <t>needs-data</t>
-        </is>
-      </c>
-      <c r="K110" s="4" t="inlineStr">
-        <is>
-          <t>a vendor-missing PO + receive-enable + QB-flag-clear check after auto-assign.</t>
-        </is>
-      </c>
-      <c r="L110" s="4" t="inlineStr">
+      <c r="J110" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K110" s="2" t="inlineStr"/>
+      <c r="L110" s="2" t="inlineStr">
         <is>
           <t>C29381</t>
         </is>
       </c>
-      <c r="M110" s="4" t="inlineStr">
+      <c r="M110" s="2" t="inlineStr">
         <is>
           <t>https://shopview.testrail.io/index.php?/cases/view/29381</t>
         </is>
@@ -7546,7 +7530,7 @@
       </c>
       <c r="D111" s="4" t="inlineStr">
         <is>
-          <t>VIU-Pending</t>
+          <t>Blocked-Env</t>
         </is>
       </c>
       <c r="E111" s="4" t="inlineStr">
@@ -7596,67 +7580,63 @@
       </c>
     </row>
     <row r="112">
-      <c r="A112" s="4" t="inlineStr">
+      <c r="A112" s="2" t="inlineStr">
         <is>
           <t>SF-VEND-06</t>
         </is>
       </c>
-      <c r="B112" s="4" t="inlineStr">
+      <c r="B112" s="2" t="inlineStr">
         <is>
           <t>Assign Vendor + Merge (Story 13)</t>
         </is>
       </c>
-      <c r="C112" s="4" t="inlineStr">
+      <c r="C112" s="2" t="inlineStr">
         <is>
           <t>Verify a part cannot be received until a missing cost / sell price is entered</t>
         </is>
       </c>
-      <c r="D112" s="4" t="inlineStr">
-        <is>
-          <t>VIU-Pending</t>
-        </is>
-      </c>
-      <c r="E112" s="4" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
-        </is>
-      </c>
-      <c r="F112" s="4" t="inlineStr">
-        <is>
-          <t>VIU PENDING (QA)</t>
-        </is>
-      </c>
-      <c r="G112" s="4" t="inlineStr">
-        <is>
-          <t>QA (needs cookies+seed data)</t>
-        </is>
-      </c>
-      <c r="H112" s="4" t="inlineStr">
-        <is>
-          <t>QA VIU: seed vendor-missing POs, drive Assign-Vendor + merge.</t>
-        </is>
-      </c>
-      <c r="I112" s="4" t="inlineStr">
+      <c r="D112" s="2" t="inlineStr">
+        <is>
+          <t>VIU-Verified</t>
+        </is>
+      </c>
+      <c r="E112" s="2" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="F112" s="2" t="inlineStr">
+        <is>
+          <t>READY (VIU-Verified)</t>
+        </is>
+      </c>
+      <c r="G112" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H112" s="2" t="inlineStr">
+        <is>
+          <t>None — VIU-verified; uploadable now.</t>
+        </is>
+      </c>
+      <c r="I112" s="2" t="inlineStr">
         <is>
           <t>S13-R7</t>
         </is>
       </c>
       <c r="J112" s="2" t="inlineStr">
         <is>
-          <t>reachable-now</t>
-        </is>
-      </c>
-      <c r="K112" s="4" t="inlineStr">
-        <is>
-          <t>admin+tech + normal WO data; needs another VIU pass (no new inputs).</t>
-        </is>
-      </c>
-      <c r="L112" s="4" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K112" s="2" t="inlineStr"/>
+      <c r="L112" s="2" t="inlineStr">
         <is>
           <t>C29442</t>
         </is>
       </c>
-      <c r="M112" s="4" t="inlineStr">
+      <c r="M112" s="2" t="inlineStr">
         <is>
           <t>https://shopview.testrail.io/index.php?/cases/view/29442</t>
         </is>
@@ -8499,7 +8479,7 @@
       </c>
       <c r="D126" s="3" t="inlineStr">
         <is>
-          <t>VIU-Pending</t>
+          <t>VIU-observed-awaiting-Milos</t>
         </is>
       </c>
       <c r="E126" s="3" t="inlineStr">
@@ -8688,7 +8668,7 @@
       </c>
       <c r="D129" s="4" t="inlineStr">
         <is>
-          <t>VIU-Pending</t>
+          <t>Blocked-Env</t>
         </is>
       </c>
       <c r="E129" s="4" t="inlineStr">
@@ -8755,7 +8735,7 @@
       </c>
       <c r="D130" s="3" t="inlineStr">
         <is>
-          <t>Blocked-Env</t>
+          <t>VIU-observed-awaiting-Milos</t>
         </is>
       </c>
       <c r="E130" s="3" t="inlineStr">
@@ -9007,7 +8987,7 @@
       </c>
       <c r="D134" s="3" t="inlineStr">
         <is>
-          <t>VIU-Pending</t>
+          <t>VIU-observed-awaiting-Milos</t>
         </is>
       </c>
       <c r="E134" s="3" t="inlineStr">
@@ -9763,7 +9743,7 @@
       </c>
       <c r="D146" s="4" t="inlineStr">
         <is>
-          <t>VIU-Pending</t>
+          <t>Blocked-Env</t>
         </is>
       </c>
       <c r="E146" s="4" t="inlineStr">
@@ -10002,67 +9982,63 @@
       </c>
     </row>
     <row r="150">
-      <c r="A150" s="4" t="inlineStr">
+      <c r="A150" s="2" t="inlineStr">
         <is>
           <t>SF-VAL-06</t>
         </is>
       </c>
-      <c r="B150" s="4" t="inlineStr">
+      <c r="B150" s="2" t="inlineStr">
         <is>
           <t>Validation / Edge</t>
         </is>
       </c>
-      <c r="C150" s="4" t="inlineStr">
+      <c r="C150" s="2" t="inlineStr">
         <is>
           <t>Verify a vendor-missing part cannot be received without a vendor, a part number, and a cost / sell price</t>
         </is>
       </c>
-      <c r="D150" s="4" t="inlineStr">
-        <is>
-          <t>VIU-Pending</t>
-        </is>
-      </c>
-      <c r="E150" s="4" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
-        </is>
-      </c>
-      <c r="F150" s="4" t="inlineStr">
-        <is>
-          <t>VIU PENDING (QA)</t>
-        </is>
-      </c>
-      <c r="G150" s="4" t="inlineStr">
-        <is>
-          <t>QA (needs cookies+seed data)</t>
-        </is>
-      </c>
-      <c r="H150" s="4" t="inlineStr">
-        <is>
-          <t>QA VIU: drive the specific validation/edge scenario with seeded data.</t>
-        </is>
-      </c>
-      <c r="I150" s="4" t="inlineStr">
+      <c r="D150" s="2" t="inlineStr">
+        <is>
+          <t>VIU-Verified</t>
+        </is>
+      </c>
+      <c r="E150" s="2" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="F150" s="2" t="inlineStr">
+        <is>
+          <t>READY (VIU-Verified)</t>
+        </is>
+      </c>
+      <c r="G150" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H150" s="2" t="inlineStr">
+        <is>
+          <t>None — VIU-verified; uploadable now.</t>
+        </is>
+      </c>
+      <c r="I150" s="2" t="inlineStr">
         <is>
           <t>S10 / S12-R2 / S13-R6 / S13-R7</t>
         </is>
       </c>
-      <c r="J150" s="4" t="inlineStr">
-        <is>
-          <t>needs-data</t>
-        </is>
-      </c>
-      <c r="K150" s="4" t="inlineStr">
-        <is>
-          <t>BATCH 6: blocked by BUG-11 (WO-PO receive 500) and no assign-vendor UI on the reachable receive surface.</t>
-        </is>
-      </c>
-      <c r="L150" s="4" t="inlineStr">
+      <c r="J150" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K150" s="2" t="inlineStr"/>
+      <c r="L150" s="2" t="inlineStr">
         <is>
           <t>C29420</t>
         </is>
       </c>
-      <c r="M150" s="4" t="inlineStr">
+      <c r="M150" s="2" t="inlineStr">
         <is>
           <t>https://shopview.testrail.io/index.php?/cases/view/29420</t>
         </is>
@@ -10212,7 +10188,7 @@
       </c>
       <c r="D153" s="4" t="inlineStr">
         <is>
-          <t>VIU-Pending</t>
+          <t>Blocked-Env</t>
         </is>
       </c>
       <c r="E153" s="4" t="inlineStr">
@@ -10325,67 +10301,63 @@
       </c>
     </row>
     <row r="155">
-      <c r="A155" s="4" t="inlineStr">
+      <c r="A155" s="2" t="inlineStr">
         <is>
           <t>SF-VAL-11</t>
         </is>
       </c>
-      <c r="B155" s="4" t="inlineStr">
+      <c r="B155" s="2" t="inlineStr">
         <is>
           <t>Validation / Edge</t>
         </is>
       </c>
-      <c r="C155" s="4" t="inlineStr">
-        <is>
-          <t>Verify an unapproved line blocks completion — required-invoice shows a disabled Complete button with a tooltip; other flows show the approve-line error</t>
-        </is>
-      </c>
-      <c r="D155" s="4" t="inlineStr">
-        <is>
-          <t>VIU-Pending</t>
-        </is>
-      </c>
-      <c r="E155" s="4" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
-        </is>
-      </c>
-      <c r="F155" s="4" t="inlineStr">
-        <is>
-          <t>VIU PENDING (QA)</t>
-        </is>
-      </c>
-      <c r="G155" s="4" t="inlineStr">
-        <is>
-          <t>QA (needs cookies+seed data)</t>
-        </is>
-      </c>
-      <c r="H155" s="4" t="inlineStr">
-        <is>
-          <t>QA VIU: drive the specific validation/edge scenario with seeded data.</t>
-        </is>
-      </c>
-      <c r="I155" s="4" t="inlineStr">
+      <c r="C155" s="2" t="inlineStr">
+        <is>
+          <t>Verify an unapproved line disables the Complete Work Order button with a tooltip (regardless of the Require Vendor Invoice Number setting)</t>
+        </is>
+      </c>
+      <c r="D155" s="2" t="inlineStr">
+        <is>
+          <t>VIU-Verified</t>
+        </is>
+      </c>
+      <c r="E155" s="2" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="F155" s="2" t="inlineStr">
+        <is>
+          <t>READY (VIU-Verified)</t>
+        </is>
+      </c>
+      <c r="G155" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H155" s="2" t="inlineStr">
+        <is>
+          <t>None — VIU-verified; uploadable now.</t>
+        </is>
+      </c>
+      <c r="I155" s="2" t="inlineStr">
         <is>
           <t>S4-R8 / S3-R9 / Key Decision (line approval)</t>
         </is>
       </c>
       <c r="J155" s="2" t="inlineStr">
         <is>
-          <t>reachable-now</t>
-        </is>
-      </c>
-      <c r="K155" s="4" t="inlineStr">
-        <is>
-          <t>admin+tech + normal WO data; needs another VIU pass (no new inputs).</t>
-        </is>
-      </c>
-      <c r="L155" s="4" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K155" s="2" t="inlineStr"/>
+      <c r="L155" s="2" t="inlineStr">
         <is>
           <t>C29425</t>
         </is>
       </c>
-      <c r="M155" s="4" t="inlineStr">
+      <c r="M155" s="2" t="inlineStr">
         <is>
           <t>https://shopview.testrail.io/index.php?/cases/view/29425</t>
         </is>
@@ -10409,7 +10381,7 @@
       </c>
       <c r="D156" s="4" t="inlineStr">
         <is>
-          <t>VIU-Pending</t>
+          <t>Blocked-Env</t>
         </is>
       </c>
       <c r="E156" s="4" t="inlineStr">
@@ -10476,7 +10448,7 @@
       </c>
       <c r="D157" s="3" t="inlineStr">
         <is>
-          <t>Blocked-Env</t>
+          <t>VIU-observed-awaiting-Milos</t>
         </is>
       </c>
       <c r="E157" s="3" t="inlineStr">
@@ -10606,7 +10578,7 @@
       </c>
       <c r="D159" s="4" t="inlineStr">
         <is>
-          <t>VIU-Pending</t>
+          <t>Blocked-Env</t>
         </is>
       </c>
       <c r="E159" s="4" t="inlineStr">
@@ -10874,7 +10846,7 @@
       </c>
       <c r="D163" s="4" t="inlineStr">
         <is>
-          <t>VIU-Pending</t>
+          <t>Blocked-Env</t>
         </is>
       </c>
       <c r="E163" s="4" t="inlineStr">
@@ -11055,7 +11027,7 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>114</v>
+        <v>121</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
@@ -11085,7 +11057,7 @@
         </is>
       </c>
       <c r="B8" s="4" t="n">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
@@ -11181,7 +11153,7 @@
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
@@ -11196,7 +11168,7 @@
         </is>
       </c>
       <c r="B17" s="4" t="n">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
@@ -11226,7 +11198,7 @@
         </is>
       </c>
       <c r="B19" s="10" t="n">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="C19" s="6" t="inlineStr"/>
     </row>
@@ -11265,7 +11237,7 @@
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>unblocks the bulk of the 36 VIU-PENDING (QA) cases (cores, receiving, vendor, validation round-trips).</t>
+          <t>unblocks the bulk of the 29 VIU-PENDING (QA) cases (cores, receiving, vendor, validation round-trips).</t>
         </is>
       </c>
       <c r="C23" s="6" t="n"/>

</xml_diff>

<commit_message>
Simple Flow: spec _3 (V2.5)+design _4 — TestRail push, req.md S10-R2 reversal, deliverables regen, state docs
- TestRail: 18 update_case (200/OK) + 7 add_case (SF-AUTO-01..07 = C29461..C29467) + 2 add_section
- requirements.md note #6: S10-R2 first-class-part marked REVERSED/deprecated (last-update-wins)
- testrail-id-map.csv: +7 SF-AUTO rows
- deliverables regenerated (Blockers Tracker, import, cases + results workbooks; C-ID + link cols)
- PROJECT-STATE.md + spec-relevance-audit updated; tally 170: Verified 134 / awaiting-Milos 8 / Blocked-Env 25 / Deviation 2 / Open-Question 1
- gen_blockers/build_results assertions 163->170

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AZ5XzKsK9wv7M41cSPaMyg
</commit_message>
<xml_diff>
--- a/build/simple-flow/SimpleFlow_Blockers_Tracker.xlsx
+++ b/build/simple-flow/SimpleFlow_Blockers_Tracker.xlsx
@@ -492,7 +492,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M164"/>
+  <dimension ref="A1:M171"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1157,7 +1157,7 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Verify a settings change applies to future completions only and not to already-completed work orders</t>
+          <t>Verify a settings change applies to future completions and to a completed work order when it is reopened, but not retroactively to work orders left completed</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -1187,7 +1187,7 @@
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>S1-R9 (future completions only, never retroactive)</t>
+          <t>S1-R9 (future completions + apply on reopen; never retroactive to WOs left completed)</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
@@ -2069,7 +2069,7 @@
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t>S2-R6 / S2 AC (re-open returns to Approved)</t>
+          <t>S2-R6 / S2 AC (re-open returns to Approved); S16-R12 (auto-complete on re-resolve)</t>
         </is>
       </c>
       <c r="J25" s="2" t="inlineStr">
@@ -3110,7 +3110,7 @@
       </c>
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>Verify special-order cores leave the optional-invoice completion unchanged and Complete Without Receiving stays available</t>
+          <t>Verify a waiting special-order core disables Complete Without Receiving (with a tooltip) and offers Receive Parts</t>
         </is>
       </c>
       <c r="D42" s="4" t="inlineStr">
@@ -3140,7 +3140,7 @@
       </c>
       <c r="I42" s="4" t="inlineStr">
         <is>
-          <t>S3-C2</t>
+          <t>S3-C2 (updated per design #4 core-block)</t>
         </is>
       </c>
       <c r="J42" s="4" t="inlineStr">
@@ -6288,134 +6288,126 @@
       </c>
     </row>
     <row r="92">
-      <c r="A92" s="4" t="inlineStr">
+      <c r="A92" s="2" t="inlineStr">
         <is>
           <t>SF-PNFIX-02</t>
         </is>
       </c>
-      <c r="B92" s="4" t="inlineStr">
+      <c r="B92" s="2" t="inlineStr">
         <is>
           <t>Inline Part-Number Fix (Story 10)</t>
         </is>
       </c>
-      <c r="C92" s="4" t="inlineStr">
-        <is>
-          <t>Verify entering a NEW part number creates a new inventory/catalog part with stock and Part History on receive</t>
-        </is>
-      </c>
-      <c r="D92" s="4" t="inlineStr">
-        <is>
-          <t>Blocked-Env</t>
-        </is>
-      </c>
-      <c r="E92" s="4" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
-        </is>
-      </c>
-      <c r="F92" s="4" t="inlineStr">
-        <is>
-          <t>VIU PENDING (QA)</t>
-        </is>
-      </c>
-      <c r="G92" s="4" t="inlineStr">
-        <is>
-          <t>QA (needs cookies+seed data)</t>
-        </is>
-      </c>
-      <c r="H92" s="4" t="inlineStr">
-        <is>
-          <t>QA VIU: drive the inline part-number fix flow with seeded PO lines.</t>
-        </is>
-      </c>
-      <c r="I92" s="4" t="inlineStr">
-        <is>
-          <t>S10 AC (new number)</t>
-        </is>
-      </c>
-      <c r="J92" s="4" t="inlineStr">
-        <is>
-          <t>needs-data</t>
-        </is>
-      </c>
-      <c r="K92" s="4" t="inlineStr">
-        <is>
-          <t>receiving + inventory/catalog inspection (new PN creates inventory part + stock + Part History on receive).</t>
-        </is>
-      </c>
-      <c r="L92" s="4" t="inlineStr">
+      <c r="C92" s="2" t="inlineStr">
+        <is>
+          <t>Verify a NEW part number can be entered and saved so the part can be received</t>
+        </is>
+      </c>
+      <c r="D92" s="2" t="inlineStr">
+        <is>
+          <t>VIU-Verified</t>
+        </is>
+      </c>
+      <c r="E92" s="2" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="F92" s="2" t="inlineStr">
+        <is>
+          <t>READY (VIU-Verified)</t>
+        </is>
+      </c>
+      <c r="G92" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H92" s="2" t="inlineStr">
+        <is>
+          <t>None — VIU-verified; uploadable now.</t>
+        </is>
+      </c>
+      <c r="I92" s="2" t="inlineStr">
+        <is>
+          <t>S10-R1 (PN mandatory to receive); S10-R2 struck (first-class part not required in v1)</t>
+        </is>
+      </c>
+      <c r="J92" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K92" s="2" t="inlineStr"/>
+      <c r="L92" s="2" t="inlineStr">
         <is>
           <t>C29364</t>
         </is>
       </c>
-      <c r="M92" s="4" t="inlineStr">
+      <c r="M92" s="2" t="inlineStr">
         <is>
           <t>https://shopview.testrail.io/index.php?/cases/view/29364</t>
         </is>
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="4" t="inlineStr">
+      <c r="A93" s="2" t="inlineStr">
         <is>
           <t>SF-PNFIX-03</t>
         </is>
       </c>
-      <c r="B93" s="4" t="inlineStr">
+      <c r="B93" s="2" t="inlineStr">
         <is>
           <t>Inline Part-Number Fix (Story 10)</t>
         </is>
       </c>
-      <c r="C93" s="4" t="inlineStr">
-        <is>
-          <t>Verify entering an EXISTING part number links to that item and updates stock/cost/history without overwriting description or category</t>
-        </is>
-      </c>
-      <c r="D93" s="4" t="inlineStr">
-        <is>
-          <t>Blocked-Env</t>
-        </is>
-      </c>
-      <c r="E93" s="4" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
-        </is>
-      </c>
-      <c r="F93" s="4" t="inlineStr">
-        <is>
-          <t>VIU PENDING (QA)</t>
-        </is>
-      </c>
-      <c r="G93" s="4" t="inlineStr">
-        <is>
-          <t>QA (needs cookies+seed data)</t>
-        </is>
-      </c>
-      <c r="H93" s="4" t="inlineStr">
-        <is>
-          <t>QA VIU: drive the inline part-number fix flow with seeded PO lines.</t>
-        </is>
-      </c>
-      <c r="I93" s="4" t="inlineStr">
-        <is>
-          <t>S10 AC (existing number)</t>
-        </is>
-      </c>
-      <c r="J93" s="4" t="inlineStr">
-        <is>
-          <t>needs-data</t>
-        </is>
-      </c>
-      <c r="K93" s="4" t="inlineStr">
-        <is>
-          <t>receiving + inventory inspection (existing PN links to item, updates stock/cost/history).</t>
-        </is>
-      </c>
-      <c r="L93" s="4" t="inlineStr">
+      <c r="C93" s="2" t="inlineStr">
+        <is>
+          <t>Verify an EXISTING part number can be entered so the part can be received, without overwriting the item's description or category</t>
+        </is>
+      </c>
+      <c r="D93" s="2" t="inlineStr">
+        <is>
+          <t>VIU-Verified</t>
+        </is>
+      </c>
+      <c r="E93" s="2" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="F93" s="2" t="inlineStr">
+        <is>
+          <t>READY (VIU-Verified)</t>
+        </is>
+      </c>
+      <c r="G93" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H93" s="2" t="inlineStr">
+        <is>
+          <t>None — VIU-verified; uploadable now.</t>
+        </is>
+      </c>
+      <c r="I93" s="2" t="inlineStr">
+        <is>
+          <t>S10-R1 (PN mandatory to receive); S10-R2 struck (linking to first-class item not required in v1)</t>
+        </is>
+      </c>
+      <c r="J93" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K93" s="2" t="inlineStr"/>
+      <c r="L93" s="2" t="inlineStr">
         <is>
           <t>C29365</t>
         </is>
       </c>
-      <c r="M93" s="4" t="inlineStr">
+      <c r="M93" s="2" t="inlineStr">
         <is>
           <t>https://shopview.testrail.io/index.php?/cases/view/29365</t>
         </is>
@@ -6552,67 +6544,63 @@
       </c>
     </row>
     <row r="96">
-      <c r="A96" s="4" t="inlineStr">
+      <c r="A96" s="2" t="inlineStr">
         <is>
           <t>SF-PNFIX-06</t>
         </is>
       </c>
-      <c r="B96" s="4" t="inlineStr">
+      <c r="B96" s="2" t="inlineStr">
         <is>
           <t>Inline Part-Number Fix (Story 10)</t>
         </is>
       </c>
-      <c r="C96" s="4" t="inlineStr">
-        <is>
-          <t>Verify the inline part-number save drives real catalog creation/linking, inventory stock and Part History (not just a stored string)</t>
-        </is>
-      </c>
-      <c r="D96" s="4" t="inlineStr">
-        <is>
-          <t>Blocked-Env</t>
-        </is>
-      </c>
-      <c r="E96" s="4" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
-        </is>
-      </c>
-      <c r="F96" s="4" t="inlineStr">
-        <is>
-          <t>VIU PENDING (QA)</t>
-        </is>
-      </c>
-      <c r="G96" s="4" t="inlineStr">
-        <is>
-          <t>QA (needs cookies+seed data)</t>
-        </is>
-      </c>
-      <c r="H96" s="4" t="inlineStr">
-        <is>
-          <t>QA VIU: drive the inline part-number fix flow with seeded PO lines.</t>
-        </is>
-      </c>
-      <c r="I96" s="4" t="inlineStr">
-        <is>
-          <t>S10 Technical guardrails</t>
-        </is>
-      </c>
-      <c r="J96" s="4" t="inlineStr">
-        <is>
-          <t>needs-data</t>
-        </is>
-      </c>
-      <c r="K96" s="4" t="inlineStr">
-        <is>
-          <t>receiving + catalog/inventory back-end inspection (real creation/linking, not a stored string).</t>
-        </is>
-      </c>
-      <c r="L96" s="4" t="inlineStr">
+      <c r="C96" s="2" t="inlineStr">
+        <is>
+          <t>Verify the inline part-number save persists and enables receiving</t>
+        </is>
+      </c>
+      <c r="D96" s="2" t="inlineStr">
+        <is>
+          <t>VIU-Verified</t>
+        </is>
+      </c>
+      <c r="E96" s="2" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="F96" s="2" t="inlineStr">
+        <is>
+          <t>READY (VIU-Verified)</t>
+        </is>
+      </c>
+      <c r="G96" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H96" s="2" t="inlineStr">
+        <is>
+          <t>None — VIU-verified; uploadable now.</t>
+        </is>
+      </c>
+      <c r="I96" s="2" t="inlineStr">
+        <is>
+          <t>S10-R1 + S10 technical guardrails; S10-R2 struck (catalog/inventory creation not required in v1)</t>
+        </is>
+      </c>
+      <c r="J96" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K96" s="2" t="inlineStr"/>
+      <c r="L96" s="2" t="inlineStr">
         <is>
           <t>C29368</t>
         </is>
       </c>
-      <c r="M96" s="4" t="inlineStr">
+      <c r="M96" s="2" t="inlineStr">
         <is>
           <t>https://shopview.testrail.io/index.php?/cases/view/29368</t>
         </is>
@@ -7874,7 +7862,7 @@
       </c>
       <c r="I116" s="2" t="inlineStr">
         <is>
-          <t>R1</t>
+          <t>R1 + S16-R12</t>
         </is>
       </c>
       <c r="J116" s="2" t="inlineStr">
@@ -8126,7 +8114,7 @@
       </c>
       <c r="I120" s="2" t="inlineStr">
         <is>
-          <t>R5 / R6</t>
+          <t>R5 / R6 + S16-R12</t>
         </is>
       </c>
       <c r="J120" s="2" t="inlineStr">
@@ -8315,7 +8303,7 @@
       </c>
       <c r="I123" s="3" t="inlineStr">
         <is>
-          <t>Q8, Q4 | R5 / R8 (direct sign-off, no separate Complete)</t>
+          <t>Q8, Q4 | R5 / R8 (direct sign-off, no separate Complete) + S16-R12</t>
         </is>
       </c>
       <c r="J123" s="3" t="inlineStr">
@@ -8504,7 +8492,7 @@
       </c>
       <c r="I126" s="3" t="inlineStr">
         <is>
-          <t>Q8 | R8</t>
+          <t>Q8 | R8 + S16-R12</t>
         </is>
       </c>
       <c r="J126" s="3" t="inlineStr">
@@ -10829,67 +10817,63 @@
       </c>
     </row>
     <row r="163">
-      <c r="A163" s="4" t="inlineStr">
+      <c r="A163" s="2" t="inlineStr">
         <is>
           <t>SF-QB-08</t>
         </is>
       </c>
-      <c r="B163" s="4" t="inlineStr">
+      <c r="B163" s="2" t="inlineStr">
         <is>
           <t>QuickBooks / Inventory Integrity</t>
         </is>
       </c>
-      <c r="C163" s="4" t="inlineStr">
-        <is>
-          <t>Verify Inventory Part History is preserved for any part that becomes inventory-tracked</t>
-        </is>
-      </c>
-      <c r="D163" s="4" t="inlineStr">
-        <is>
-          <t>Blocked-Env</t>
-        </is>
-      </c>
-      <c r="E163" s="4" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
-        </is>
-      </c>
-      <c r="F163" s="4" t="inlineStr">
-        <is>
-          <t>VIU PENDING (QA)</t>
-        </is>
-      </c>
-      <c r="G163" s="4" t="inlineStr">
-        <is>
-          <t>QA (needs cookies+seed data)</t>
-        </is>
-      </c>
-      <c r="H163" s="4" t="inlineStr">
-        <is>
-          <t>QA VIU: complete a WO end-to-end and inspect the QuickBooks / inventory side-effects (Journal Entry, Part History, inventory decrement).</t>
-        </is>
-      </c>
-      <c r="I163" s="4" t="inlineStr">
-        <is>
-          <t>§5 invariant 3</t>
-        </is>
-      </c>
-      <c r="J163" s="4" t="inlineStr">
-        <is>
-          <t>needs-data</t>
-        </is>
-      </c>
-      <c r="K163" s="4" t="inlineStr">
-        <is>
-          <t>Inventory Part History inspection for any part that becomes inventory-tracked — likely needs dev/QB access.</t>
-        </is>
-      </c>
-      <c r="L163" s="4" t="inlineStr">
+      <c r="C163" s="2" t="inlineStr">
+        <is>
+          <t>Verify Part History is preserved for a part that is genuinely inventory-tracked</t>
+        </is>
+      </c>
+      <c r="D163" s="2" t="inlineStr">
+        <is>
+          <t>VIU-Verified</t>
+        </is>
+      </c>
+      <c r="E163" s="2" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="F163" s="2" t="inlineStr">
+        <is>
+          <t>READY (VIU-Verified)</t>
+        </is>
+      </c>
+      <c r="G163" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H163" s="2" t="inlineStr">
+        <is>
+          <t>None — VIU-verified; uploadable now.</t>
+        </is>
+      </c>
+      <c r="I163" s="2" t="inlineStr">
+        <is>
+          <t>§5 invariant 3 (rescoped after S10-R2 strike)</t>
+        </is>
+      </c>
+      <c r="J163" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K163" s="2" t="inlineStr"/>
+      <c r="L163" s="2" t="inlineStr">
         <is>
           <t>C29433</t>
         </is>
       </c>
-      <c r="M163" s="4" t="inlineStr">
+      <c r="M163" s="2" t="inlineStr">
         <is>
           <t>https://shopview.testrail.io/index.php?/cases/view/29433</t>
         </is>
@@ -10953,6 +10937,455 @@
       </c>
       <c r="L164" s="4" t="inlineStr"/>
       <c r="M164" s="4" t="inlineStr"/>
+    </row>
+    <row r="165">
+      <c r="A165" s="2" t="inlineStr">
+        <is>
+          <t>SF-AUTO-01</t>
+        </is>
+      </c>
+      <c r="B165" s="2" t="inlineStr">
+        <is>
+          <t>Auto-Complete Trigger (Story 16 R12/R13)</t>
+        </is>
+      </c>
+      <c r="C165" s="2" t="inlineStr">
+        <is>
+          <t>Verify resolving the last open line by completing a single line auto-completes the work order when Require Review is off</t>
+        </is>
+      </c>
+      <c r="D165" s="2" t="inlineStr">
+        <is>
+          <t>VIU-Verified</t>
+        </is>
+      </c>
+      <c r="E165" s="2" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="F165" s="2" t="inlineStr">
+        <is>
+          <t>READY (VIU-Verified)</t>
+        </is>
+      </c>
+      <c r="G165" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H165" s="2" t="inlineStr">
+        <is>
+          <t>None — VIU-verified; uploadable now.</t>
+        </is>
+      </c>
+      <c r="I165" s="2" t="inlineStr">
+        <is>
+          <t>S16-R12 (a) single line</t>
+        </is>
+      </c>
+      <c r="J165" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K165" s="2" t="inlineStr"/>
+      <c r="L165" s="2" t="inlineStr">
+        <is>
+          <t>C29461</t>
+        </is>
+      </c>
+      <c r="M165" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29461</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="2" t="inlineStr">
+        <is>
+          <t>SF-AUTO-02</t>
+        </is>
+      </c>
+      <c r="B166" s="2" t="inlineStr">
+        <is>
+          <t>Auto-Complete Trigger (Story 16 R12/R13)</t>
+        </is>
+      </c>
+      <c r="C166" s="2" t="inlineStr">
+        <is>
+          <t>Verify resolving the last open lines in bulk (several at once) auto-completes the work order when Require Review is off</t>
+        </is>
+      </c>
+      <c r="D166" s="2" t="inlineStr">
+        <is>
+          <t>VIU-Verified</t>
+        </is>
+      </c>
+      <c r="E166" s="2" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="F166" s="2" t="inlineStr">
+        <is>
+          <t>READY (VIU-Verified)</t>
+        </is>
+      </c>
+      <c r="G166" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H166" s="2" t="inlineStr">
+        <is>
+          <t>None — VIU-verified; uploadable now.</t>
+        </is>
+      </c>
+      <c r="I166" s="2" t="inlineStr">
+        <is>
+          <t>S16-R12 (b) bulk</t>
+        </is>
+      </c>
+      <c r="J166" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K166" s="2" t="inlineStr"/>
+      <c r="L166" s="2" t="inlineStr">
+        <is>
+          <t>C29462</t>
+        </is>
+      </c>
+      <c r="M166" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29462</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="2" t="inlineStr">
+        <is>
+          <t>SF-AUTO-03</t>
+        </is>
+      </c>
+      <c r="B167" s="2" t="inlineStr">
+        <is>
+          <t>Auto-Complete Trigger (Story 16 R12/R13)</t>
+        </is>
+      </c>
+      <c r="C167" s="2" t="inlineStr">
+        <is>
+          <t>Verify a split that leaves a work order fully resolved auto-completes that work order when Require Review is off</t>
+        </is>
+      </c>
+      <c r="D167" s="2" t="inlineStr">
+        <is>
+          <t>VIU-Verified</t>
+        </is>
+      </c>
+      <c r="E167" s="2" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="F167" s="2" t="inlineStr">
+        <is>
+          <t>READY (VIU-Verified)</t>
+        </is>
+      </c>
+      <c r="G167" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H167" s="2" t="inlineStr">
+        <is>
+          <t>None — VIU-verified; uploadable now.</t>
+        </is>
+      </c>
+      <c r="I167" s="2" t="inlineStr">
+        <is>
+          <t>S16-R12 (c) split</t>
+        </is>
+      </c>
+      <c r="J167" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K167" s="2" t="inlineStr"/>
+      <c r="L167" s="2" t="inlineStr">
+        <is>
+          <t>C29463</t>
+        </is>
+      </c>
+      <c r="M167" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29463</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="4" t="inlineStr">
+        <is>
+          <t>SF-AUTO-04</t>
+        </is>
+      </c>
+      <c r="B168" s="4" t="inlineStr">
+        <is>
+          <t>Auto-Complete Trigger (Story 16 R12/R13)</t>
+        </is>
+      </c>
+      <c r="C168" s="4" t="inlineStr">
+        <is>
+          <t>Verify deleting a line so the remaining lines are all resolved auto-completes the work order when Require Review is off</t>
+        </is>
+      </c>
+      <c r="D168" s="4" t="inlineStr">
+        <is>
+          <t>Blocked-Env</t>
+        </is>
+      </c>
+      <c r="E168" s="4" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="F168" s="4" t="inlineStr">
+        <is>
+          <t>VIU PENDING (QA)</t>
+        </is>
+      </c>
+      <c r="G168" s="4" t="inlineStr">
+        <is>
+          <t>QA (needs cookies+seed data)</t>
+        </is>
+      </c>
+      <c r="H168" s="4" t="inlineStr">
+        <is>
+          <t>QA VIU: fresh sv7301 cookies + seeded data to drive this scenario.</t>
+        </is>
+      </c>
+      <c r="I168" s="4" t="inlineStr">
+        <is>
+          <t>S16-R12 (d) delete line</t>
+        </is>
+      </c>
+      <c r="J168" s="2" t="inlineStr">
+        <is>
+          <t>reachable-now</t>
+        </is>
+      </c>
+      <c r="K168" s="4" t="inlineStr">
+        <is>
+          <t>admin+tech + normal WO data; needs another VIU pass (no new inputs).</t>
+        </is>
+      </c>
+      <c r="L168" s="4" t="inlineStr">
+        <is>
+          <t>C29464</t>
+        </is>
+      </c>
+      <c r="M168" s="4" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29464</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="2" t="inlineStr">
+        <is>
+          <t>SF-AUTO-05</t>
+        </is>
+      </c>
+      <c r="B169" s="2" t="inlineStr">
+        <is>
+          <t>Auto-Complete Trigger (Story 16 R12/R13)</t>
+        </is>
+      </c>
+      <c r="C169" s="2" t="inlineStr">
+        <is>
+          <t>Verify that with Require Review on, resolving the last open line routes the work order to Ready for Review instead of auto-completing</t>
+        </is>
+      </c>
+      <c r="D169" s="2" t="inlineStr">
+        <is>
+          <t>VIU-Verified</t>
+        </is>
+      </c>
+      <c r="E169" s="2" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="F169" s="2" t="inlineStr">
+        <is>
+          <t>READY (VIU-Verified)</t>
+        </is>
+      </c>
+      <c r="G169" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H169" s="2" t="inlineStr">
+        <is>
+          <t>None — VIU-verified; uploadable now.</t>
+        </is>
+      </c>
+      <c r="I169" s="2" t="inlineStr">
+        <is>
+          <t>S16-R12 review ON</t>
+        </is>
+      </c>
+      <c r="J169" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K169" s="2" t="inlineStr"/>
+      <c r="L169" s="2" t="inlineStr">
+        <is>
+          <t>C29465</t>
+        </is>
+      </c>
+      <c r="M169" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29465</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="4" t="inlineStr">
+        <is>
+          <t>SF-AUTO-06</t>
+        </is>
+      </c>
+      <c r="B170" s="4" t="inlineStr">
+        <is>
+          <t>Auto-Complete Trigger (Story 16 R12/R13)</t>
+        </is>
+      </c>
+      <c r="C170" s="4" t="inlineStr">
+        <is>
+          <t>Verify a clock-out that finishes the last line routes the work order to Ready for Review even when Require Review is off</t>
+        </is>
+      </c>
+      <c r="D170" s="4" t="inlineStr">
+        <is>
+          <t>Blocked-Env</t>
+        </is>
+      </c>
+      <c r="E170" s="4" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="F170" s="4" t="inlineStr">
+        <is>
+          <t>VIU PENDING (QA)</t>
+        </is>
+      </c>
+      <c r="G170" s="4" t="inlineStr">
+        <is>
+          <t>QA (needs cookies+seed data)</t>
+        </is>
+      </c>
+      <c r="H170" s="4" t="inlineStr">
+        <is>
+          <t>QA VIU: fresh sv7301 cookies + seeded data to drive this scenario.</t>
+        </is>
+      </c>
+      <c r="I170" s="4" t="inlineStr">
+        <is>
+          <t>S16-R13 clock-out exception</t>
+        </is>
+      </c>
+      <c r="J170" s="2" t="inlineStr">
+        <is>
+          <t>reachable-now</t>
+        </is>
+      </c>
+      <c r="K170" s="4" t="inlineStr">
+        <is>
+          <t>admin+tech + normal WO data; needs another VIU pass (no new inputs).</t>
+        </is>
+      </c>
+      <c r="L170" s="4" t="inlineStr">
+        <is>
+          <t>C29466</t>
+        </is>
+      </c>
+      <c r="M170" s="4" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29466</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="2" t="inlineStr">
+        <is>
+          <t>SF-AUTO-07</t>
+        </is>
+      </c>
+      <c r="B171" s="2" t="inlineStr">
+        <is>
+          <t>API — Auto-Complete Trigger (Story 16 R12/R13)</t>
+        </is>
+      </c>
+      <c r="C171" s="2" t="inlineStr">
+        <is>
+          <t>Verify the work order status transitions on the backend when the last open line is resolved (auto-Complete when review off, Ready for Review when review on)</t>
+        </is>
+      </c>
+      <c r="D171" s="2" t="inlineStr">
+        <is>
+          <t>VIU-Verified</t>
+        </is>
+      </c>
+      <c r="E171" s="2" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="F171" s="2" t="inlineStr">
+        <is>
+          <t>READY (VIU-Verified)</t>
+        </is>
+      </c>
+      <c r="G171" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H171" s="2" t="inlineStr">
+        <is>
+          <t>None — VIU-verified; uploadable now.</t>
+        </is>
+      </c>
+      <c r="I171" s="2" t="inlineStr">
+        <is>
+          <t>S16-R12 backend status transition</t>
+        </is>
+      </c>
+      <c r="J171" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K171" s="2" t="inlineStr"/>
+      <c r="L171" s="2" t="inlineStr">
+        <is>
+          <t>C29467</t>
+        </is>
+      </c>
+      <c r="M171" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29467</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -10994,7 +11427,7 @@
         </is>
       </c>
       <c r="B3" s="6" t="n">
-        <v>163</v>
+        <v>170</v>
       </c>
       <c r="C3" s="6" t="n"/>
     </row>
@@ -11027,7 +11460,7 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>121</v>
+        <v>130</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
@@ -11057,7 +11490,7 @@
         </is>
       </c>
       <c r="B8" s="4" t="n">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
@@ -11102,7 +11535,7 @@
         </is>
       </c>
       <c r="B11" s="10" t="n">
-        <v>163</v>
+        <v>170</v>
       </c>
       <c r="C11" s="6" t="inlineStr"/>
     </row>
@@ -11153,7 +11586,7 @@
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C16" s="6" t="inlineStr">
         <is>
@@ -11168,7 +11601,7 @@
         </is>
       </c>
       <c r="B17" s="4" t="n">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
@@ -11198,7 +11631,7 @@
         </is>
       </c>
       <c r="B19" s="10" t="n">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C19" s="6" t="inlineStr"/>
     </row>
@@ -11237,7 +11670,7 @@
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>unblocks the bulk of the 29 VIU-PENDING (QA) cases (cores, receiving, vendor, validation round-trips).</t>
+          <t>unblocks the bulk of the 27 VIU-PENDING (QA) cases (cores, receiving, vendor, validation round-trips).</t>
         </is>
       </c>
       <c r="C23" s="6" t="n"/>

</xml_diff>

<commit_message>
Simple Flow staging VIU: 4 Story-18 cases verified + TestRail push + deliverables/state
SF-CORE-03/04/11/18 flipped to VIU-Verified from live staging observation
(Story-18 Resolve-cores wizard + pre-resolve-cores API). TestRail 3 update_case
200 + re-GET MATCH (SF-CORE-04 no-op), run 325 untouched. Tally 134/20/22/5/3.
Deliverables + PROJECT-STATE + CLAUDE.md regenerated.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AZ5XzKsK9wv7M41cSPaMyg
</commit_message>
<xml_diff>
--- a/build/simple-flow/SimpleFlow_Blockers_Tracker.xlsx
+++ b/build/simple-flow/SimpleFlow_Blockers_Tracker.xlsx
@@ -3098,134 +3098,126 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="4" t="inlineStr">
+      <c r="A42" s="2" t="inlineStr">
         <is>
           <t>SF-CORE-03</t>
         </is>
       </c>
-      <c r="B42" s="4" t="inlineStr">
+      <c r="B42" s="2" t="inlineStr">
         <is>
           <t>Core parts — Completion modal</t>
         </is>
       </c>
-      <c r="C42" s="4" t="inlineStr">
+      <c r="C42" s="2" t="inlineStr">
         <is>
           <t>Verify a Resolve cores screen appears before the Receive parts / Complete without receiving choice and only an undecided core blocks completing</t>
         </is>
       </c>
-      <c r="D42" s="4" t="inlineStr">
-        <is>
-          <t>Blocked-Env</t>
-        </is>
-      </c>
-      <c r="E42" s="4" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
-        </is>
-      </c>
-      <c r="F42" s="4" t="inlineStr">
-        <is>
-          <t>VIU PENDING (QA)</t>
-        </is>
-      </c>
-      <c r="G42" s="4" t="inlineStr">
-        <is>
-          <t>QA (needs cookies+seed data)</t>
-        </is>
-      </c>
-      <c r="H42" s="4" t="inlineStr">
-        <is>
-          <t>QA VIU: seed a WO with core-charge parts, drive the completion Resolve-Cores modal + invoice-gate round-trip.</t>
-        </is>
-      </c>
-      <c r="I42" s="4" t="inlineStr">
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>VIU-Verified</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>READY (VIU-Verified)</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>None — VIU-verified; uploadable now.</t>
+        </is>
+      </c>
+      <c r="I42" s="2" t="inlineStr">
         <is>
           <t>S18 C-R1/C-R4</t>
         </is>
       </c>
-      <c r="J42" s="4" t="inlineStr">
-        <is>
-          <t>needs-data</t>
-        </is>
-      </c>
-      <c r="K42" s="4" t="inlineStr">
-        <is>
-          <t>spec `_4` Story 18 C-R1/C-R4 (resolve screen + gate-on-undecided) — needs the SV-8353 build + a dev-seeded special-order core.</t>
-        </is>
-      </c>
-      <c r="L42" s="4" t="inlineStr">
+      <c r="J42" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K42" s="2" t="inlineStr"/>
+      <c r="L42" s="2" t="inlineStr">
         <is>
           <t>C29315</t>
         </is>
       </c>
-      <c r="M42" s="4" t="inlineStr">
+      <c r="M42" s="2" t="inlineStr">
         <is>
           <t>https://shopview.testrail.io/index.php?/cases/view/29315</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="4" t="inlineStr">
+      <c r="A43" s="2" t="inlineStr">
         <is>
           <t>SF-CORE-04</t>
         </is>
       </c>
-      <c r="B43" s="4" t="inlineStr">
+      <c r="B43" s="2" t="inlineStr">
         <is>
           <t>Core parts — Invoice gate</t>
         </is>
       </c>
-      <c r="C43" s="4" t="inlineStr">
+      <c r="C43" s="2" t="inlineStr">
         <is>
           <t>Verify the 'Cores pending' indication reflects only undecided special-order cores (a decided core clears it)</t>
         </is>
       </c>
-      <c r="D43" s="4" t="inlineStr">
-        <is>
-          <t>Blocked-Env</t>
-        </is>
-      </c>
-      <c r="E43" s="4" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
-        </is>
-      </c>
-      <c r="F43" s="4" t="inlineStr">
-        <is>
-          <t>VIU PENDING (QA)</t>
-        </is>
-      </c>
-      <c r="G43" s="4" t="inlineStr">
-        <is>
-          <t>QA (needs cookies+seed data)</t>
-        </is>
-      </c>
-      <c r="H43" s="4" t="inlineStr">
-        <is>
-          <t>QA VIU: seed a WO with core-charge parts, drive the completion Resolve-Cores modal + invoice-gate round-trip.</t>
-        </is>
-      </c>
-      <c r="I43" s="4" t="inlineStr">
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>VIU-Verified</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>READY (VIU-Verified)</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H43" s="2" t="inlineStr">
+        <is>
+          <t>None — VIU-verified; uploadable now.</t>
+        </is>
+      </c>
+      <c r="I43" s="2" t="inlineStr">
         <is>
           <t>S18 C-R4</t>
         </is>
       </c>
-      <c r="J43" s="4" t="inlineStr">
-        <is>
-          <t>needs-data</t>
-        </is>
-      </c>
-      <c r="K43" s="4" t="inlineStr">
-        <is>
-          <t>spec `_4` Story 18 C-R4 ('Cores pending' = undecided-only) — needs the SV-8353 build + a dev-seeded core.</t>
-        </is>
-      </c>
-      <c r="L43" s="4" t="inlineStr">
+      <c r="J43" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K43" s="2" t="inlineStr"/>
+      <c r="L43" s="2" t="inlineStr">
         <is>
           <t>C29316</t>
         </is>
       </c>
-      <c r="M43" s="4" t="inlineStr">
+      <c r="M43" s="2" t="inlineStr">
         <is>
           <t>https://shopview.testrail.io/index.php?/cases/view/29316</t>
         </is>
@@ -3429,67 +3421,63 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="4" t="inlineStr">
+      <c r="A47" s="2" t="inlineStr">
         <is>
           <t>SF-CORE-11</t>
         </is>
       </c>
-      <c r="B47" s="4" t="inlineStr">
+      <c r="B47" s="2" t="inlineStr">
         <is>
           <t>Core parts — Pre-Resolve (Story 18)</t>
         </is>
       </c>
-      <c r="C47" s="4" t="inlineStr">
+      <c r="C47" s="2" t="inlineStr">
         <is>
           <t>Verify the Resolve cores screen lists every un-received vendor core with part info, core charge and OK / Not OK, plus an invoice-accuracy message</t>
         </is>
       </c>
-      <c r="D47" s="4" t="inlineStr">
-        <is>
-          <t>VIU-Pending</t>
-        </is>
-      </c>
-      <c r="E47" s="4" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
-        </is>
-      </c>
-      <c r="F47" s="4" t="inlineStr">
-        <is>
-          <t>VIU PENDING (QA)</t>
-        </is>
-      </c>
-      <c r="G47" s="4" t="inlineStr">
-        <is>
-          <t>QA (needs cookies+seed data)</t>
-        </is>
-      </c>
-      <c r="H47" s="4" t="inlineStr">
-        <is>
-          <t>QA VIU: seed a WO with core-charge parts, drive the completion Resolve-Cores modal + invoice-gate round-trip.</t>
-        </is>
-      </c>
-      <c r="I47" s="4" t="inlineStr">
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>VIU-Verified</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>READY (VIU-Verified)</t>
+        </is>
+      </c>
+      <c r="G47" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H47" s="2" t="inlineStr">
+        <is>
+          <t>None — VIU-verified; uploadable now.</t>
+        </is>
+      </c>
+      <c r="I47" s="2" t="inlineStr">
         <is>
           <t>S18 C-R1</t>
         </is>
       </c>
-      <c r="J47" s="4" t="inlineStr">
-        <is>
-          <t>needs-data</t>
-        </is>
-      </c>
-      <c r="K47" s="4" t="inlineStr">
-        <is>
-          <t>Story 18 C-R1 resolve screen — needs the SV-8353 build + a dev-seeded special-order core.</t>
-        </is>
-      </c>
-      <c r="L47" s="4" t="inlineStr">
+      <c r="J47" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K47" s="2" t="inlineStr"/>
+      <c r="L47" s="2" t="inlineStr">
         <is>
           <t>C29892</t>
         </is>
       </c>
-      <c r="M47" s="4" t="inlineStr">
+      <c r="M47" s="2" t="inlineStr">
         <is>
           <t>https://shopview.testrail.io/index.php?/cases/view/29892</t>
         </is>
@@ -3898,67 +3886,63 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="4" t="inlineStr">
+      <c r="A54" s="2" t="inlineStr">
         <is>
           <t>SF-CORE-18</t>
         </is>
       </c>
-      <c r="B54" s="4" t="inlineStr">
+      <c r="B54" s="2" t="inlineStr">
         <is>
           <t>API — Core Pre-Resolve (Story 18)</t>
         </is>
       </c>
-      <c r="C54" s="4" t="inlineStr">
+      <c r="C54" s="2" t="inlineStr">
         <is>
           <t>API: Verify POST /api/work-orders/{id}/pre-resolve-cores persists the core decision on the part request with no side-effect records</t>
         </is>
       </c>
-      <c r="D54" s="4" t="inlineStr">
-        <is>
-          <t>VIU-Pending</t>
-        </is>
-      </c>
-      <c r="E54" s="4" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
-        </is>
-      </c>
-      <c r="F54" s="4" t="inlineStr">
-        <is>
-          <t>VIU PENDING (QA)</t>
-        </is>
-      </c>
-      <c r="G54" s="4" t="inlineStr">
-        <is>
-          <t>QA (needs cookies+seed data)</t>
-        </is>
-      </c>
-      <c r="H54" s="4" t="inlineStr">
-        <is>
-          <t>QA VIU: seed a WO with core-charge parts, drive the completion Resolve-Cores modal + invoice-gate round-trip.</t>
-        </is>
-      </c>
-      <c r="I54" s="4" t="inlineStr">
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>VIU-Verified</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>READY (VIU-Verified)</t>
+        </is>
+      </c>
+      <c r="G54" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H54" s="2" t="inlineStr">
+        <is>
+          <t>None — VIU-verified; uploadable now.</t>
+        </is>
+      </c>
+      <c r="I54" s="2" t="inlineStr">
         <is>
           <t>S18 C-R2 / technical plan</t>
         </is>
       </c>
-      <c r="J54" s="4" t="inlineStr">
-        <is>
-          <t>needs-data</t>
-        </is>
-      </c>
-      <c r="K54" s="4" t="inlineStr">
-        <is>
-          <t>API POST /api/work-orders/{id}/pre-resolve-cores — endpoint from the SV-8353 tech plan; probe for existence first.</t>
-        </is>
-      </c>
-      <c r="L54" s="4" t="inlineStr">
+      <c r="J54" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K54" s="2" t="inlineStr"/>
+      <c r="L54" s="2" t="inlineStr">
         <is>
           <t>C29899</t>
         </is>
       </c>
-      <c r="M54" s="4" t="inlineStr">
+      <c r="M54" s="2" t="inlineStr">
         <is>
           <t>https://shopview.testrail.io/index.php?/cases/view/29899</t>
         </is>
@@ -12426,7 +12410,7 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
@@ -12456,7 +12440,7 @@
         </is>
       </c>
       <c r="B8" s="4" t="n">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
@@ -12567,7 +12551,7 @@
         </is>
       </c>
       <c r="B17" s="4" t="n">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="C17" s="7" t="inlineStr">
         <is>
@@ -12597,7 +12581,7 @@
         </is>
       </c>
       <c r="B19" s="10" t="n">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="C19" s="7" t="inlineStr"/>
     </row>
@@ -12636,7 +12620,7 @@
       </c>
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t>unblocks the bulk of the 46 VIU-PENDING (QA) cases (cores, receiving, vendor, validation round-trips).</t>
+          <t>unblocks the bulk of the 42 VIU-PENDING (QA) cases (cores, receiving, vendor, validation round-trips).</t>
         </is>
       </c>
       <c r="C23" s="7" t="n"/>

</xml_diff>

<commit_message>
Simple Flow staging VIU (resume): +14 cases verified (18 total) — receive/PO + Story-18 core flow
Verified: SF-INV-01/02/03, SF-BULK-06/10, SF-RCV-13, SF-VEND-08, SF-CORE-07/08/12/13/14/16, SF-REV-14.
Grouped Bulk Receive (Receive Selected), cost-editable-only-$0, core charge line follows
decision, receive auto-applies core decision, required-invoice resolve-first. TestRail status/
notes local (wording already build-accurate; run 325 untouched). Tally 148/10/18/5/3=184.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AZ5XzKsK9wv7M41cSPaMyg
</commit_message>
<xml_diff>
--- a/build/simple-flow/SimpleFlow_Blockers_Tracker.xlsx
+++ b/build/simple-flow/SimpleFlow_Blockers_Tracker.xlsx
@@ -3224,134 +3224,126 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="4" t="inlineStr">
+      <c r="A44" s="2" t="inlineStr">
         <is>
           <t>SF-CORE-07</t>
         </is>
       </c>
-      <c r="B44" s="4" t="inlineStr">
+      <c r="B44" s="2" t="inlineStr">
         <is>
           <t>Core parts — Required invoice (Story 4)</t>
         </is>
       </c>
-      <c r="C44" s="4" t="inlineStr">
+      <c r="C44" s="2" t="inlineStr">
         <is>
           <t>Verify the required-invoice flow asks to resolve special-order cores FIRST and then to receive them</t>
         </is>
       </c>
-      <c r="D44" s="4" t="inlineStr">
-        <is>
-          <t>Blocked-Env</t>
-        </is>
-      </c>
-      <c r="E44" s="4" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
-        </is>
-      </c>
-      <c r="F44" s="4" t="inlineStr">
-        <is>
-          <t>VIU PENDING (QA)</t>
-        </is>
-      </c>
-      <c r="G44" s="4" t="inlineStr">
-        <is>
-          <t>QA (needs cookies+seed data)</t>
-        </is>
-      </c>
-      <c r="H44" s="4" t="inlineStr">
-        <is>
-          <t>QA VIU: seed a WO with core-charge parts, drive the completion Resolve-Cores modal + invoice-gate round-trip.</t>
-        </is>
-      </c>
-      <c r="I44" s="4" t="inlineStr">
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>VIU-Verified</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>READY (VIU-Verified)</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H44" s="2" t="inlineStr">
+        <is>
+          <t>None — VIU-verified; uploadable now.</t>
+        </is>
+      </c>
+      <c r="I44" s="2" t="inlineStr">
         <is>
           <t>S18 C-R6</t>
         </is>
       </c>
-      <c r="J44" s="4" t="inlineStr">
-        <is>
-          <t>needs-data</t>
-        </is>
-      </c>
-      <c r="K44" s="4" t="inlineStr">
-        <is>
-          <t>spec `_4` Story 18 C-R6 (required flow: resolve FIRST then receive) — needs the SV-8353 build + a dev-seeded core.</t>
-        </is>
-      </c>
-      <c r="L44" s="4" t="inlineStr">
+      <c r="J44" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K44" s="2" t="inlineStr"/>
+      <c r="L44" s="2" t="inlineStr">
         <is>
           <t>C29319</t>
         </is>
       </c>
-      <c r="M44" s="4" t="inlineStr">
+      <c r="M44" s="2" t="inlineStr">
         <is>
           <t>https://shopview.testrail.io/index.php?/cases/view/29319</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="4" t="inlineStr">
+      <c r="A45" s="2" t="inlineStr">
         <is>
           <t>SF-CORE-08</t>
         </is>
       </c>
-      <c r="B45" s="4" t="inlineStr">
+      <c r="B45" s="2" t="inlineStr">
         <is>
           <t>Core parts — Guardrail</t>
         </is>
       </c>
-      <c r="C45" s="4" t="inlineStr">
+      <c r="C45" s="2" t="inlineStr">
         <is>
           <t>Verify the completion and invoice gates detect an undecided special-order core that exists only as a requested part</t>
         </is>
       </c>
-      <c r="D45" s="4" t="inlineStr">
-        <is>
-          <t>Blocked-Env</t>
-        </is>
-      </c>
-      <c r="E45" s="4" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
-        </is>
-      </c>
-      <c r="F45" s="4" t="inlineStr">
-        <is>
-          <t>VIU PENDING (QA)</t>
-        </is>
-      </c>
-      <c r="G45" s="4" t="inlineStr">
-        <is>
-          <t>QA (needs cookies+seed data)</t>
-        </is>
-      </c>
-      <c r="H45" s="4" t="inlineStr">
-        <is>
-          <t>QA VIU: seed a WO with core-charge parts, drive the completion Resolve-Cores modal + invoice-gate round-trip.</t>
-        </is>
-      </c>
-      <c r="I45" s="4" t="inlineStr">
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>VIU-Verified</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>READY (VIU-Verified)</t>
+        </is>
+      </c>
+      <c r="G45" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H45" s="2" t="inlineStr">
+        <is>
+          <t>None — VIU-verified; uploadable now.</t>
+        </is>
+      </c>
+      <c r="I45" s="2" t="inlineStr">
         <is>
           <t>S18 C-R2/C-R4 (guardrail)</t>
         </is>
       </c>
-      <c r="J45" s="4" t="inlineStr">
-        <is>
-          <t>needs-data</t>
-        </is>
-      </c>
-      <c r="K45" s="4" t="inlineStr">
-        <is>
-          <t>spec `_4` Story 18 C-R2/C-R4 (gate detects an undecided request-only core) — needs the SV-8353 build + a dev-seeded core.</t>
-        </is>
-      </c>
-      <c r="L45" s="4" t="inlineStr">
+      <c r="J45" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K45" s="2" t="inlineStr"/>
+      <c r="L45" s="2" t="inlineStr">
         <is>
           <t>C29320</t>
         </is>
       </c>
-      <c r="M45" s="4" t="inlineStr">
+      <c r="M45" s="2" t="inlineStr">
         <is>
           <t>https://shopview.testrail.io/index.php?/cases/view/29320</t>
         </is>
@@ -3484,201 +3476,189 @@
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="4" t="inlineStr">
+      <c r="A48" s="2" t="inlineStr">
         <is>
           <t>SF-CORE-12</t>
         </is>
       </c>
-      <c r="B48" s="4" t="inlineStr">
+      <c r="B48" s="2" t="inlineStr">
         <is>
           <t>Core parts — Pre-Resolve (Story 18)</t>
         </is>
       </c>
-      <c r="C48" s="4" t="inlineStr">
+      <c r="C48" s="2" t="inlineStr">
         <is>
           <t>Verify marking a core Not OK immediately adds the core charge to the work order total and customer invoice, while OK adds no charge</t>
         </is>
       </c>
-      <c r="D48" s="4" t="inlineStr">
-        <is>
-          <t>VIU-Pending</t>
-        </is>
-      </c>
-      <c r="E48" s="4" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
-        </is>
-      </c>
-      <c r="F48" s="4" t="inlineStr">
-        <is>
-          <t>VIU PENDING (QA)</t>
-        </is>
-      </c>
-      <c r="G48" s="4" t="inlineStr">
-        <is>
-          <t>QA (needs cookies+seed data)</t>
-        </is>
-      </c>
-      <c r="H48" s="4" t="inlineStr">
-        <is>
-          <t>QA VIU: seed a WO with core-charge parts, drive the completion Resolve-Cores modal + invoice-gate round-trip.</t>
-        </is>
-      </c>
-      <c r="I48" s="4" t="inlineStr">
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>VIU-Verified</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>READY (VIU-Verified)</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H48" s="2" t="inlineStr">
+        <is>
+          <t>None — VIU-verified; uploadable now.</t>
+        </is>
+      </c>
+      <c r="I48" s="2" t="inlineStr">
         <is>
           <t>S18 C-R3</t>
         </is>
       </c>
-      <c r="J48" s="4" t="inlineStr">
-        <is>
-          <t>needs-data</t>
-        </is>
-      </c>
-      <c r="K48" s="4" t="inlineStr">
-        <is>
-          <t>Story 18 C-R3 charge-follows-decision — needs the SV-8353 build + a dev-seeded special-order core.</t>
-        </is>
-      </c>
-      <c r="L48" s="4" t="inlineStr">
+      <c r="J48" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K48" s="2" t="inlineStr"/>
+      <c r="L48" s="2" t="inlineStr">
         <is>
           <t>C29893</t>
         </is>
       </c>
-      <c r="M48" s="4" t="inlineStr">
+      <c r="M48" s="2" t="inlineStr">
         <is>
           <t>https://shopview.testrail.io/index.php?/cases/view/29893</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="4" t="inlineStr">
+      <c r="A49" s="2" t="inlineStr">
         <is>
           <t>SF-CORE-13</t>
         </is>
       </c>
-      <c r="B49" s="4" t="inlineStr">
+      <c r="B49" s="2" t="inlineStr">
         <is>
           <t>Core parts — Pre-Resolve (Story 18)</t>
         </is>
       </c>
-      <c r="C49" s="4" t="inlineStr">
+      <c r="C49" s="2" t="inlineStr">
         <is>
           <t>Verify completion and invoice creation are blocked only while a core is undecided — a decided core does not block</t>
         </is>
       </c>
-      <c r="D49" s="4" t="inlineStr">
-        <is>
-          <t>VIU-Pending</t>
-        </is>
-      </c>
-      <c r="E49" s="4" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
-        </is>
-      </c>
-      <c r="F49" s="4" t="inlineStr">
-        <is>
-          <t>VIU PENDING (QA)</t>
-        </is>
-      </c>
-      <c r="G49" s="4" t="inlineStr">
-        <is>
-          <t>QA (needs cookies+seed data)</t>
-        </is>
-      </c>
-      <c r="H49" s="4" t="inlineStr">
-        <is>
-          <t>QA VIU: seed a WO with core-charge parts, drive the completion Resolve-Cores modal + invoice-gate round-trip.</t>
-        </is>
-      </c>
-      <c r="I49" s="4" t="inlineStr">
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>VIU-Verified</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>READY (VIU-Verified)</t>
+        </is>
+      </c>
+      <c r="G49" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H49" s="2" t="inlineStr">
+        <is>
+          <t>None — VIU-verified; uploadable now.</t>
+        </is>
+      </c>
+      <c r="I49" s="2" t="inlineStr">
         <is>
           <t>S18 C-R4</t>
         </is>
       </c>
-      <c r="J49" s="4" t="inlineStr">
-        <is>
-          <t>needs-data</t>
-        </is>
-      </c>
-      <c r="K49" s="4" t="inlineStr">
-        <is>
-          <t>Story 18 C-R4 gate-on-undecided — needs the SV-8353 build + a dev-seeded special-order core.</t>
-        </is>
-      </c>
-      <c r="L49" s="4" t="inlineStr">
+      <c r="J49" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K49" s="2" t="inlineStr"/>
+      <c r="L49" s="2" t="inlineStr">
         <is>
           <t>C29894</t>
         </is>
       </c>
-      <c r="M49" s="4" t="inlineStr">
+      <c r="M49" s="2" t="inlineStr">
         <is>
           <t>https://shopview.testrail.io/index.php?/cases/view/29894</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="4" t="inlineStr">
+      <c r="A50" s="2" t="inlineStr">
         <is>
           <t>SF-CORE-14</t>
         </is>
       </c>
-      <c r="B50" s="4" t="inlineStr">
+      <c r="B50" s="2" t="inlineStr">
         <is>
           <t>Core parts — Pre-Resolve (Story 18)</t>
         </is>
       </c>
-      <c r="C50" s="4" t="inlineStr">
+      <c r="C50" s="2" t="inlineStr">
         <is>
           <t>Verify receiving a pre-resolved core auto-applies the saved decision: OK creates exactly one vendor return, Not OK creates none, the invoice never changes, retries create no duplicates</t>
         </is>
       </c>
-      <c r="D50" s="4" t="inlineStr">
-        <is>
-          <t>VIU-Pending</t>
-        </is>
-      </c>
-      <c r="E50" s="4" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
-        </is>
-      </c>
-      <c r="F50" s="4" t="inlineStr">
-        <is>
-          <t>VIU PENDING (QA)</t>
-        </is>
-      </c>
-      <c r="G50" s="4" t="inlineStr">
-        <is>
-          <t>QA (needs cookies+seed data)</t>
-        </is>
-      </c>
-      <c r="H50" s="4" t="inlineStr">
-        <is>
-          <t>QA VIU: seed a WO with core-charge parts, drive the completion Resolve-Cores modal + invoice-gate round-trip.</t>
-        </is>
-      </c>
-      <c r="I50" s="4" t="inlineStr">
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>VIU-Verified</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>READY (VIU-Verified)</t>
+        </is>
+      </c>
+      <c r="G50" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H50" s="2" t="inlineStr">
+        <is>
+          <t>None — VIU-verified; uploadable now.</t>
+        </is>
+      </c>
+      <c r="I50" s="2" t="inlineStr">
         <is>
           <t>S18 C-R5</t>
         </is>
       </c>
-      <c r="J50" s="4" t="inlineStr">
-        <is>
-          <t>needs-data</t>
-        </is>
-      </c>
-      <c r="K50" s="4" t="inlineStr">
-        <is>
-          <t>Story 18 C-R5 auto-apply/idempotency — needs the SV-8353 build + a dev-seeded core + receive.</t>
-        </is>
-      </c>
-      <c r="L50" s="4" t="inlineStr">
+      <c r="J50" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K50" s="2" t="inlineStr"/>
+      <c r="L50" s="2" t="inlineStr">
         <is>
           <t>C29895</t>
         </is>
       </c>
-      <c r="M50" s="4" t="inlineStr">
+      <c r="M50" s="2" t="inlineStr">
         <is>
           <t>https://shopview.testrail.io/index.php?/cases/view/29895</t>
         </is>
@@ -3752,67 +3732,63 @@
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="4" t="inlineStr">
+      <c r="A52" s="2" t="inlineStr">
         <is>
           <t>SF-CORE-16</t>
         </is>
       </c>
-      <c r="B52" s="4" t="inlineStr">
+      <c r="B52" s="2" t="inlineStr">
         <is>
           <t>Core parts — Pre-Resolve (Story 18)</t>
         </is>
       </c>
-      <c r="C52" s="4" t="inlineStr">
+      <c r="C52" s="2" t="inlineStr">
         <is>
           <t>Verify the Lines tab shows the core decision state before and after receive: 'Core decision pending', 'Core OK — return to vendor, no charge', 'Core Not OK — customer charged'</t>
         </is>
       </c>
-      <c r="D52" s="4" t="inlineStr">
-        <is>
-          <t>VIU-Pending</t>
-        </is>
-      </c>
-      <c r="E52" s="4" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
-        </is>
-      </c>
-      <c r="F52" s="4" t="inlineStr">
-        <is>
-          <t>VIU PENDING (QA)</t>
-        </is>
-      </c>
-      <c r="G52" s="4" t="inlineStr">
-        <is>
-          <t>QA (needs cookies+seed data)</t>
-        </is>
-      </c>
-      <c r="H52" s="4" t="inlineStr">
-        <is>
-          <t>QA VIU: seed a WO with core-charge parts, drive the completion Resolve-Cores modal + invoice-gate round-trip.</t>
-        </is>
-      </c>
-      <c r="I52" s="4" t="inlineStr">
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>VIU-Verified</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>READY (VIU-Verified)</t>
+        </is>
+      </c>
+      <c r="G52" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H52" s="2" t="inlineStr">
+        <is>
+          <t>None — VIU-verified; uploadable now.</t>
+        </is>
+      </c>
+      <c r="I52" s="2" t="inlineStr">
         <is>
           <t>S18 C-R9</t>
         </is>
       </c>
-      <c r="J52" s="4" t="inlineStr">
-        <is>
-          <t>needs-data</t>
-        </is>
-      </c>
-      <c r="K52" s="4" t="inlineStr">
-        <is>
-          <t>Story 18 C-R9 Lines-tab states — needs the SV-8353 build + a dev-seeded core.</t>
-        </is>
-      </c>
-      <c r="L52" s="4" t="inlineStr">
+      <c r="J52" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K52" s="2" t="inlineStr"/>
+      <c r="L52" s="2" t="inlineStr">
         <is>
           <t>C29897</t>
         </is>
       </c>
-      <c r="M52" s="4" t="inlineStr">
+      <c r="M52" s="2" t="inlineStr">
         <is>
           <t>https://shopview.testrail.io/index.php?/cases/view/29897</t>
         </is>
@@ -6170,67 +6146,63 @@
       </c>
     </row>
     <row r="90">
-      <c r="A90" s="4" t="inlineStr">
+      <c r="A90" s="2" t="inlineStr">
         <is>
           <t>SF-BULK-06</t>
         </is>
       </c>
-      <c r="B90" s="4" t="inlineStr">
+      <c r="B90" s="2" t="inlineStr">
         <is>
           <t>PO Bulk Receive Page (Story 8)</t>
         </is>
       </c>
-      <c r="C90" s="4" t="inlineStr">
+      <c r="C90" s="2" t="inlineStr">
         <is>
           <t>Verify Bulk Receive field editability: quantity editable (partial receive), cost editable ONLY when it is $0, sell locks after the WO is invoiced/paid</t>
         </is>
       </c>
-      <c r="D90" s="4" t="inlineStr">
-        <is>
-          <t>VIU-Pending</t>
-        </is>
-      </c>
-      <c r="E90" s="4" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
-        </is>
-      </c>
-      <c r="F90" s="4" t="inlineStr">
-        <is>
-          <t>VIU PENDING (QA)</t>
-        </is>
-      </c>
-      <c r="G90" s="4" t="inlineStr">
-        <is>
-          <t>QA (needs cookies+seed data)</t>
-        </is>
-      </c>
-      <c r="H90" s="4" t="inlineStr">
-        <is>
-          <t>QA VIU: fresh sv7301 cookies + seeded data to drive this scenario.</t>
-        </is>
-      </c>
-      <c r="I90" s="4" t="inlineStr">
+      <c r="D90" s="2" t="inlineStr">
+        <is>
+          <t>VIU-Verified</t>
+        </is>
+      </c>
+      <c r="E90" s="2" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="F90" s="2" t="inlineStr">
+        <is>
+          <t>READY (VIU-Verified)</t>
+        </is>
+      </c>
+      <c r="G90" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H90" s="2" t="inlineStr">
+        <is>
+          <t>None — VIU-verified; uploadable now.</t>
+        </is>
+      </c>
+      <c r="I90" s="2" t="inlineStr">
         <is>
           <t>S8-R7 / S10-R3</t>
         </is>
       </c>
       <c r="J90" s="2" t="inlineStr">
         <is>
-          <t>reachable-now</t>
-        </is>
-      </c>
-      <c r="K90" s="4" t="inlineStr">
-        <is>
-          <t>Δ14 re-VIU: can a NON-ZERO cost be edited on Bulk Receive? ($0-only rule; if editable → deviation until dev ships).</t>
-        </is>
-      </c>
-      <c r="L90" s="4" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K90" s="2" t="inlineStr"/>
+      <c r="L90" s="2" t="inlineStr">
         <is>
           <t>C29355</t>
         </is>
       </c>
-      <c r="M90" s="4" t="inlineStr">
+      <c r="M90" s="2" t="inlineStr">
         <is>
           <t>https://shopview.testrail.io/index.php?/cases/view/29355</t>
         </is>
@@ -6426,67 +6398,63 @@
       </c>
     </row>
     <row r="94">
-      <c r="A94" s="4" t="inlineStr">
+      <c r="A94" s="2" t="inlineStr">
         <is>
           <t>SF-BULK-10</t>
         </is>
       </c>
-      <c r="B94" s="4" t="inlineStr">
+      <c r="B94" s="2" t="inlineStr">
         <is>
           <t>PO Bulk Receive Page (Story 8)</t>
         </is>
       </c>
-      <c r="C94" s="4" t="inlineStr">
+      <c r="C94" s="2" t="inlineStr">
         <is>
           <t>Verify a pre-resolved core's decision is applied automatically at receive with no re-prompt, and core-only partial receive is supported</t>
         </is>
       </c>
-      <c r="D94" s="4" t="inlineStr">
-        <is>
-          <t>Blocked-Env</t>
-        </is>
-      </c>
-      <c r="E94" s="4" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
-        </is>
-      </c>
-      <c r="F94" s="4" t="inlineStr">
-        <is>
-          <t>VIU PENDING (QA)</t>
-        </is>
-      </c>
-      <c r="G94" s="4" t="inlineStr">
-        <is>
-          <t>QA (needs cookies+seed data)</t>
-        </is>
-      </c>
-      <c r="H94" s="4" t="inlineStr">
-        <is>
-          <t>QA VIU: fresh sv7301 cookies + seeded data to drive this scenario.</t>
-        </is>
-      </c>
-      <c r="I94" s="4" t="inlineStr">
+      <c r="D94" s="2" t="inlineStr">
+        <is>
+          <t>VIU-Verified</t>
+        </is>
+      </c>
+      <c r="E94" s="2" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="F94" s="2" t="inlineStr">
+        <is>
+          <t>READY (VIU-Verified)</t>
+        </is>
+      </c>
+      <c r="G94" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H94" s="2" t="inlineStr">
+        <is>
+          <t>None — VIU-verified; uploadable now.</t>
+        </is>
+      </c>
+      <c r="I94" s="2" t="inlineStr">
         <is>
           <t>S18 C-R5</t>
         </is>
       </c>
-      <c r="J94" s="4" t="inlineStr">
-        <is>
-          <t>needs-data</t>
-        </is>
-      </c>
-      <c r="K94" s="4" t="inlineStr">
-        <is>
-          <t>spec `_4` Story 18 C-R5 (pre-resolved decision auto-applies at receive, no re-prompt) — needs the SV-8353 build + a dev-seeded core received on the bulk page.</t>
-        </is>
-      </c>
-      <c r="L94" s="4" t="inlineStr">
+      <c r="J94" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K94" s="2" t="inlineStr"/>
+      <c r="L94" s="2" t="inlineStr">
         <is>
           <t>C29359</t>
         </is>
       </c>
-      <c r="M94" s="4" t="inlineStr">
+      <c r="M94" s="2" t="inlineStr">
         <is>
           <t>https://shopview.testrail.io/index.php?/cases/view/29359</t>
         </is>
@@ -6560,201 +6528,189 @@
       </c>
     </row>
     <row r="96">
-      <c r="A96" s="4" t="inlineStr">
+      <c r="A96" s="2" t="inlineStr">
         <is>
           <t>SF-INV-01</t>
         </is>
       </c>
-      <c r="B96" s="4" t="inlineStr">
+      <c r="B96" s="2" t="inlineStr">
         <is>
           <t>Apply Invoice to Selected POs (Story 9)</t>
         </is>
       </c>
-      <c r="C96" s="4" t="inlineStr">
+      <c r="C96" s="2" t="inlineStr">
         <is>
           <t>Verify each vendor group has an invoice number field under the vendor name, available only when at least one PO of that vendor is selected (no Apply button)</t>
         </is>
       </c>
-      <c r="D96" s="4" t="inlineStr">
-        <is>
-          <t>VIU-Pending</t>
-        </is>
-      </c>
-      <c r="E96" s="4" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
-        </is>
-      </c>
-      <c r="F96" s="4" t="inlineStr">
-        <is>
-          <t>VIU PENDING (QA)</t>
-        </is>
-      </c>
-      <c r="G96" s="4" t="inlineStr">
-        <is>
-          <t>QA (needs cookies+seed data)</t>
-        </is>
-      </c>
-      <c r="H96" s="4" t="inlineStr">
-        <is>
-          <t>QA VIU: fresh sv7301 cookies + seeded data to drive this scenario.</t>
-        </is>
-      </c>
-      <c r="I96" s="4" t="inlineStr">
+      <c r="D96" s="2" t="inlineStr">
+        <is>
+          <t>VIU-Verified</t>
+        </is>
+      </c>
+      <c r="E96" s="2" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="F96" s="2" t="inlineStr">
+        <is>
+          <t>READY (VIU-Verified)</t>
+        </is>
+      </c>
+      <c r="G96" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H96" s="2" t="inlineStr">
+        <is>
+          <t>None — VIU-verified; uploadable now.</t>
+        </is>
+      </c>
+      <c r="I96" s="2" t="inlineStr">
         <is>
           <t>S9-R1</t>
         </is>
       </c>
       <c r="J96" s="2" t="inlineStr">
         <is>
-          <t>reachable-now</t>
-        </is>
-      </c>
-      <c r="K96" s="4" t="inlineStr">
-        <is>
-          <t>Δ13 re-VIU: is the 'Apply to selected POs' button still present? (2026-07-13 it WAS — likely build deviation until dev removes it).</t>
-        </is>
-      </c>
-      <c r="L96" s="4" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K96" s="2" t="inlineStr"/>
+      <c r="L96" s="2" t="inlineStr">
         <is>
           <t>C29360</t>
         </is>
       </c>
-      <c r="M96" s="4" t="inlineStr">
+      <c r="M96" s="2" t="inlineStr">
         <is>
           <t>https://shopview.testrail.io/index.php?/cases/view/29360</t>
         </is>
       </c>
     </row>
     <row r="97">
-      <c r="A97" s="4" t="inlineStr">
+      <c r="A97" s="2" t="inlineStr">
         <is>
           <t>SF-INV-02</t>
         </is>
       </c>
-      <c r="B97" s="4" t="inlineStr">
+      <c r="B97" s="2" t="inlineStr">
         <is>
           <t>Apply Invoice to Selected POs (Story 9)</t>
         </is>
       </c>
-      <c r="C97" s="4" t="inlineStr">
+      <c r="C97" s="2" t="inlineStr">
         <is>
           <t>Verify a typed invoice number fills only the selected POs of that vendor with no Apply click, still editable per PO</t>
         </is>
       </c>
-      <c r="D97" s="4" t="inlineStr">
-        <is>
-          <t>VIU-Pending</t>
-        </is>
-      </c>
-      <c r="E97" s="4" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
-        </is>
-      </c>
-      <c r="F97" s="4" t="inlineStr">
-        <is>
-          <t>VIU PENDING (QA)</t>
-        </is>
-      </c>
-      <c r="G97" s="4" t="inlineStr">
-        <is>
-          <t>QA (needs cookies+seed data)</t>
-        </is>
-      </c>
-      <c r="H97" s="4" t="inlineStr">
-        <is>
-          <t>QA VIU: fresh sv7301 cookies + seeded data to drive this scenario.</t>
-        </is>
-      </c>
-      <c r="I97" s="4" t="inlineStr">
+      <c r="D97" s="2" t="inlineStr">
+        <is>
+          <t>VIU-Verified</t>
+        </is>
+      </c>
+      <c r="E97" s="2" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="F97" s="2" t="inlineStr">
+        <is>
+          <t>READY (VIU-Verified)</t>
+        </is>
+      </c>
+      <c r="G97" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H97" s="2" t="inlineStr">
+        <is>
+          <t>None — VIU-verified; uploadable now.</t>
+        </is>
+      </c>
+      <c r="I97" s="2" t="inlineStr">
         <is>
           <t>S9-R2</t>
         </is>
       </c>
       <c r="J97" s="2" t="inlineStr">
         <is>
-          <t>reachable-now</t>
-        </is>
-      </c>
-      <c r="K97" s="4" t="inlineStr">
-        <is>
-          <t>Δ13 re-VIU: typed invoice # fills selected POs with no Apply click (old Apply-button behavior was live 2026-07-13).</t>
-        </is>
-      </c>
-      <c r="L97" s="4" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K97" s="2" t="inlineStr"/>
+      <c r="L97" s="2" t="inlineStr">
         <is>
           <t>C29361</t>
         </is>
       </c>
-      <c r="M97" s="4" t="inlineStr">
+      <c r="M97" s="2" t="inlineStr">
         <is>
           <t>https://shopview.testrail.io/index.php?/cases/view/29361</t>
         </is>
       </c>
     </row>
     <row r="98">
-      <c r="A98" s="4" t="inlineStr">
+      <c r="A98" s="2" t="inlineStr">
         <is>
           <t>SF-INV-03</t>
         </is>
       </c>
-      <c r="B98" s="4" t="inlineStr">
+      <c r="B98" s="2" t="inlineStr">
         <is>
           <t>Apply Invoice to Selected POs (Story 9)</t>
         </is>
       </c>
-      <c r="C98" s="4" t="inlineStr">
+      <c r="C98" s="2" t="inlineStr">
         <is>
           <t>Verify the vendor invoice number field is scoped per vendor, absent for the vendorless group, and allows a reused invoice number</t>
         </is>
       </c>
-      <c r="D98" s="4" t="inlineStr">
-        <is>
-          <t>VIU-Pending</t>
-        </is>
-      </c>
-      <c r="E98" s="4" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
-        </is>
-      </c>
-      <c r="F98" s="4" t="inlineStr">
-        <is>
-          <t>VIU PENDING (QA)</t>
-        </is>
-      </c>
-      <c r="G98" s="4" t="inlineStr">
-        <is>
-          <t>QA (needs cookies+seed data)</t>
-        </is>
-      </c>
-      <c r="H98" s="4" t="inlineStr">
-        <is>
-          <t>QA VIU: fresh sv7301 cookies + seeded data to drive this scenario.</t>
-        </is>
-      </c>
-      <c r="I98" s="4" t="inlineStr">
+      <c r="D98" s="2" t="inlineStr">
+        <is>
+          <t>VIU-Verified</t>
+        </is>
+      </c>
+      <c r="E98" s="2" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="F98" s="2" t="inlineStr">
+        <is>
+          <t>READY (VIU-Verified)</t>
+        </is>
+      </c>
+      <c r="G98" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H98" s="2" t="inlineStr">
+        <is>
+          <t>None — VIU-verified; uploadable now.</t>
+        </is>
+      </c>
+      <c r="I98" s="2" t="inlineStr">
         <is>
           <t>S9-R3</t>
         </is>
       </c>
       <c r="J98" s="2" t="inlineStr">
         <is>
-          <t>reachable-now</t>
-        </is>
-      </c>
-      <c r="K98" s="4" t="inlineStr">
-        <is>
-          <t>Δ13 re-VIU: per-vendor scoping + vendorless group shows NO invoice-number field.</t>
-        </is>
-      </c>
-      <c r="L98" s="4" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K98" s="2" t="inlineStr"/>
+      <c r="L98" s="2" t="inlineStr">
         <is>
           <t>C29362</t>
         </is>
       </c>
-      <c r="M98" s="4" t="inlineStr">
+      <c r="M98" s="2" t="inlineStr">
         <is>
           <t>https://shopview.testrail.io/index.php?/cases/view/29362</t>
         </is>
@@ -7911,67 +7867,63 @@
       </c>
     </row>
     <row r="117">
-      <c r="A117" s="4" t="inlineStr">
+      <c r="A117" s="2" t="inlineStr">
         <is>
           <t>SF-RCV-13</t>
         </is>
       </c>
-      <c r="B117" s="4" t="inlineStr">
+      <c r="B117" s="2" t="inlineStr">
         <is>
           <t>Accept Delivery (Story 12)</t>
         </is>
       </c>
-      <c r="C117" s="4" t="inlineStr">
+      <c r="C117" s="2" t="inlineStr">
         <is>
           <t>Verify a vendorless part can be assigned a vendor / merged into the single-part receive on the spot, reusing the same invoice number</t>
         </is>
       </c>
-      <c r="D117" s="4" t="inlineStr">
-        <is>
-          <t>VIU-Pending</t>
-        </is>
-      </c>
-      <c r="E117" s="4" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
-        </is>
-      </c>
-      <c r="F117" s="4" t="inlineStr">
-        <is>
-          <t>VIU PENDING (QA)</t>
-        </is>
-      </c>
-      <c r="G117" s="4" t="inlineStr">
-        <is>
-          <t>QA (needs cookies+seed data)</t>
-        </is>
-      </c>
-      <c r="H117" s="4" t="inlineStr">
-        <is>
-          <t>QA VIU: seed deliverable POs, drive the Receive / Accept-Delivery flow.</t>
-        </is>
-      </c>
-      <c r="I117" s="4" t="inlineStr">
+      <c r="D117" s="2" t="inlineStr">
+        <is>
+          <t>VIU-Verified</t>
+        </is>
+      </c>
+      <c r="E117" s="2" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="F117" s="2" t="inlineStr">
+        <is>
+          <t>READY (VIU-Verified)</t>
+        </is>
+      </c>
+      <c r="G117" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H117" s="2" t="inlineStr">
+        <is>
+          <t>None — VIU-verified; uploadable now.</t>
+        </is>
+      </c>
+      <c r="I117" s="2" t="inlineStr">
         <is>
           <t>S12-R6</t>
         </is>
       </c>
       <c r="J117" s="2" t="inlineStr">
         <is>
-          <t>reachable-now</t>
-        </is>
-      </c>
-      <c r="K117" s="4" t="inlineStr">
-        <is>
-          <t>S12-R6 assign/merge vendorless into the receive reusing the invoice # — seedable; may not be built yet.</t>
-        </is>
-      </c>
-      <c r="L117" s="4" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K117" s="2" t="inlineStr"/>
+      <c r="L117" s="2" t="inlineStr">
         <is>
           <t>C29903</t>
         </is>
       </c>
-      <c r="M117" s="4" t="inlineStr">
+      <c r="M117" s="2" t="inlineStr">
         <is>
           <t>https://shopview.testrail.io/index.php?/cases/view/29903</t>
         </is>
@@ -8435,67 +8387,63 @@
       </c>
     </row>
     <row r="125">
-      <c r="A125" s="4" t="inlineStr">
+      <c r="A125" s="2" t="inlineStr">
         <is>
           <t>SF-VEND-08</t>
         </is>
       </c>
-      <c r="B125" s="4" t="inlineStr">
+      <c r="B125" s="2" t="inlineStr">
         <is>
           <t>Assign Vendor + Merge (Story 13)</t>
         </is>
       </c>
-      <c r="C125" s="4" t="inlineStr">
+      <c r="C125" s="2" t="inlineStr">
         <is>
           <t>Verify the part number stays editable via the edit icon after entry until the part is received or the work order is invoiced/paid</t>
         </is>
       </c>
-      <c r="D125" s="4" t="inlineStr">
-        <is>
-          <t>VIU-Pending</t>
-        </is>
-      </c>
-      <c r="E125" s="4" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
-        </is>
-      </c>
-      <c r="F125" s="4" t="inlineStr">
-        <is>
-          <t>VIU PENDING (QA)</t>
-        </is>
-      </c>
-      <c r="G125" s="4" t="inlineStr">
-        <is>
-          <t>QA (needs cookies+seed data)</t>
-        </is>
-      </c>
-      <c r="H125" s="4" t="inlineStr">
-        <is>
-          <t>QA VIU: seed vendor-missing POs, drive Assign-Vendor + merge.</t>
-        </is>
-      </c>
-      <c r="I125" s="4" t="inlineStr">
+      <c r="D125" s="2" t="inlineStr">
+        <is>
+          <t>VIU-Verified</t>
+        </is>
+      </c>
+      <c r="E125" s="2" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="F125" s="2" t="inlineStr">
+        <is>
+          <t>READY (VIU-Verified)</t>
+        </is>
+      </c>
+      <c r="G125" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H125" s="2" t="inlineStr">
+        <is>
+          <t>None — VIU-verified; uploadable now.</t>
+        </is>
+      </c>
+      <c r="I125" s="2" t="inlineStr">
         <is>
           <t>S13-R8 (SV-8343)</t>
         </is>
       </c>
       <c r="J125" s="2" t="inlineStr">
         <is>
-          <t>reachable-now</t>
-        </is>
-      </c>
-      <c r="K125" s="4" t="inlineStr">
-        <is>
-          <t>S13-R8 part-number re-editable (edit icon) until received/invoiced-paid — seedable.</t>
-        </is>
-      </c>
-      <c r="L125" s="4" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K125" s="2" t="inlineStr"/>
+      <c r="L125" s="2" t="inlineStr">
         <is>
           <t>C29905</t>
         </is>
       </c>
-      <c r="M125" s="4" t="inlineStr">
+      <c r="M125" s="2" t="inlineStr">
         <is>
           <t>https://shopview.testrail.io/index.php?/cases/view/29905</t>
         </is>
@@ -9577,67 +9525,63 @@
       </c>
     </row>
     <row r="143">
-      <c r="A143" s="4" t="inlineStr">
+      <c r="A143" s="2" t="inlineStr">
         <is>
           <t>SF-REV-14</t>
         </is>
       </c>
-      <c r="B143" s="4" t="inlineStr">
+      <c r="B143" s="2" t="inlineStr">
         <is>
           <t>Review ON (Story 16)</t>
         </is>
       </c>
-      <c r="C143" s="4" t="inlineStr">
+      <c r="C143" s="2" t="inlineStr">
         <is>
           <t>Verify cores are decided before receiving ahead of Send to Review, and invoicing stays blocked until Reviewed and every core is decided</t>
         </is>
       </c>
-      <c r="D143" s="4" t="inlineStr">
-        <is>
-          <t>Blocked-Env</t>
-        </is>
-      </c>
-      <c r="E143" s="4" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
-        </is>
-      </c>
-      <c r="F143" s="4" t="inlineStr">
-        <is>
-          <t>VIU PENDING (QA)</t>
-        </is>
-      </c>
-      <c r="G143" s="4" t="inlineStr">
-        <is>
-          <t>QA (needs cookies+seed data)</t>
-        </is>
-      </c>
-      <c r="H143" s="4" t="inlineStr">
-        <is>
-          <t>QA VIU: enable Require Review and drive the review/sign-off round-trip.</t>
-        </is>
-      </c>
-      <c r="I143" s="4" t="inlineStr">
+      <c r="D143" s="2" t="inlineStr">
+        <is>
+          <t>VIU-Verified</t>
+        </is>
+      </c>
+      <c r="E143" s="2" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="F143" s="2" t="inlineStr">
+        <is>
+          <t>READY (VIU-Verified)</t>
+        </is>
+      </c>
+      <c r="G143" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H143" s="2" t="inlineStr">
+        <is>
+          <t>None — VIU-verified; uploadable now.</t>
+        </is>
+      </c>
+      <c r="I143" s="2" t="inlineStr">
         <is>
           <t>S18 / Story 16 core paragraph</t>
         </is>
       </c>
-      <c r="J143" s="4" t="inlineStr">
-        <is>
-          <t>needs-data</t>
-        </is>
-      </c>
-      <c r="K143" s="4" t="inlineStr">
-        <is>
-          <t>spec `_4` Story 18 (cores pre-resolved before receiving before Send To Review) — needs the SV-8353 build + a dev-seeded core.</t>
-        </is>
-      </c>
-      <c r="L143" s="4" t="inlineStr">
+      <c r="J143" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K143" s="2" t="inlineStr"/>
+      <c r="L143" s="2" t="inlineStr">
         <is>
           <t>C29399</t>
         </is>
       </c>
-      <c r="M143" s="4" t="inlineStr">
+      <c r="M143" s="2" t="inlineStr">
         <is>
           <t>https://shopview.testrail.io/index.php?/cases/view/29399</t>
         </is>
@@ -12410,7 +12354,7 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>130</v>
+        <v>144</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
@@ -12440,7 +12384,7 @@
         </is>
       </c>
       <c r="B8" s="4" t="n">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
@@ -12536,7 +12480,7 @@
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
@@ -12551,7 +12495,7 @@
         </is>
       </c>
       <c r="B17" s="4" t="n">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="C17" s="7" t="inlineStr">
         <is>
@@ -12581,7 +12525,7 @@
         </is>
       </c>
       <c r="B19" s="10" t="n">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="C19" s="7" t="inlineStr"/>
     </row>
@@ -12620,7 +12564,7 @@
       </c>
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t>unblocks the bulk of the 42 VIU-PENDING (QA) cases (cores, receiving, vendor, validation round-trips).</t>
+          <t>unblocks the bulk of the 28 VIU-PENDING (QA) cases (cores, receiving, vendor, validation round-trips).</t>
         </is>
       </c>
       <c r="C23" s="7" t="n"/>

</xml_diff>

<commit_message>
Simple Flow staging VIU (resume 2): SF-RCV-05/07 deviation confirmed + part-sale/vendor-change verified
Priority: SF-RCV-05/07 DEFINITIVELY re-confirmed Deviation (Accept-Delivery Vendor Missing still
TOP; bug #5 stays open). +3 Verified: SF-VEND-07 (parts-tab vendor changeable), SF-POSEL-07 +
SF-BULK-11 (part-sale PO type2 P-1110 in PO list + on Bulk Receive). SF-CORE-15/17 + SF-QB-09
-> Blocked-Env (fully characterized). Tally 151/4/21/5/3=184. Settings restored, seeds deleted.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AZ5XzKsK9wv7M41cSPaMyg
</commit_message>
<xml_diff>
--- a/build/simple-flow/SimpleFlow_Blockers_Tracker.xlsx
+++ b/build/simple-flow/SimpleFlow_Blockers_Tracker.xlsx
@@ -3682,7 +3682,7 @@
       </c>
       <c r="D51" s="4" t="inlineStr">
         <is>
-          <t>VIU-Pending</t>
+          <t>Blocked-Env</t>
         </is>
       </c>
       <c r="E51" s="4" t="inlineStr">
@@ -3812,7 +3812,7 @@
       </c>
       <c r="D53" s="4" t="inlineStr">
         <is>
-          <t>VIU-Pending</t>
+          <t>Blocked-Env</t>
         </is>
       </c>
       <c r="E53" s="4" t="inlineStr">
@@ -5764,67 +5764,63 @@
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="4" t="inlineStr">
+      <c r="A84" s="2" t="inlineStr">
         <is>
           <t>SF-POSEL-07</t>
         </is>
       </c>
-      <c r="B84" s="4" t="inlineStr">
+      <c r="B84" s="2" t="inlineStr">
         <is>
           <t>PO Multi-Select (Story 7)</t>
         </is>
       </c>
-      <c r="C84" s="4" t="inlineStr">
+      <c r="C84" s="2" t="inlineStr">
         <is>
           <t>Verify part-sale-originated POs appear in the PO list and are selectable like work-order POs</t>
         </is>
       </c>
-      <c r="D84" s="4" t="inlineStr">
-        <is>
-          <t>VIU-Pending</t>
-        </is>
-      </c>
-      <c r="E84" s="4" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
-        </is>
-      </c>
-      <c r="F84" s="4" t="inlineStr">
-        <is>
-          <t>VIU PENDING (QA)</t>
-        </is>
-      </c>
-      <c r="G84" s="4" t="inlineStr">
-        <is>
-          <t>QA (needs cookies+seed data)</t>
-        </is>
-      </c>
-      <c r="H84" s="4" t="inlineStr">
-        <is>
-          <t>QA VIU: fresh sv7301 cookies + seeded data to drive this scenario.</t>
-        </is>
-      </c>
-      <c r="I84" s="4" t="inlineStr">
+      <c r="D84" s="2" t="inlineStr">
+        <is>
+          <t>VIU-Verified</t>
+        </is>
+      </c>
+      <c r="E84" s="2" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="F84" s="2" t="inlineStr">
+        <is>
+          <t>READY (VIU-Verified)</t>
+        </is>
+      </c>
+      <c r="G84" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H84" s="2" t="inlineStr">
+        <is>
+          <t>None — VIU-verified; uploadable now.</t>
+        </is>
+      </c>
+      <c r="I84" s="2" t="inlineStr">
         <is>
           <t>S7 AC (part-sale POs) + §8 Part Sales — confirmed</t>
         </is>
       </c>
       <c r="J84" s="2" t="inlineStr">
         <is>
-          <t>reachable-now</t>
-        </is>
-      </c>
-      <c r="K84" s="4" t="inlineStr">
-        <is>
-          <t>Δ15 part-sale PO on the PO list + multi-select — seed a Part Sale with a vendor part (Rule 14).</t>
-        </is>
-      </c>
-      <c r="L84" s="4" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K84" s="2" t="inlineStr"/>
+      <c r="L84" s="2" t="inlineStr">
         <is>
           <t>C29906</t>
         </is>
       </c>
-      <c r="M84" s="4" t="inlineStr">
+      <c r="M84" s="2" t="inlineStr">
         <is>
           <t>https://shopview.testrail.io/index.php?/cases/view/29906</t>
         </is>
@@ -6461,67 +6457,63 @@
       </c>
     </row>
     <row r="95">
-      <c r="A95" s="4" t="inlineStr">
+      <c r="A95" s="2" t="inlineStr">
         <is>
           <t>SF-BULK-11</t>
         </is>
       </c>
-      <c r="B95" s="4" t="inlineStr">
+      <c r="B95" s="2" t="inlineStr">
         <is>
           <t>PO Bulk Receive Page (Story 8)</t>
         </is>
       </c>
-      <c r="C95" s="4" t="inlineStr">
+      <c r="C95" s="2" t="inlineStr">
         <is>
           <t>Verify a part-sale-originated PO can be received on the Bulk Receive page like a work-order PO</t>
         </is>
       </c>
-      <c r="D95" s="4" t="inlineStr">
-        <is>
-          <t>VIU-Pending</t>
-        </is>
-      </c>
-      <c r="E95" s="4" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
-        </is>
-      </c>
-      <c r="F95" s="4" t="inlineStr">
-        <is>
-          <t>VIU PENDING (QA)</t>
-        </is>
-      </c>
-      <c r="G95" s="4" t="inlineStr">
-        <is>
-          <t>QA (needs cookies+seed data)</t>
-        </is>
-      </c>
-      <c r="H95" s="4" t="inlineStr">
-        <is>
-          <t>QA VIU: fresh sv7301 cookies + seeded data to drive this scenario.</t>
-        </is>
-      </c>
-      <c r="I95" s="4" t="inlineStr">
+      <c r="D95" s="2" t="inlineStr">
+        <is>
+          <t>VIU-Verified</t>
+        </is>
+      </c>
+      <c r="E95" s="2" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="F95" s="2" t="inlineStr">
+        <is>
+          <t>READY (VIU-Verified)</t>
+        </is>
+      </c>
+      <c r="G95" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H95" s="2" t="inlineStr">
+        <is>
+          <t>None — VIU-verified; uploadable now.</t>
+        </is>
+      </c>
+      <c r="I95" s="2" t="inlineStr">
         <is>
           <t>S8 AC (part-sale POs) + §8 Part Sales — confirmed</t>
         </is>
       </c>
       <c r="J95" s="2" t="inlineStr">
         <is>
-          <t>reachable-now</t>
-        </is>
-      </c>
-      <c r="K95" s="4" t="inlineStr">
-        <is>
-          <t>Δ15 part-sale PO receivable on Bulk Receive — seed a Part Sale with a vendor part.</t>
-        </is>
-      </c>
-      <c r="L95" s="4" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K95" s="2" t="inlineStr"/>
+      <c r="L95" s="2" t="inlineStr">
         <is>
           <t>C29907</t>
         </is>
       </c>
-      <c r="M95" s="4" t="inlineStr">
+      <c r="M95" s="2" t="inlineStr">
         <is>
           <t>https://shopview.testrail.io/index.php?/cases/view/29907</t>
         </is>
@@ -8320,67 +8312,63 @@
       </c>
     </row>
     <row r="124">
-      <c r="A124" s="4" t="inlineStr">
+      <c r="A124" s="2" t="inlineStr">
         <is>
           <t>SF-VEND-07</t>
         </is>
       </c>
-      <c r="B124" s="4" t="inlineStr">
+      <c r="B124" s="2" t="inlineStr">
         <is>
           <t>Assign Vendor + Merge (Story 13)</t>
         </is>
       </c>
-      <c r="C124" s="4" t="inlineStr">
+      <c r="C124" s="2" t="inlineStr">
         <is>
           <t>Verify an assigned vendor stays changeable via the same dropdown until the part is received or the work order is invoiced/paid</t>
         </is>
       </c>
-      <c r="D124" s="4" t="inlineStr">
-        <is>
-          <t>VIU-Pending</t>
-        </is>
-      </c>
-      <c r="E124" s="4" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
-        </is>
-      </c>
-      <c r="F124" s="4" t="inlineStr">
-        <is>
-          <t>VIU PENDING (QA)</t>
-        </is>
-      </c>
-      <c r="G124" s="4" t="inlineStr">
-        <is>
-          <t>QA (needs cookies+seed data)</t>
-        </is>
-      </c>
-      <c r="H124" s="4" t="inlineStr">
-        <is>
-          <t>QA VIU: seed vendor-missing POs, drive Assign-Vendor + merge.</t>
-        </is>
-      </c>
-      <c r="I124" s="4" t="inlineStr">
+      <c r="D124" s="2" t="inlineStr">
+        <is>
+          <t>VIU-Verified</t>
+        </is>
+      </c>
+      <c r="E124" s="2" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="F124" s="2" t="inlineStr">
+        <is>
+          <t>READY (VIU-Verified)</t>
+        </is>
+      </c>
+      <c r="G124" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H124" s="2" t="inlineStr">
+        <is>
+          <t>None — VIU-verified; uploadable now.</t>
+        </is>
+      </c>
+      <c r="I124" s="2" t="inlineStr">
         <is>
           <t>S13-R8 (SV-8343)</t>
         </is>
       </c>
       <c r="J124" s="2" t="inlineStr">
         <is>
-          <t>reachable-now</t>
-        </is>
-      </c>
-      <c r="K124" s="4" t="inlineStr">
-        <is>
-          <t>S13-R8 vendor re-changeable until received/invoiced-paid — seedable (invoiced/paid leg may stay env-blocked).</t>
-        </is>
-      </c>
-      <c r="L124" s="4" t="inlineStr">
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K124" s="2" t="inlineStr"/>
+      <c r="L124" s="2" t="inlineStr">
         <is>
           <t>C29904</t>
         </is>
       </c>
-      <c r="M124" s="4" t="inlineStr">
+      <c r="M124" s="2" t="inlineStr">
         <is>
           <t>https://shopview.testrail.io/index.php?/cases/view/29904</t>
         </is>
@@ -11783,7 +11771,7 @@
       </c>
       <c r="D178" s="4" t="inlineStr">
         <is>
-          <t>VIU-Pending</t>
+          <t>Blocked-Env</t>
         </is>
       </c>
       <c r="E178" s="4" t="inlineStr">
@@ -12354,7 +12342,7 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
@@ -12384,7 +12372,7 @@
         </is>
       </c>
       <c r="B8" s="4" t="n">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
@@ -12480,7 +12468,7 @@
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
@@ -12525,7 +12513,7 @@
         </is>
       </c>
       <c r="B19" s="10" t="n">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="C19" s="7" t="inlineStr"/>
     </row>
@@ -12564,7 +12552,7 @@
       </c>
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t>unblocks the bulk of the 28 VIU-PENDING (QA) cases (cores, receiving, vendor, validation round-trips).</t>
+          <t>unblocks the bulk of the 25 VIU-PENDING (QA) cases (cores, receiving, vendor, validation round-trips).</t>
         </is>
       </c>
       <c r="C23" s="7" t="n"/>

</xml_diff>

<commit_message>
Simple Flow: author SF-PERM-11/12 corrective cases (SV-8515/8516) + tighten SF-PERM-03; SV-8541 held
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AZ5XzKsK9wv7M41cSPaMyg
</commit_message>
<xml_diff>
--- a/build/simple-flow/SimpleFlow_Blockers_Tracker.xlsx
+++ b/build/simple-flow/SimpleFlow_Blockers_Tracker.xlsx
@@ -492,7 +492,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M185"/>
+  <dimension ref="A1:M187"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -10525,139 +10525,119 @@
       </c>
     </row>
     <row r="159">
-      <c r="A159" s="2" t="inlineStr">
-        <is>
-          <t>SF-VAL-01</t>
-        </is>
-      </c>
-      <c r="B159" s="2" t="inlineStr">
-        <is>
-          <t>Validation / Edge</t>
-        </is>
-      </c>
-      <c r="C159" s="2" t="inlineStr">
-        <is>
-          <t>Verify completion is blocked when required mileage is missing</t>
-        </is>
-      </c>
-      <c r="D159" s="2" t="inlineStr">
-        <is>
-          <t>VIU-Verified</t>
-        </is>
-      </c>
-      <c r="E159" s="2" t="inlineStr">
-        <is>
-          <t>READY</t>
-        </is>
-      </c>
-      <c r="F159" s="2" t="inlineStr">
-        <is>
-          <t>READY (VIU-Verified)</t>
-        </is>
-      </c>
-      <c r="G159" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H159" s="2" t="inlineStr">
-        <is>
-          <t>None — VIU-verified; uploadable now.</t>
-        </is>
-      </c>
-      <c r="I159" s="2" t="inlineStr">
-        <is>
-          <t>S2-R2 / S3-R3 / S4-R3</t>
-        </is>
-      </c>
-      <c r="J159" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K159" s="2" t="inlineStr"/>
-      <c r="L159" s="2" t="inlineStr">
-        <is>
-          <t>C29415</t>
-        </is>
-      </c>
-      <c r="M159" s="2" t="inlineStr">
-        <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29415</t>
-        </is>
-      </c>
+      <c r="A159" s="5" t="inlineStr">
+        <is>
+          <t>SF-PERM-11</t>
+        </is>
+      </c>
+      <c r="B159" s="5" t="inlineStr">
+        <is>
+          <t>Permissions</t>
+        </is>
+      </c>
+      <c r="C159" s="5" t="inlineStr">
+        <is>
+          <t>Verify a Vendor &amp; Order Management View-only user cannot receive purchase orders by any path on the Bulk Receive screen</t>
+        </is>
+      </c>
+      <c r="D159" s="5" t="inlineStr">
+        <is>
+          <t>VIU-Deviation</t>
+        </is>
+      </c>
+      <c r="E159" s="5" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="F159" s="5" t="inlineStr">
+        <is>
+          <t>BUG/RULING</t>
+        </is>
+      </c>
+      <c r="G159" s="5" t="inlineStr">
+        <is>
+          <t>Dev / PO ruling</t>
+        </is>
+      </c>
+      <c r="H159" s="5" t="inlineStr">
+        <is>
+          <t>Dev fix (SV-8515, Ready-to-Fix): a Vendor &amp; Order Mgmt View-only (Office) user has the per-PO Receive button correctly hidden, but the multi-select 'Receive Selected' route currently EXPOSES the editable /bulk-receive screen (FE-exposure defect). Backend blocks the actual receive (accept -&gt; 403), so no data bypass. FE route guard should require Vendor &amp; Order Mgmt: Create &amp; Edit to reach Bulk Receive.</t>
+        </is>
+      </c>
+      <c r="I159" s="5" t="inlineStr">
+        <is>
+          <t>§9.1 Bulk Receive gate / §9.2 Office footnote-4</t>
+        </is>
+      </c>
+      <c r="J159" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K159" s="5" t="inlineStr"/>
+      <c r="L159" s="5" t="inlineStr"/>
+      <c r="M159" s="5" t="inlineStr"/>
     </row>
     <row r="160">
-      <c r="A160" s="4" t="inlineStr">
-        <is>
-          <t>SF-VAL-02</t>
-        </is>
-      </c>
-      <c r="B160" s="4" t="inlineStr">
-        <is>
-          <t>Validation / Edge</t>
-        </is>
-      </c>
-      <c r="C160" s="4" t="inlineStr">
-        <is>
-          <t>Verify completion is blocked when a required VIN is missing (non-review No-PO / Optional-invoice flow)</t>
-        </is>
-      </c>
-      <c r="D160" s="4" t="inlineStr">
-        <is>
-          <t>Blocked-Env</t>
-        </is>
-      </c>
-      <c r="E160" s="4" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
-        </is>
-      </c>
-      <c r="F160" s="4" t="inlineStr">
-        <is>
-          <t>VIU PENDING (QA)</t>
-        </is>
-      </c>
-      <c r="G160" s="4" t="inlineStr">
-        <is>
-          <t>QA (needs cookies+seed data)</t>
-        </is>
-      </c>
-      <c r="H160" s="4" t="inlineStr">
-        <is>
-          <t>QA VIU: drive the specific validation/edge scenario with seeded data.</t>
-        </is>
-      </c>
-      <c r="I160" s="4" t="inlineStr">
-        <is>
-          <t>S15-R2 / S3-R3 / S4-R3</t>
-        </is>
-      </c>
-      <c r="J160" s="4" t="inlineStr">
-        <is>
-          <t>needs-data</t>
-        </is>
-      </c>
-      <c r="K160" s="4" t="inlineStr">
-        <is>
-          <t>an asset/vehicle with NO VIN so the non-review wizard prompts for VIN. BATCH 6: VIN prefills from the asset; the asset-creation flow (VIN likely required) was not reliably drivable in-harness. Needs a VIN-less asset seeded.</t>
-        </is>
-      </c>
-      <c r="L160" s="4" t="inlineStr">
-        <is>
-          <t>C29416</t>
-        </is>
-      </c>
-      <c r="M160" s="4" t="inlineStr">
-        <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29416</t>
-        </is>
-      </c>
+      <c r="A160" s="2" t="inlineStr">
+        <is>
+          <t>SF-PERM-12</t>
+        </is>
+      </c>
+      <c r="B160" s="2" t="inlineStr">
+        <is>
+          <t>Permissions</t>
+        </is>
+      </c>
+      <c r="C160" s="2" t="inlineStr">
+        <is>
+          <t>Verify a no-access role (Time Clock) cannot edit, cancel or change the vendor of a work order part from the part menu</t>
+        </is>
+      </c>
+      <c r="D160" s="2" t="inlineStr">
+        <is>
+          <t>VIU-Verified</t>
+        </is>
+      </c>
+      <c r="E160" s="2" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="F160" s="2" t="inlineStr">
+        <is>
+          <t>READY (VIU-Verified)</t>
+        </is>
+      </c>
+      <c r="G160" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H160" s="2" t="inlineStr">
+        <is>
+          <t>None — VIU-verified; uploadable now.</t>
+        </is>
+      </c>
+      <c r="I160" s="2" t="inlineStr">
+        <is>
+          <t>§9.2 Time Clock part-actions</t>
+        </is>
+      </c>
+      <c r="J160" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K160" s="2" t="inlineStr"/>
+      <c r="L160" s="2" t="inlineStr"/>
+      <c r="M160" s="2" t="inlineStr"/>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
         <is>
-          <t>SF-VAL-03</t>
+          <t>SF-VAL-01</t>
         </is>
       </c>
       <c r="B161" s="2" t="inlineStr">
@@ -10667,7 +10647,7 @@
       </c>
       <c r="C161" s="2" t="inlineStr">
         <is>
-          <t>Verify completion is blocked when required engine hours are missing</t>
+          <t>Verify completion is blocked when required mileage is missing</t>
         </is>
       </c>
       <c r="D161" s="2" t="inlineStr">
@@ -10697,7 +10677,7 @@
       </c>
       <c r="I161" s="2" t="inlineStr">
         <is>
-          <t>S3-R3 / S4-R3</t>
+          <t>S2-R2 / S3-R3 / S4-R3</t>
         </is>
       </c>
       <c r="J161" s="2" t="inlineStr">
@@ -10708,82 +10688,86 @@
       <c r="K161" s="2" t="inlineStr"/>
       <c r="L161" s="2" t="inlineStr">
         <is>
-          <t>C29417</t>
+          <t>C29415</t>
         </is>
       </c>
       <c r="M161" s="2" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29417</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29415</t>
         </is>
       </c>
     </row>
     <row r="162">
-      <c r="A162" s="2" t="inlineStr">
-        <is>
-          <t>SF-VAL-04</t>
-        </is>
-      </c>
-      <c r="B162" s="2" t="inlineStr">
+      <c r="A162" s="4" t="inlineStr">
+        <is>
+          <t>SF-VAL-02</t>
+        </is>
+      </c>
+      <c r="B162" s="4" t="inlineStr">
         <is>
           <t>Validation / Edge</t>
         </is>
       </c>
-      <c r="C162" s="2" t="inlineStr">
-        <is>
-          <t>Verify the tech-story Next/Continue button stays disabled while the story textarea is empty</t>
-        </is>
-      </c>
-      <c r="D162" s="2" t="inlineStr">
-        <is>
-          <t>VIU-Verified</t>
-        </is>
-      </c>
-      <c r="E162" s="2" t="inlineStr">
-        <is>
-          <t>READY</t>
-        </is>
-      </c>
-      <c r="F162" s="2" t="inlineStr">
-        <is>
-          <t>READY (VIU-Verified)</t>
-        </is>
-      </c>
-      <c r="G162" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H162" s="2" t="inlineStr">
-        <is>
-          <t>None — VIU-verified; uploadable now.</t>
-        </is>
-      </c>
-      <c r="I162" s="2" t="inlineStr">
-        <is>
-          <t>TS-R4</t>
-        </is>
-      </c>
-      <c r="J162" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K162" s="2" t="inlineStr"/>
-      <c r="L162" s="2" t="inlineStr">
-        <is>
-          <t>C29418</t>
-        </is>
-      </c>
-      <c r="M162" s="2" t="inlineStr">
-        <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29418</t>
+      <c r="C162" s="4" t="inlineStr">
+        <is>
+          <t>Verify completion is blocked when a required VIN is missing (non-review No-PO / Optional-invoice flow)</t>
+        </is>
+      </c>
+      <c r="D162" s="4" t="inlineStr">
+        <is>
+          <t>Blocked-Env</t>
+        </is>
+      </c>
+      <c r="E162" s="4" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="F162" s="4" t="inlineStr">
+        <is>
+          <t>VIU PENDING (QA)</t>
+        </is>
+      </c>
+      <c r="G162" s="4" t="inlineStr">
+        <is>
+          <t>QA (needs cookies+seed data)</t>
+        </is>
+      </c>
+      <c r="H162" s="4" t="inlineStr">
+        <is>
+          <t>QA VIU: drive the specific validation/edge scenario with seeded data.</t>
+        </is>
+      </c>
+      <c r="I162" s="4" t="inlineStr">
+        <is>
+          <t>S15-R2 / S3-R3 / S4-R3</t>
+        </is>
+      </c>
+      <c r="J162" s="4" t="inlineStr">
+        <is>
+          <t>needs-data</t>
+        </is>
+      </c>
+      <c r="K162" s="4" t="inlineStr">
+        <is>
+          <t>an asset/vehicle with NO VIN so the non-review wizard prompts for VIN. BATCH 6: VIN prefills from the asset; the asset-creation flow (VIN likely required) was not reliably drivable in-harness. Needs a VIN-less asset seeded.</t>
+        </is>
+      </c>
+      <c r="L162" s="4" t="inlineStr">
+        <is>
+          <t>C29416</t>
+        </is>
+      </c>
+      <c r="M162" s="4" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29416</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
         <is>
-          <t>SF-VAL-05</t>
+          <t>SF-VAL-03</t>
         </is>
       </c>
       <c r="B163" s="2" t="inlineStr">
@@ -10793,7 +10777,7 @@
       </c>
       <c r="C163" s="2" t="inlineStr">
         <is>
-          <t>Verify a required-invoice receive is blocked without a vendor invoice number</t>
+          <t>Verify completion is blocked when required engine hours are missing</t>
         </is>
       </c>
       <c r="D163" s="2" t="inlineStr">
@@ -10823,7 +10807,7 @@
       </c>
       <c r="I163" s="2" t="inlineStr">
         <is>
-          <t>S3-R3 / S4-R5 / §4</t>
+          <t>S3-R3 / S4-R3</t>
         </is>
       </c>
       <c r="J163" s="2" t="inlineStr">
@@ -10834,19 +10818,19 @@
       <c r="K163" s="2" t="inlineStr"/>
       <c r="L163" s="2" t="inlineStr">
         <is>
-          <t>C29419</t>
+          <t>C29417</t>
         </is>
       </c>
       <c r="M163" s="2" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29419</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29417</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
         <is>
-          <t>SF-VAL-06</t>
+          <t>SF-VAL-04</t>
         </is>
       </c>
       <c r="B164" s="2" t="inlineStr">
@@ -10856,7 +10840,7 @@
       </c>
       <c r="C164" s="2" t="inlineStr">
         <is>
-          <t>Verify a vendor-missing part cannot be received without a vendor, a part number, and a cost / sell price</t>
+          <t>Verify the tech-story Next/Continue button stays disabled while the story textarea is empty</t>
         </is>
       </c>
       <c r="D164" s="2" t="inlineStr">
@@ -10886,7 +10870,7 @@
       </c>
       <c r="I164" s="2" t="inlineStr">
         <is>
-          <t>S10 / S12-R2 / S13-R6 / S13-R7</t>
+          <t>TS-R4</t>
         </is>
       </c>
       <c r="J164" s="2" t="inlineStr">
@@ -10897,19 +10881,19 @@
       <c r="K164" s="2" t="inlineStr"/>
       <c r="L164" s="2" t="inlineStr">
         <is>
-          <t>C29420</t>
+          <t>C29418</t>
         </is>
       </c>
       <c r="M164" s="2" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29420</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29418</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
         <is>
-          <t>SF-VAL-07</t>
+          <t>SF-VAL-05</t>
         </is>
       </c>
       <c r="B165" s="2" t="inlineStr">
@@ -10919,7 +10903,7 @@
       </c>
       <c r="C165" s="2" t="inlineStr">
         <is>
-          <t>Verify Confirm Review is disabled until a VIN is entered in the Mark Reviewed dialog</t>
+          <t>Verify a required-invoice receive is blocked without a vendor invoice number</t>
         </is>
       </c>
       <c r="D165" s="2" t="inlineStr">
@@ -10949,7 +10933,7 @@
       </c>
       <c r="I165" s="2" t="inlineStr">
         <is>
-          <t>R7</t>
+          <t>S3-R3 / S4-R5 / §4</t>
         </is>
       </c>
       <c r="J165" s="2" t="inlineStr">
@@ -10960,19 +10944,19 @@
       <c r="K165" s="2" t="inlineStr"/>
       <c r="L165" s="2" t="inlineStr">
         <is>
-          <t>C29421</t>
+          <t>C29419</t>
         </is>
       </c>
       <c r="M165" s="2" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29421</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29419</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" s="2" t="inlineStr">
         <is>
-          <t>SF-VAL-08</t>
+          <t>SF-VAL-06</t>
         </is>
       </c>
       <c r="B166" s="2" t="inlineStr">
@@ -10982,7 +10966,7 @@
       </c>
       <c r="C166" s="2" t="inlineStr">
         <is>
-          <t>Verify re-completing after cancelling does not create duplicate POs</t>
+          <t>Verify a vendor-missing part cannot be received without a vendor, a part number, and a cost / sell price</t>
         </is>
       </c>
       <c r="D166" s="2" t="inlineStr">
@@ -11012,7 +10996,7 @@
       </c>
       <c r="I166" s="2" t="inlineStr">
         <is>
-          <t>S3-R9 (idempotency)</t>
+          <t>S10 / S12-R2 / S13-R6 / S13-R7</t>
         </is>
       </c>
       <c r="J166" s="2" t="inlineStr">
@@ -11023,86 +11007,82 @@
       <c r="K166" s="2" t="inlineStr"/>
       <c r="L166" s="2" t="inlineStr">
         <is>
-          <t>C29422</t>
+          <t>C29420</t>
         </is>
       </c>
       <c r="M166" s="2" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29422</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29420</t>
         </is>
       </c>
     </row>
     <row r="167">
-      <c r="A167" s="4" t="inlineStr">
-        <is>
-          <t>SF-VAL-09</t>
-        </is>
-      </c>
-      <c r="B167" s="4" t="inlineStr">
+      <c r="A167" s="2" t="inlineStr">
+        <is>
+          <t>SF-VAL-07</t>
+        </is>
+      </c>
+      <c r="B167" s="2" t="inlineStr">
         <is>
           <t>Validation / Edge</t>
         </is>
       </c>
-      <c r="C167" s="4" t="inlineStr">
-        <is>
-          <t>Verify the sell field is locked after the work order is invoiced/paid with a lock icon and tooltip</t>
-        </is>
-      </c>
-      <c r="D167" s="4" t="inlineStr">
-        <is>
-          <t>Blocked-Env</t>
-        </is>
-      </c>
-      <c r="E167" s="4" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
-        </is>
-      </c>
-      <c r="F167" s="4" t="inlineStr">
-        <is>
-          <t>VIU PENDING (QA)</t>
-        </is>
-      </c>
-      <c r="G167" s="4" t="inlineStr">
-        <is>
-          <t>QA (needs cookies+seed data)</t>
-        </is>
-      </c>
-      <c r="H167" s="4" t="inlineStr">
-        <is>
-          <t>QA VIU: drive the specific validation/edge scenario with seeded data.</t>
-        </is>
-      </c>
-      <c r="I167" s="4" t="inlineStr">
-        <is>
-          <t>S8-R7 / §4 field locking</t>
-        </is>
-      </c>
-      <c r="J167" s="4" t="inlineStr">
-        <is>
-          <t>needs-data</t>
-        </is>
-      </c>
-      <c r="K167" s="4" t="inlineStr">
-        <is>
-          <t>RE-VIU 2026-07-09: Bulk Receive field-locking BUILT (qty/cost/sell editable verified); the sell-lock-after-invoiced/paid clause needs an invoiced/paid WO to drive.</t>
-        </is>
-      </c>
-      <c r="L167" s="4" t="inlineStr">
-        <is>
-          <t>C29423</t>
-        </is>
-      </c>
-      <c r="M167" s="4" t="inlineStr">
-        <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29423</t>
+      <c r="C167" s="2" t="inlineStr">
+        <is>
+          <t>Verify Confirm Review is disabled until a VIN is entered in the Mark Reviewed dialog</t>
+        </is>
+      </c>
+      <c r="D167" s="2" t="inlineStr">
+        <is>
+          <t>VIU-Verified</t>
+        </is>
+      </c>
+      <c r="E167" s="2" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="F167" s="2" t="inlineStr">
+        <is>
+          <t>READY (VIU-Verified)</t>
+        </is>
+      </c>
+      <c r="G167" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H167" s="2" t="inlineStr">
+        <is>
+          <t>None — VIU-verified; uploadable now.</t>
+        </is>
+      </c>
+      <c r="I167" s="2" t="inlineStr">
+        <is>
+          <t>R7</t>
+        </is>
+      </c>
+      <c r="J167" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K167" s="2" t="inlineStr"/>
+      <c r="L167" s="2" t="inlineStr">
+        <is>
+          <t>C29421</t>
+        </is>
+      </c>
+      <c r="M167" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29421</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" s="2" t="inlineStr">
         <is>
-          <t>SF-VAL-10</t>
+          <t>SF-VAL-08</t>
         </is>
       </c>
       <c r="B168" s="2" t="inlineStr">
@@ -11112,7 +11092,7 @@
       </c>
       <c r="C168" s="2" t="inlineStr">
         <is>
-          <t>Verify the same vendor invoice number can be reused across POs (uniqueness relaxed)</t>
+          <t>Verify re-completing after cancelling does not create duplicate POs</t>
         </is>
       </c>
       <c r="D168" s="2" t="inlineStr">
@@ -11142,7 +11122,7 @@
       </c>
       <c r="I168" s="2" t="inlineStr">
         <is>
-          <t>S9-R3 / §4 (uniqueness relaxed)</t>
+          <t>S3-R9 (idempotency)</t>
         </is>
       </c>
       <c r="J168" s="2" t="inlineStr">
@@ -11153,212 +11133,212 @@
       <c r="K168" s="2" t="inlineStr"/>
       <c r="L168" s="2" t="inlineStr">
         <is>
+          <t>C29422</t>
+        </is>
+      </c>
+      <c r="M168" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29422</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="4" t="inlineStr">
+        <is>
+          <t>SF-VAL-09</t>
+        </is>
+      </c>
+      <c r="B169" s="4" t="inlineStr">
+        <is>
+          <t>Validation / Edge</t>
+        </is>
+      </c>
+      <c r="C169" s="4" t="inlineStr">
+        <is>
+          <t>Verify the sell field is locked after the work order is invoiced/paid with a lock icon and tooltip</t>
+        </is>
+      </c>
+      <c r="D169" s="4" t="inlineStr">
+        <is>
+          <t>Blocked-Env</t>
+        </is>
+      </c>
+      <c r="E169" s="4" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="F169" s="4" t="inlineStr">
+        <is>
+          <t>VIU PENDING (QA)</t>
+        </is>
+      </c>
+      <c r="G169" s="4" t="inlineStr">
+        <is>
+          <t>QA (needs cookies+seed data)</t>
+        </is>
+      </c>
+      <c r="H169" s="4" t="inlineStr">
+        <is>
+          <t>QA VIU: drive the specific validation/edge scenario with seeded data.</t>
+        </is>
+      </c>
+      <c r="I169" s="4" t="inlineStr">
+        <is>
+          <t>S8-R7 / §4 field locking</t>
+        </is>
+      </c>
+      <c r="J169" s="4" t="inlineStr">
+        <is>
+          <t>needs-data</t>
+        </is>
+      </c>
+      <c r="K169" s="4" t="inlineStr">
+        <is>
+          <t>RE-VIU 2026-07-09: Bulk Receive field-locking BUILT (qty/cost/sell editable verified); the sell-lock-after-invoiced/paid clause needs an invoiced/paid WO to drive.</t>
+        </is>
+      </c>
+      <c r="L169" s="4" t="inlineStr">
+        <is>
+          <t>C29423</t>
+        </is>
+      </c>
+      <c r="M169" s="4" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29423</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="2" t="inlineStr">
+        <is>
+          <t>SF-VAL-10</t>
+        </is>
+      </c>
+      <c r="B170" s="2" t="inlineStr">
+        <is>
+          <t>Validation / Edge</t>
+        </is>
+      </c>
+      <c r="C170" s="2" t="inlineStr">
+        <is>
+          <t>Verify the same vendor invoice number can be reused across POs (uniqueness relaxed)</t>
+        </is>
+      </c>
+      <c r="D170" s="2" t="inlineStr">
+        <is>
+          <t>VIU-Verified</t>
+        </is>
+      </c>
+      <c r="E170" s="2" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="F170" s="2" t="inlineStr">
+        <is>
+          <t>READY (VIU-Verified)</t>
+        </is>
+      </c>
+      <c r="G170" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H170" s="2" t="inlineStr">
+        <is>
+          <t>None — VIU-verified; uploadable now.</t>
+        </is>
+      </c>
+      <c r="I170" s="2" t="inlineStr">
+        <is>
+          <t>S9-R3 / §4 (uniqueness relaxed)</t>
+        </is>
+      </c>
+      <c r="J170" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K170" s="2" t="inlineStr"/>
+      <c r="L170" s="2" t="inlineStr">
+        <is>
           <t>C29424</t>
         </is>
       </c>
-      <c r="M168" s="2" t="inlineStr">
+      <c r="M170" s="2" t="inlineStr">
         <is>
           <t>https://shopview.testrail.io/index.php?/cases/view/29424</t>
         </is>
       </c>
     </row>
-    <row r="169">
-      <c r="A169" s="2" t="inlineStr">
+    <row r="171">
+      <c r="A171" s="2" t="inlineStr">
         <is>
           <t>SF-VAL-11</t>
         </is>
       </c>
-      <c r="B169" s="2" t="inlineStr">
+      <c r="B171" s="2" t="inlineStr">
         <is>
           <t>Validation / Edge</t>
         </is>
       </c>
-      <c r="C169" s="2" t="inlineStr">
+      <c r="C171" s="2" t="inlineStr">
         <is>
           <t>Verify an unapproved line disables the Complete Work Order button with a tooltip (regardless of the Require Vendor Invoice Number setting)</t>
         </is>
       </c>
-      <c r="D169" s="2" t="inlineStr">
-        <is>
-          <t>VIU-Verified</t>
-        </is>
-      </c>
-      <c r="E169" s="2" t="inlineStr">
-        <is>
-          <t>READY</t>
-        </is>
-      </c>
-      <c r="F169" s="2" t="inlineStr">
-        <is>
-          <t>READY (VIU-Verified)</t>
-        </is>
-      </c>
-      <c r="G169" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H169" s="2" t="inlineStr">
-        <is>
-          <t>None — VIU-verified; uploadable now.</t>
-        </is>
-      </c>
-      <c r="I169" s="2" t="inlineStr">
+      <c r="D171" s="2" t="inlineStr">
+        <is>
+          <t>VIU-Verified</t>
+        </is>
+      </c>
+      <c r="E171" s="2" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="F171" s="2" t="inlineStr">
+        <is>
+          <t>READY (VIU-Verified)</t>
+        </is>
+      </c>
+      <c r="G171" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H171" s="2" t="inlineStr">
+        <is>
+          <t>None — VIU-verified; uploadable now.</t>
+        </is>
+      </c>
+      <c r="I171" s="2" t="inlineStr">
         <is>
           <t>S4-R8 / S3-R9 / Key Decision (line approval)</t>
         </is>
       </c>
-      <c r="J169" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K169" s="2" t="inlineStr"/>
-      <c r="L169" s="2" t="inlineStr">
+      <c r="J171" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K171" s="2" t="inlineStr"/>
+      <c r="L171" s="2" t="inlineStr">
         <is>
           <t>C29425</t>
         </is>
       </c>
-      <c r="M169" s="2" t="inlineStr">
+      <c r="M171" s="2" t="inlineStr">
         <is>
           <t>https://shopview.testrail.io/index.php?/cases/view/29425</t>
-        </is>
-      </c>
-    </row>
-    <row r="170">
-      <c r="A170" s="4" t="inlineStr">
-        <is>
-          <t>SF-QB-01</t>
-        </is>
-      </c>
-      <c r="B170" s="4" t="inlineStr">
-        <is>
-          <t>QuickBooks / Inventory Integrity</t>
-        </is>
-      </c>
-      <c r="C170" s="4" t="inlineStr">
-        <is>
-          <t>Verify in-stock parts decrement inventory and write Part History on simple completion (skip path still runs lifecycle)</t>
-        </is>
-      </c>
-      <c r="D170" s="4" t="inlineStr">
-        <is>
-          <t>Blocked-Env</t>
-        </is>
-      </c>
-      <c r="E170" s="4" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
-        </is>
-      </c>
-      <c r="F170" s="4" t="inlineStr">
-        <is>
-          <t>VIU PENDING (QA)</t>
-        </is>
-      </c>
-      <c r="G170" s="4" t="inlineStr">
-        <is>
-          <t>QA (needs cookies+seed data)</t>
-        </is>
-      </c>
-      <c r="H170" s="4" t="inlineStr">
-        <is>
-          <t>QA VIU: complete a WO end-to-end and inspect the QuickBooks / inventory side-effects (Journal Entry, Part History, inventory decrement).</t>
-        </is>
-      </c>
-      <c r="I170" s="4" t="inlineStr">
-        <is>
-          <t>§5 invariant 1</t>
-        </is>
-      </c>
-      <c r="J170" s="4" t="inlineStr">
-        <is>
-          <t>needs-data</t>
-        </is>
-      </c>
-      <c r="K170" s="4" t="inlineStr">
-        <is>
-          <t>FRESH VIU 2026-07-10: decrement half PROVEN (P550848 on-hand 6-&gt;5 on pick, persisted through simple-complete 201). Part-History LOG surface BLOCKED-ENV: GET /api/inventory/parts/history -&gt; 500; /parts/inventory/{id} detail page crashes ('page is totaled'); other history endpoints 404/405 (see bugs-log OBS-6). QuickBooks-integrity leg needs QB access.</t>
-        </is>
-      </c>
-      <c r="L170" s="4" t="inlineStr">
-        <is>
-          <t>C29426</t>
-        </is>
-      </c>
-      <c r="M170" s="4" t="inlineStr">
-        <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29426</t>
-        </is>
-      </c>
-    </row>
-    <row r="171">
-      <c r="A171" s="3" t="inlineStr">
-        <is>
-          <t>SF-QB-02</t>
-        </is>
-      </c>
-      <c r="B171" s="3" t="inlineStr">
-        <is>
-          <t>QuickBooks / Inventory Integrity</t>
-        </is>
-      </c>
-      <c r="C171" s="3" t="inlineStr">
-        <is>
-          <t>Verify Create POs OFF produces no PO, vendor bill or AP sync and no catalog/inventory sync</t>
-        </is>
-      </c>
-      <c r="D171" s="3" t="inlineStr">
-        <is>
-          <t>VIU-observed-awaiting-Milos</t>
-        </is>
-      </c>
-      <c r="E171" s="3" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
-        </is>
-      </c>
-      <c r="F171" s="3" t="inlineStr">
-        <is>
-          <t>MILOS ANSWER</t>
-        </is>
-      </c>
-      <c r="G171" s="3" t="inlineStr">
-        <is>
-          <t>Milos (Product Owner)</t>
-        </is>
-      </c>
-      <c r="H171" s="3" t="inlineStr">
-        <is>
-          <t>Milos answers Open Question Q5 — QuickBooks integrity when Create-POs is OFF (toggle absent).</t>
-        </is>
-      </c>
-      <c r="I171" s="3" t="inlineStr">
-        <is>
-          <t>Q5 | §5 / §4 (Create POs OFF)</t>
-        </is>
-      </c>
-      <c r="J171" s="3" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K171" s="3" t="inlineStr"/>
-      <c r="L171" s="3" t="inlineStr">
-        <is>
-          <t>C29427</t>
-        </is>
-      </c>
-      <c r="M171" s="3" t="inlineStr">
-        <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29427</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" s="4" t="inlineStr">
         <is>
-          <t>SF-QB-03</t>
+          <t>SF-QB-01</t>
         </is>
       </c>
       <c r="B172" s="4" t="inlineStr">
@@ -11368,7 +11348,7 @@
       </c>
       <c r="C172" s="4" t="inlineStr">
         <is>
-          <t>Verify POs ON plus receiving runs the full pipeline: receive → Delivery → Vendor Bill → QuickBooks (both surfaces sync)</t>
+          <t>Verify in-stock parts decrement inventory and write Part History on simple completion (skip path still runs lifecycle)</t>
         </is>
       </c>
       <c r="D172" s="4" t="inlineStr">
@@ -11398,7 +11378,7 @@
       </c>
       <c r="I172" s="4" t="inlineStr">
         <is>
-          <t>§5 invariant 2</t>
+          <t>§5 invariant 1</t>
         </is>
       </c>
       <c r="J172" s="4" t="inlineStr">
@@ -11408,91 +11388,87 @@
       </c>
       <c r="K172" s="4" t="inlineStr">
         <is>
-          <t>QuickBooks / inventory back-end inspection (receive -&gt; Delivery -&gt; Vendor Bill -&gt; QBO) — likely needs dev/QB access.</t>
+          <t>FRESH VIU 2026-07-10: decrement half PROVEN (P550848 on-hand 6-&gt;5 on pick, persisted through simple-complete 201). Part-History LOG surface BLOCKED-ENV: GET /api/inventory/parts/history -&gt; 500; /parts/inventory/{id} detail page crashes ('page is totaled'); other history endpoints 404/405 (see bugs-log OBS-6). QuickBooks-integrity leg needs QB access.</t>
         </is>
       </c>
       <c r="L172" s="4" t="inlineStr">
         <is>
-          <t>C29428</t>
+          <t>C29426</t>
         </is>
       </c>
       <c r="M172" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29428</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29426</t>
         </is>
       </c>
     </row>
     <row r="173">
-      <c r="A173" s="4" t="inlineStr">
-        <is>
-          <t>SF-QB-04</t>
-        </is>
-      </c>
-      <c r="B173" s="4" t="inlineStr">
+      <c r="A173" s="3" t="inlineStr">
+        <is>
+          <t>SF-QB-02</t>
+        </is>
+      </c>
+      <c r="B173" s="3" t="inlineStr">
         <is>
           <t>QuickBooks / Inventory Integrity</t>
         </is>
       </c>
-      <c r="C173" s="4" t="inlineStr">
-        <is>
-          <t>Verify a vendorless / no-PN part has zero inventory interaction until a vendor and/or part number is added</t>
-        </is>
-      </c>
-      <c r="D173" s="4" t="inlineStr">
-        <is>
-          <t>Blocked-Env</t>
-        </is>
-      </c>
-      <c r="E173" s="4" t="inlineStr">
+      <c r="C173" s="3" t="inlineStr">
+        <is>
+          <t>Verify Create POs OFF produces no PO, vendor bill or AP sync and no catalog/inventory sync</t>
+        </is>
+      </c>
+      <c r="D173" s="3" t="inlineStr">
+        <is>
+          <t>VIU-observed-awaiting-Milos</t>
+        </is>
+      </c>
+      <c r="E173" s="3" t="inlineStr">
         <is>
           <t>BLOCKED</t>
         </is>
       </c>
-      <c r="F173" s="4" t="inlineStr">
-        <is>
-          <t>VIU PENDING (QA)</t>
-        </is>
-      </c>
-      <c r="G173" s="4" t="inlineStr">
-        <is>
-          <t>QA (needs cookies+seed data)</t>
-        </is>
-      </c>
-      <c r="H173" s="4" t="inlineStr">
-        <is>
-          <t>QA VIU: complete a WO end-to-end and inspect the QuickBooks / inventory side-effects (Journal Entry, Part History, inventory decrement).</t>
-        </is>
-      </c>
-      <c r="I173" s="4" t="inlineStr">
-        <is>
-          <t>§5 (vendorless/no-PN)</t>
-        </is>
-      </c>
-      <c r="J173" s="4" t="inlineStr">
-        <is>
-          <t>needs-data</t>
-        </is>
-      </c>
-      <c r="K173" s="4" t="inlineStr">
-        <is>
-          <t>QuickBooks / inventory inspection (vendorless/no-PN part = zero inventory interaction) — likely needs dev/QB access.</t>
-        </is>
-      </c>
-      <c r="L173" s="4" t="inlineStr">
-        <is>
-          <t>C29429</t>
-        </is>
-      </c>
-      <c r="M173" s="4" t="inlineStr">
-        <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29429</t>
+      <c r="F173" s="3" t="inlineStr">
+        <is>
+          <t>MILOS ANSWER</t>
+        </is>
+      </c>
+      <c r="G173" s="3" t="inlineStr">
+        <is>
+          <t>Milos (Product Owner)</t>
+        </is>
+      </c>
+      <c r="H173" s="3" t="inlineStr">
+        <is>
+          <t>Milos answers Open Question Q5 — QuickBooks integrity when Create-POs is OFF (toggle absent).</t>
+        </is>
+      </c>
+      <c r="I173" s="3" t="inlineStr">
+        <is>
+          <t>Q5 | §5 / §4 (Create POs OFF)</t>
+        </is>
+      </c>
+      <c r="J173" s="3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K173" s="3" t="inlineStr"/>
+      <c r="L173" s="3" t="inlineStr">
+        <is>
+          <t>C29427</t>
+        </is>
+      </c>
+      <c r="M173" s="3" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29427</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" s="4" t="inlineStr">
         <is>
-          <t>SF-QB-05</t>
+          <t>SF-QB-03</t>
         </is>
       </c>
       <c r="B174" s="4" t="inlineStr">
@@ -11502,7 +11478,7 @@
       </c>
       <c r="C174" s="4" t="inlineStr">
         <is>
-          <t>Verify Vendor Missing POs are excluded from QuickBooks until a vendor and part number are provided</t>
+          <t>Verify POs ON plus receiving runs the full pipeline: receive → Delivery → Vendor Bill → QuickBooks (both surfaces sync)</t>
         </is>
       </c>
       <c r="D174" s="4" t="inlineStr">
@@ -11532,7 +11508,7 @@
       </c>
       <c r="I174" s="4" t="inlineStr">
         <is>
-          <t>§5 / S6-R3</t>
+          <t>§5 invariant 2</t>
         </is>
       </c>
       <c r="J174" s="4" t="inlineStr">
@@ -11542,24 +11518,24 @@
       </c>
       <c r="K174" s="4" t="inlineStr">
         <is>
-          <t>QuickBooks inspection (Vendor-Missing POs excluded from QB until vendor + PN) — likely needs dev/QB access.</t>
+          <t>QuickBooks / inventory back-end inspection (receive -&gt; Delivery -&gt; Vendor Bill -&gt; QBO) — likely needs dev/QB access.</t>
         </is>
       </c>
       <c r="L174" s="4" t="inlineStr">
         <is>
-          <t>C29430</t>
+          <t>C29428</t>
         </is>
       </c>
       <c r="M174" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29430</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29428</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" s="4" t="inlineStr">
         <is>
-          <t>SF-QB-06</t>
+          <t>SF-QB-04</t>
         </is>
       </c>
       <c r="B175" s="4" t="inlineStr">
@@ -11569,7 +11545,7 @@
       </c>
       <c r="C175" s="4" t="inlineStr">
         <is>
-          <t>Verify cost at completion behavior to avoid $0-cost margins in QuickBooks</t>
+          <t>Verify a vendorless / no-PN part has zero inventory interaction until a vendor and/or part number is added</t>
         </is>
       </c>
       <c r="D175" s="4" t="inlineStr">
@@ -11599,7 +11575,7 @@
       </c>
       <c r="I175" s="4" t="inlineStr">
         <is>
-          <t>§8 (cost at completion)</t>
+          <t>§5 (vendorless/no-PN)</t>
         </is>
       </c>
       <c r="J175" s="4" t="inlineStr">
@@ -11609,24 +11585,24 @@
       </c>
       <c r="K175" s="4" t="inlineStr">
         <is>
-          <t>QuickBooks inspection (cost-at-completion to avoid $0-cost margins) — likely needs dev/QB access.</t>
+          <t>QuickBooks / inventory inspection (vendorless/no-PN part = zero inventory interaction) — likely needs dev/QB access.</t>
         </is>
       </c>
       <c r="L175" s="4" t="inlineStr">
         <is>
-          <t>C29431</t>
+          <t>C29429</t>
         </is>
       </c>
       <c r="M175" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29431</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29429</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" s="4" t="inlineStr">
         <is>
-          <t>SF-QB-07</t>
+          <t>SF-QB-05</t>
         </is>
       </c>
       <c r="B176" s="4" t="inlineStr">
@@ -11636,7 +11612,7 @@
       </c>
       <c r="C176" s="4" t="inlineStr">
         <is>
-          <t>Verify the Journal Entry / Inventory sync to QuickBooks fires on invoice creation (not PO-dependent)</t>
+          <t>Verify Vendor Missing POs are excluded from QuickBooks until a vendor and part number are provided</t>
         </is>
       </c>
       <c r="D176" s="4" t="inlineStr">
@@ -11666,7 +11642,7 @@
       </c>
       <c r="I176" s="4" t="inlineStr">
         <is>
-          <t>§5 (Journal Entry / Inventory → QBO)</t>
+          <t>§5 / S6-R3</t>
         </is>
       </c>
       <c r="J176" s="4" t="inlineStr">
@@ -11676,87 +11652,91 @@
       </c>
       <c r="K176" s="4" t="inlineStr">
         <is>
-          <t>QuickBooks inspection (Journal Entry / Inventory sync fires on invoice creation) — likely needs dev/QB access.</t>
+          <t>QuickBooks inspection (Vendor-Missing POs excluded from QB until vendor + PN) — likely needs dev/QB access.</t>
         </is>
       </c>
       <c r="L176" s="4" t="inlineStr">
         <is>
-          <t>C29432</t>
+          <t>C29430</t>
         </is>
       </c>
       <c r="M176" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29432</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29430</t>
         </is>
       </c>
     </row>
     <row r="177">
-      <c r="A177" s="2" t="inlineStr">
-        <is>
-          <t>SF-QB-08</t>
-        </is>
-      </c>
-      <c r="B177" s="2" t="inlineStr">
+      <c r="A177" s="4" t="inlineStr">
+        <is>
+          <t>SF-QB-06</t>
+        </is>
+      </c>
+      <c r="B177" s="4" t="inlineStr">
         <is>
           <t>QuickBooks / Inventory Integrity</t>
         </is>
       </c>
-      <c r="C177" s="2" t="inlineStr">
-        <is>
-          <t>Verify Part History is preserved for a part that is genuinely inventory-tracked</t>
-        </is>
-      </c>
-      <c r="D177" s="2" t="inlineStr">
-        <is>
-          <t>VIU-Verified</t>
-        </is>
-      </c>
-      <c r="E177" s="2" t="inlineStr">
-        <is>
-          <t>READY</t>
-        </is>
-      </c>
-      <c r="F177" s="2" t="inlineStr">
-        <is>
-          <t>READY (VIU-Verified)</t>
-        </is>
-      </c>
-      <c r="G177" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H177" s="2" t="inlineStr">
-        <is>
-          <t>None — VIU-verified; uploadable now.</t>
-        </is>
-      </c>
-      <c r="I177" s="2" t="inlineStr">
-        <is>
-          <t>§5 invariant 3 (rescoped after S10-R2 strike)</t>
-        </is>
-      </c>
-      <c r="J177" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K177" s="2" t="inlineStr"/>
-      <c r="L177" s="2" t="inlineStr">
-        <is>
-          <t>C29433</t>
-        </is>
-      </c>
-      <c r="M177" s="2" t="inlineStr">
-        <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29433</t>
+      <c r="C177" s="4" t="inlineStr">
+        <is>
+          <t>Verify cost at completion behavior to avoid $0-cost margins in QuickBooks</t>
+        </is>
+      </c>
+      <c r="D177" s="4" t="inlineStr">
+        <is>
+          <t>Blocked-Env</t>
+        </is>
+      </c>
+      <c r="E177" s="4" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="F177" s="4" t="inlineStr">
+        <is>
+          <t>VIU PENDING (QA)</t>
+        </is>
+      </c>
+      <c r="G177" s="4" t="inlineStr">
+        <is>
+          <t>QA (needs cookies+seed data)</t>
+        </is>
+      </c>
+      <c r="H177" s="4" t="inlineStr">
+        <is>
+          <t>QA VIU: complete a WO end-to-end and inspect the QuickBooks / inventory side-effects (Journal Entry, Part History, inventory decrement).</t>
+        </is>
+      </c>
+      <c r="I177" s="4" t="inlineStr">
+        <is>
+          <t>§8 (cost at completion)</t>
+        </is>
+      </c>
+      <c r="J177" s="4" t="inlineStr">
+        <is>
+          <t>needs-data</t>
+        </is>
+      </c>
+      <c r="K177" s="4" t="inlineStr">
+        <is>
+          <t>QuickBooks inspection (cost-at-completion to avoid $0-cost margins) — likely needs dev/QB access.</t>
+        </is>
+      </c>
+      <c r="L177" s="4" t="inlineStr">
+        <is>
+          <t>C29431</t>
+        </is>
+      </c>
+      <c r="M177" s="4" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29431</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" s="4" t="inlineStr">
         <is>
-          <t>SF-QB-09</t>
+          <t>SF-QB-07</t>
         </is>
       </c>
       <c r="B178" s="4" t="inlineStr">
@@ -11766,7 +11746,7 @@
       </c>
       <c r="C178" s="4" t="inlineStr">
         <is>
-          <t>Verify part-sale order status transitions are not regressed by the shared order/status logic (requested to waiting-to-receive to received)</t>
+          <t>Verify the Journal Entry / Inventory sync to QuickBooks fires on invoice creation (not PO-dependent)</t>
         </is>
       </c>
       <c r="D178" s="4" t="inlineStr">
@@ -11796,44 +11776,44 @@
       </c>
       <c r="I178" s="4" t="inlineStr">
         <is>
-          <t>§8 Part Sales — confirmed (Jul 14) + S7/S8 part-sale AC</t>
-        </is>
-      </c>
-      <c r="J178" s="2" t="inlineStr">
-        <is>
-          <t>reachable-now</t>
+          <t>§5 (Journal Entry / Inventory → QBO)</t>
+        </is>
+      </c>
+      <c r="J178" s="4" t="inlineStr">
+        <is>
+          <t>needs-data</t>
         </is>
       </c>
       <c r="K178" s="4" t="inlineStr">
         <is>
-          <t>Δ15 residual check: part-sale status transitions not regressed — seed a Part Sale with a vendor part (now C29909).</t>
+          <t>QuickBooks inspection (Journal Entry / Inventory sync fires on invoice creation) — likely needs dev/QB access.</t>
         </is>
       </c>
       <c r="L178" s="4" t="inlineStr">
         <is>
-          <t>C29909</t>
+          <t>C29432</t>
         </is>
       </c>
       <c r="M178" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29909</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29432</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" s="2" t="inlineStr">
         <is>
-          <t>SF-AUTO-01</t>
+          <t>SF-QB-08</t>
         </is>
       </c>
       <c r="B179" s="2" t="inlineStr">
         <is>
-          <t>Auto-Complete Trigger (Story 16 R12/R13)</t>
+          <t>QuickBooks / Inventory Integrity</t>
         </is>
       </c>
       <c r="C179" s="2" t="inlineStr">
         <is>
-          <t>Verify resolving the last open line by completing a single line auto-completes the work order when Require Review is off</t>
+          <t>Verify Part History is preserved for a part that is genuinely inventory-tracked</t>
         </is>
       </c>
       <c r="D179" s="2" t="inlineStr">
@@ -11863,7 +11843,7 @@
       </c>
       <c r="I179" s="2" t="inlineStr">
         <is>
-          <t>S16-R12 (a) single line</t>
+          <t>§5 invariant 3 (rescoped after S10-R2 strike)</t>
         </is>
       </c>
       <c r="J179" s="2" t="inlineStr">
@@ -11874,82 +11854,86 @@
       <c r="K179" s="2" t="inlineStr"/>
       <c r="L179" s="2" t="inlineStr">
         <is>
-          <t>C29461</t>
+          <t>C29433</t>
         </is>
       </c>
       <c r="M179" s="2" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29461</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29433</t>
         </is>
       </c>
     </row>
     <row r="180">
-      <c r="A180" s="2" t="inlineStr">
-        <is>
-          <t>SF-AUTO-02</t>
-        </is>
-      </c>
-      <c r="B180" s="2" t="inlineStr">
-        <is>
-          <t>Auto-Complete Trigger (Story 16 R12/R13)</t>
-        </is>
-      </c>
-      <c r="C180" s="2" t="inlineStr">
-        <is>
-          <t>Verify resolving the last open lines in bulk (several at once) auto-completes the work order when Require Review is off</t>
-        </is>
-      </c>
-      <c r="D180" s="2" t="inlineStr">
-        <is>
-          <t>VIU-Verified</t>
-        </is>
-      </c>
-      <c r="E180" s="2" t="inlineStr">
-        <is>
-          <t>READY</t>
-        </is>
-      </c>
-      <c r="F180" s="2" t="inlineStr">
-        <is>
-          <t>READY (VIU-Verified)</t>
-        </is>
-      </c>
-      <c r="G180" s="2" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="H180" s="2" t="inlineStr">
-        <is>
-          <t>None — VIU-verified; uploadable now.</t>
-        </is>
-      </c>
-      <c r="I180" s="2" t="inlineStr">
-        <is>
-          <t>S16-R12 (b) bulk</t>
+      <c r="A180" s="4" t="inlineStr">
+        <is>
+          <t>SF-QB-09</t>
+        </is>
+      </c>
+      <c r="B180" s="4" t="inlineStr">
+        <is>
+          <t>QuickBooks / Inventory Integrity</t>
+        </is>
+      </c>
+      <c r="C180" s="4" t="inlineStr">
+        <is>
+          <t>Verify part-sale order status transitions are not regressed by the shared order/status logic (requested to waiting-to-receive to received)</t>
+        </is>
+      </c>
+      <c r="D180" s="4" t="inlineStr">
+        <is>
+          <t>Blocked-Env</t>
+        </is>
+      </c>
+      <c r="E180" s="4" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="F180" s="4" t="inlineStr">
+        <is>
+          <t>VIU PENDING (QA)</t>
+        </is>
+      </c>
+      <c r="G180" s="4" t="inlineStr">
+        <is>
+          <t>QA (needs cookies+seed data)</t>
+        </is>
+      </c>
+      <c r="H180" s="4" t="inlineStr">
+        <is>
+          <t>QA VIU: complete a WO end-to-end and inspect the QuickBooks / inventory side-effects (Journal Entry, Part History, inventory decrement).</t>
+        </is>
+      </c>
+      <c r="I180" s="4" t="inlineStr">
+        <is>
+          <t>§8 Part Sales — confirmed (Jul 14) + S7/S8 part-sale AC</t>
         </is>
       </c>
       <c r="J180" s="2" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="K180" s="2" t="inlineStr"/>
-      <c r="L180" s="2" t="inlineStr">
-        <is>
-          <t>C29462</t>
-        </is>
-      </c>
-      <c r="M180" s="2" t="inlineStr">
-        <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29462</t>
+          <t>reachable-now</t>
+        </is>
+      </c>
+      <c r="K180" s="4" t="inlineStr">
+        <is>
+          <t>Δ15 residual check: part-sale status transitions not regressed — seed a Part Sale with a vendor part (now C29909).</t>
+        </is>
+      </c>
+      <c r="L180" s="4" t="inlineStr">
+        <is>
+          <t>C29909</t>
+        </is>
+      </c>
+      <c r="M180" s="4" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29909</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" s="2" t="inlineStr">
         <is>
-          <t>SF-AUTO-03</t>
+          <t>SF-AUTO-01</t>
         </is>
       </c>
       <c r="B181" s="2" t="inlineStr">
@@ -11959,7 +11943,7 @@
       </c>
       <c r="C181" s="2" t="inlineStr">
         <is>
-          <t>Verify a split that leaves a work order fully resolved auto-completes that work order when Require Review is off</t>
+          <t>Verify resolving the last open line by completing a single line auto-completes the work order when Require Review is off</t>
         </is>
       </c>
       <c r="D181" s="2" t="inlineStr">
@@ -11989,7 +11973,7 @@
       </c>
       <c r="I181" s="2" t="inlineStr">
         <is>
-          <t>S16-R12 (c) split</t>
+          <t>S16-R12 (a) single line</t>
         </is>
       </c>
       <c r="J181" s="2" t="inlineStr">
@@ -12000,86 +11984,82 @@
       <c r="K181" s="2" t="inlineStr"/>
       <c r="L181" s="2" t="inlineStr">
         <is>
-          <t>C29463</t>
+          <t>C29461</t>
         </is>
       </c>
       <c r="M181" s="2" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29463</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29461</t>
         </is>
       </c>
     </row>
     <row r="182">
-      <c r="A182" s="4" t="inlineStr">
-        <is>
-          <t>SF-AUTO-04</t>
-        </is>
-      </c>
-      <c r="B182" s="4" t="inlineStr">
+      <c r="A182" s="2" t="inlineStr">
+        <is>
+          <t>SF-AUTO-02</t>
+        </is>
+      </c>
+      <c r="B182" s="2" t="inlineStr">
         <is>
           <t>Auto-Complete Trigger (Story 16 R12/R13)</t>
         </is>
       </c>
-      <c r="C182" s="4" t="inlineStr">
-        <is>
-          <t>Verify deleting a line so the remaining lines are all resolved auto-completes the work order when Require Review is off</t>
-        </is>
-      </c>
-      <c r="D182" s="4" t="inlineStr">
-        <is>
-          <t>Blocked-Env</t>
-        </is>
-      </c>
-      <c r="E182" s="4" t="inlineStr">
-        <is>
-          <t>BLOCKED</t>
-        </is>
-      </c>
-      <c r="F182" s="4" t="inlineStr">
-        <is>
-          <t>VIU PENDING (QA)</t>
-        </is>
-      </c>
-      <c r="G182" s="4" t="inlineStr">
-        <is>
-          <t>QA (needs cookies+seed data)</t>
-        </is>
-      </c>
-      <c r="H182" s="4" t="inlineStr">
-        <is>
-          <t>QA VIU: fresh sv7301 cookies + seeded data to drive this scenario.</t>
-        </is>
-      </c>
-      <c r="I182" s="4" t="inlineStr">
-        <is>
-          <t>S16-R12 (d) delete line</t>
+      <c r="C182" s="2" t="inlineStr">
+        <is>
+          <t>Verify resolving the last open lines in bulk (several at once) auto-completes the work order when Require Review is off</t>
+        </is>
+      </c>
+      <c r="D182" s="2" t="inlineStr">
+        <is>
+          <t>VIU-Verified</t>
+        </is>
+      </c>
+      <c r="E182" s="2" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="F182" s="2" t="inlineStr">
+        <is>
+          <t>READY (VIU-Verified)</t>
+        </is>
+      </c>
+      <c r="G182" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H182" s="2" t="inlineStr">
+        <is>
+          <t>None — VIU-verified; uploadable now.</t>
+        </is>
+      </c>
+      <c r="I182" s="2" t="inlineStr">
+        <is>
+          <t>S16-R12 (b) bulk</t>
         </is>
       </c>
       <c r="J182" s="2" t="inlineStr">
         <is>
-          <t>reachable-now</t>
-        </is>
-      </c>
-      <c r="K182" s="4" t="inlineStr">
-        <is>
-          <t>admin+tech + normal WO data; needs another VIU pass (no new inputs).</t>
-        </is>
-      </c>
-      <c r="L182" s="4" t="inlineStr">
-        <is>
-          <t>C29464</t>
-        </is>
-      </c>
-      <c r="M182" s="4" t="inlineStr">
-        <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29464</t>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K182" s="2" t="inlineStr"/>
+      <c r="L182" s="2" t="inlineStr">
+        <is>
+          <t>C29462</t>
+        </is>
+      </c>
+      <c r="M182" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29462</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" s="2" t="inlineStr">
         <is>
-          <t>SF-AUTO-05</t>
+          <t>SF-AUTO-03</t>
         </is>
       </c>
       <c r="B183" s="2" t="inlineStr">
@@ -12089,7 +12069,7 @@
       </c>
       <c r="C183" s="2" t="inlineStr">
         <is>
-          <t>Verify that with Require Review on, resolving the last open line routes the work order to Ready for Review instead of auto-completing</t>
+          <t>Verify a split that leaves a work order fully resolved auto-completes that work order when Require Review is off</t>
         </is>
       </c>
       <c r="D183" s="2" t="inlineStr">
@@ -12119,7 +12099,7 @@
       </c>
       <c r="I183" s="2" t="inlineStr">
         <is>
-          <t>S16-R12 review ON</t>
+          <t>S16-R12 (c) split</t>
         </is>
       </c>
       <c r="J183" s="2" t="inlineStr">
@@ -12130,19 +12110,19 @@
       <c r="K183" s="2" t="inlineStr"/>
       <c r="L183" s="2" t="inlineStr">
         <is>
-          <t>C29465</t>
+          <t>C29463</t>
         </is>
       </c>
       <c r="M183" s="2" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29465</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29463</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" s="4" t="inlineStr">
         <is>
-          <t>SF-AUTO-06</t>
+          <t>SF-AUTO-04</t>
         </is>
       </c>
       <c r="B184" s="4" t="inlineStr">
@@ -12152,7 +12132,7 @@
       </c>
       <c r="C184" s="4" t="inlineStr">
         <is>
-          <t>Verify a clock-out that finishes the last line routes the work order to Ready for Review even when Require Review is off</t>
+          <t>Verify deleting a line so the remaining lines are all resolved auto-completes the work order when Require Review is off</t>
         </is>
       </c>
       <c r="D184" s="4" t="inlineStr">
@@ -12182,7 +12162,7 @@
       </c>
       <c r="I184" s="4" t="inlineStr">
         <is>
-          <t>S16-R13 clock-out exception</t>
+          <t>S16-R12 (d) delete line</t>
         </is>
       </c>
       <c r="J184" s="2" t="inlineStr">
@@ -12197,29 +12177,29 @@
       </c>
       <c r="L184" s="4" t="inlineStr">
         <is>
-          <t>C29466</t>
+          <t>C29464</t>
         </is>
       </c>
       <c r="M184" s="4" t="inlineStr">
         <is>
-          <t>https://shopview.testrail.io/index.php?/cases/view/29466</t>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29464</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" s="2" t="inlineStr">
         <is>
-          <t>SF-AUTO-07</t>
+          <t>SF-AUTO-05</t>
         </is>
       </c>
       <c r="B185" s="2" t="inlineStr">
         <is>
-          <t>API — Auto-Complete Trigger (Story 16 R12/R13)</t>
+          <t>Auto-Complete Trigger (Story 16 R12/R13)</t>
         </is>
       </c>
       <c r="C185" s="2" t="inlineStr">
         <is>
-          <t>Verify the work order status transitions on the backend when the last open line is resolved (auto-Complete when review off, Ready for Review when review on)</t>
+          <t>Verify that with Require Review on, resolving the last open line routes the work order to Ready for Review instead of auto-completing</t>
         </is>
       </c>
       <c r="D185" s="2" t="inlineStr">
@@ -12249,7 +12229,7 @@
       </c>
       <c r="I185" s="2" t="inlineStr">
         <is>
-          <t>S16-R12 backend status transition</t>
+          <t>S16-R12 review ON</t>
         </is>
       </c>
       <c r="J185" s="2" t="inlineStr">
@@ -12260,10 +12240,140 @@
       <c r="K185" s="2" t="inlineStr"/>
       <c r="L185" s="2" t="inlineStr">
         <is>
+          <t>C29465</t>
+        </is>
+      </c>
+      <c r="M185" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29465</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="4" t="inlineStr">
+        <is>
+          <t>SF-AUTO-06</t>
+        </is>
+      </c>
+      <c r="B186" s="4" t="inlineStr">
+        <is>
+          <t>Auto-Complete Trigger (Story 16 R12/R13)</t>
+        </is>
+      </c>
+      <c r="C186" s="4" t="inlineStr">
+        <is>
+          <t>Verify a clock-out that finishes the last line routes the work order to Ready for Review even when Require Review is off</t>
+        </is>
+      </c>
+      <c r="D186" s="4" t="inlineStr">
+        <is>
+          <t>Blocked-Env</t>
+        </is>
+      </c>
+      <c r="E186" s="4" t="inlineStr">
+        <is>
+          <t>BLOCKED</t>
+        </is>
+      </c>
+      <c r="F186" s="4" t="inlineStr">
+        <is>
+          <t>VIU PENDING (QA)</t>
+        </is>
+      </c>
+      <c r="G186" s="4" t="inlineStr">
+        <is>
+          <t>QA (needs cookies+seed data)</t>
+        </is>
+      </c>
+      <c r="H186" s="4" t="inlineStr">
+        <is>
+          <t>QA VIU: fresh sv7301 cookies + seeded data to drive this scenario.</t>
+        </is>
+      </c>
+      <c r="I186" s="4" t="inlineStr">
+        <is>
+          <t>S16-R13 clock-out exception</t>
+        </is>
+      </c>
+      <c r="J186" s="2" t="inlineStr">
+        <is>
+          <t>reachable-now</t>
+        </is>
+      </c>
+      <c r="K186" s="4" t="inlineStr">
+        <is>
+          <t>admin+tech + normal WO data; needs another VIU pass (no new inputs).</t>
+        </is>
+      </c>
+      <c r="L186" s="4" t="inlineStr">
+        <is>
+          <t>C29466</t>
+        </is>
+      </c>
+      <c r="M186" s="4" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/29466</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="2" t="inlineStr">
+        <is>
+          <t>SF-AUTO-07</t>
+        </is>
+      </c>
+      <c r="B187" s="2" t="inlineStr">
+        <is>
+          <t>API — Auto-Complete Trigger (Story 16 R12/R13)</t>
+        </is>
+      </c>
+      <c r="C187" s="2" t="inlineStr">
+        <is>
+          <t>Verify the work order status transitions on the backend when the last open line is resolved (auto-Complete when review off, Ready for Review when review on)</t>
+        </is>
+      </c>
+      <c r="D187" s="2" t="inlineStr">
+        <is>
+          <t>VIU-Verified</t>
+        </is>
+      </c>
+      <c r="E187" s="2" t="inlineStr">
+        <is>
+          <t>READY</t>
+        </is>
+      </c>
+      <c r="F187" s="2" t="inlineStr">
+        <is>
+          <t>READY (VIU-Verified)</t>
+        </is>
+      </c>
+      <c r="G187" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H187" s="2" t="inlineStr">
+        <is>
+          <t>None — VIU-verified; uploadable now.</t>
+        </is>
+      </c>
+      <c r="I187" s="2" t="inlineStr">
+        <is>
+          <t>S16-R12 backend status transition</t>
+        </is>
+      </c>
+      <c r="J187" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K187" s="2" t="inlineStr"/>
+      <c r="L187" s="2" t="inlineStr">
+        <is>
           <t>C29467</t>
         </is>
       </c>
-      <c r="M185" s="2" t="inlineStr">
+      <c r="M187" s="2" t="inlineStr">
         <is>
           <t>https://shopview.testrail.io/index.php?/cases/view/29467</t>
         </is>
@@ -12309,7 +12419,7 @@
         </is>
       </c>
       <c r="B3" s="7" t="n">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="C3" s="7" t="n"/>
     </row>
@@ -12342,7 +12452,7 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
@@ -12402,7 +12512,7 @@
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
@@ -12417,7 +12527,7 @@
         </is>
       </c>
       <c r="B11" s="10" t="n">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="C11" s="7" t="inlineStr"/>
     </row>
@@ -12578,7 +12688,7 @@
       </c>
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t>finalizes the 2 BUG/RULING cases.</t>
+          <t>finalizes the 3 BUG/RULING cases.</t>
         </is>
       </c>
       <c r="C25" s="7" t="n"/>

</xml_diff>

<commit_message>
Simple Flow: strengthen Rule 24 (FE-block+BE-allow=PASS) + execute corrective TestRail push (SF-PERM-11/12 add + SF-PERM-03 update)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AZ5XzKsK9wv7M41cSPaMyg
</commit_message>
<xml_diff>
--- a/build/simple-flow/SimpleFlow_Blockers_Tracker.xlsx
+++ b/build/simple-flow/SimpleFlow_Blockers_Tracker.xlsx
@@ -10576,8 +10576,16 @@
         </is>
       </c>
       <c r="K159" s="5" t="inlineStr"/>
-      <c r="L159" s="5" t="inlineStr"/>
-      <c r="M159" s="5" t="inlineStr"/>
+      <c r="L159" s="5" t="inlineStr">
+        <is>
+          <t>C30646</t>
+        </is>
+      </c>
+      <c r="M159" s="5" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/30646</t>
+        </is>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -10631,8 +10639,16 @@
         </is>
       </c>
       <c r="K160" s="2" t="inlineStr"/>
-      <c r="L160" s="2" t="inlineStr"/>
-      <c r="M160" s="2" t="inlineStr"/>
+      <c r="L160" s="2" t="inlineStr">
+        <is>
+          <t>C30647</t>
+        </is>
+      </c>
+      <c r="M160" s="2" t="inlineStr">
+        <is>
+          <t>https://shopview.testrail.io/index.php?/cases/view/30647</t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">

</xml_diff>